<commit_message>
fixed bug and recalibrated greens
</commit_message>
<xml_diff>
--- a/frontend/data/uk_election_predictions.xlsx
+++ b/frontend/data/uk_election_predictions.xlsx
@@ -4360,7 +4360,7 @@
         <v>6</v>
       </c>
       <c r="C2">
-        <v>0.2743444238476875</v>
+        <v>0.2707688023253016</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -4377,7 +4377,7 @@
         <v>10</v>
       </c>
       <c r="C3">
-        <v>0.4306257315310673</v>
+        <v>0.4273550040153515</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -4394,7 +4394,7 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>0.373494124041068</v>
+        <v>0.3721229598856683</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -4411,7 +4411,7 @@
         <v>15</v>
       </c>
       <c r="C5">
-        <v>0.3628350310946563</v>
+        <v>0.3557925576187628</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -4428,7 +4428,7 @@
         <v>10</v>
       </c>
       <c r="C6">
-        <v>0.3981919005891298</v>
+        <v>0.3941300358670415</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -4445,7 +4445,7 @@
         <v>15</v>
       </c>
       <c r="C7">
-        <v>0.288756374381785</v>
+        <v>0.2830914975431358</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
@@ -4462,7 +4462,7 @@
         <v>15</v>
       </c>
       <c r="C8">
-        <v>0.3704416954380614</v>
+        <v>0.3653476068513238</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
@@ -4479,7 +4479,7 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>0.3489600248924803</v>
+        <v>0.3412451391907707</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
@@ -4496,7 +4496,7 @@
         <v>10</v>
       </c>
       <c r="C10">
-        <v>0.3488926235782247</v>
+        <v>0.3464507969288235</v>
       </c>
       <c r="D10" t="s">
         <v>7</v>
@@ -4513,7 +4513,7 @@
         <v>15</v>
       </c>
       <c r="C11">
-        <v>0.2592917531370745</v>
+        <v>0.2539011792253815</v>
       </c>
       <c r="D11" t="s">
         <v>7</v>
@@ -4530,7 +4530,7 @@
         <v>6</v>
       </c>
       <c r="C12">
-        <v>0.420396247153849</v>
+        <v>0.4147227394802035</v>
       </c>
       <c r="D12" t="s">
         <v>7</v>
@@ -4547,7 +4547,7 @@
         <v>15</v>
       </c>
       <c r="C13">
-        <v>0.331350451680347</v>
+        <v>0.3247670644942205</v>
       </c>
       <c r="D13" t="s">
         <v>7</v>
@@ -4564,7 +4564,7 @@
         <v>15</v>
       </c>
       <c r="C14">
-        <v>0.4376222424814795</v>
+        <v>0.4307827381421535</v>
       </c>
       <c r="D14" t="s">
         <v>7</v>
@@ -4581,7 +4581,7 @@
         <v>10</v>
       </c>
       <c r="C15">
-        <v>0.358822867810817</v>
+        <v>0.3553771857214677</v>
       </c>
       <c r="D15" t="s">
         <v>7</v>
@@ -4598,7 +4598,7 @@
         <v>6</v>
       </c>
       <c r="C16">
-        <v>0.2960141810973982</v>
+        <v>0.2933009965118885</v>
       </c>
       <c r="D16" t="s">
         <v>7</v>
@@ -4615,7 +4615,7 @@
         <v>15</v>
       </c>
       <c r="C17">
-        <v>0.2799300224866167</v>
+        <v>0.2753778203808029</v>
       </c>
       <c r="D17" t="s">
         <v>7</v>
@@ -4632,7 +4632,7 @@
         <v>10</v>
       </c>
       <c r="C18">
-        <v>0.2990320534284463</v>
+        <v>0.2947385930946325</v>
       </c>
       <c r="D18" t="s">
         <v>7</v>
@@ -4649,7 +4649,7 @@
         <v>44</v>
       </c>
       <c r="C19">
-        <v>0.4395706191880912</v>
+        <v>0.4360049105756226</v>
       </c>
       <c r="D19" t="s">
         <v>7</v>
@@ -4666,7 +4666,7 @@
         <v>6</v>
       </c>
       <c r="C20">
-        <v>0.4289788063058347</v>
+        <v>0.4189960882201127</v>
       </c>
       <c r="D20" t="s">
         <v>7</v>
@@ -4683,7 +4683,7 @@
         <v>10</v>
       </c>
       <c r="C21">
-        <v>0.4362543298434937</v>
+        <v>0.4361717024392023</v>
       </c>
       <c r="D21" t="s">
         <v>7</v>
@@ -4700,7 +4700,7 @@
         <v>6</v>
       </c>
       <c r="C22">
-        <v>0.3315892761078534</v>
+        <v>0.327776106359753</v>
       </c>
       <c r="D22" t="s">
         <v>7</v>
@@ -4717,7 +4717,7 @@
         <v>6</v>
       </c>
       <c r="C23">
-        <v>0.3992717543703808</v>
+        <v>0.3969006339241101</v>
       </c>
       <c r="D23" t="s">
         <v>7</v>
@@ -4734,7 +4734,7 @@
         <v>6</v>
       </c>
       <c r="C24">
-        <v>0.3617409043902401</v>
+        <v>0.3439240076363249</v>
       </c>
       <c r="D24" t="s">
         <v>7</v>
@@ -4751,7 +4751,7 @@
         <v>6</v>
       </c>
       <c r="C25">
-        <v>0.6451364534577115</v>
+        <v>0.6223155428152148</v>
       </c>
       <c r="D25" t="s">
         <v>7</v>
@@ -4768,7 +4768,7 @@
         <v>6</v>
       </c>
       <c r="C26">
-        <v>0.310625971837748</v>
+        <v>0.3073101306719332</v>
       </c>
       <c r="D26" t="s">
         <v>7</v>
@@ -4785,7 +4785,7 @@
         <v>10</v>
       </c>
       <c r="C27">
-        <v>0.2872011873757053</v>
+        <v>0.2844572302731646</v>
       </c>
       <c r="D27" t="s">
         <v>7</v>
@@ -4802,7 +4802,7 @@
         <v>10</v>
       </c>
       <c r="C28">
-        <v>0.3219530658013316</v>
+        <v>0.3176173211194649</v>
       </c>
       <c r="D28" t="s">
         <v>7</v>
@@ -4819,7 +4819,7 @@
         <v>44</v>
       </c>
       <c r="C29">
-        <v>0.4792689177560632</v>
+        <v>0.4788310853692099</v>
       </c>
       <c r="D29" t="s">
         <v>7</v>
@@ -4836,7 +4836,7 @@
         <v>6</v>
       </c>
       <c r="C30">
-        <v>0.3868608482301406</v>
+        <v>0.378042005269581</v>
       </c>
       <c r="D30" t="s">
         <v>7</v>
@@ -4853,7 +4853,7 @@
         <v>6</v>
       </c>
       <c r="C31">
-        <v>0.4261490112537247</v>
+        <v>0.4242921960687304</v>
       </c>
       <c r="D31" t="s">
         <v>7</v>
@@ -4870,7 +4870,7 @@
         <v>15</v>
       </c>
       <c r="C32">
-        <v>0.4285784189418017</v>
+        <v>0.4226553042105923</v>
       </c>
       <c r="D32" t="s">
         <v>7</v>
@@ -4887,7 +4887,7 @@
         <v>6</v>
       </c>
       <c r="C33">
-        <v>0.3964205475865312</v>
+        <v>0.3901552397622838</v>
       </c>
       <c r="D33" t="s">
         <v>7</v>
@@ -4904,7 +4904,7 @@
         <v>15</v>
       </c>
       <c r="C34">
-        <v>0.339615188084268</v>
+        <v>0.3312561804615002</v>
       </c>
       <c r="D34" t="s">
         <v>7</v>
@@ -4921,7 +4921,7 @@
         <v>6</v>
       </c>
       <c r="C35">
-        <v>0.4882366263833827</v>
+        <v>0.4669123446346876</v>
       </c>
       <c r="D35" t="s">
         <v>7</v>
@@ -4938,7 +4938,7 @@
         <v>79</v>
       </c>
       <c r="C36">
-        <v>0.2289664496481518</v>
+        <v>0.2625399423195997</v>
       </c>
       <c r="D36" t="s">
         <v>7</v>
@@ -4955,7 +4955,7 @@
         <v>15</v>
       </c>
       <c r="C37">
-        <v>0.3069074787993796</v>
+        <v>0.2991815861609693</v>
       </c>
       <c r="D37" t="s">
         <v>7</v>
@@ -4972,7 +4972,7 @@
         <v>6</v>
       </c>
       <c r="C38">
-        <v>0.3469283668127385</v>
+        <v>0.3375690440010488</v>
       </c>
       <c r="D38" t="s">
         <v>7</v>
@@ -4989,7 +4989,7 @@
         <v>15</v>
       </c>
       <c r="C39">
-        <v>0.374704157142648</v>
+        <v>0.3678491486038083</v>
       </c>
       <c r="D39" t="s">
         <v>7</v>
@@ -5006,7 +5006,7 @@
         <v>6</v>
       </c>
       <c r="C40">
-        <v>0.4620618260676042</v>
+        <v>0.4606636025130146</v>
       </c>
       <c r="D40" t="s">
         <v>7</v>
@@ -5023,7 +5023,7 @@
         <v>90</v>
       </c>
       <c r="C41">
-        <v>0.2721288066982321</v>
+        <v>0.2721692936521675</v>
       </c>
       <c r="D41" t="s">
         <v>7</v>
@@ -5040,7 +5040,7 @@
         <v>6</v>
       </c>
       <c r="C42">
-        <v>0.5476223114334171</v>
+        <v>0.5414220825177557</v>
       </c>
       <c r="D42" t="s">
         <v>7</v>
@@ -5057,7 +5057,7 @@
         <v>15</v>
       </c>
       <c r="C43">
-        <v>0.4110831855074111</v>
+        <v>0.4060875385124043</v>
       </c>
       <c r="D43" t="s">
         <v>7</v>
@@ -5074,7 +5074,7 @@
         <v>15</v>
       </c>
       <c r="C44">
-        <v>0.4167067244624789</v>
+        <v>0.411634669568714</v>
       </c>
       <c r="D44" t="s">
         <v>7</v>
@@ -5091,7 +5091,7 @@
         <v>6</v>
       </c>
       <c r="C45">
-        <v>0.401540474342546</v>
+        <v>0.39770654985971</v>
       </c>
       <c r="D45" t="s">
         <v>7</v>
@@ -5108,7 +5108,7 @@
         <v>6</v>
       </c>
       <c r="C46">
-        <v>0.4369714045974112</v>
+        <v>0.4339180874155192</v>
       </c>
       <c r="D46" t="s">
         <v>7</v>
@@ -5125,7 +5125,7 @@
         <v>15</v>
       </c>
       <c r="C47">
-        <v>0.2951391246925901</v>
+        <v>0.2915652766643496</v>
       </c>
       <c r="D47" t="s">
         <v>7</v>
@@ -5142,7 +5142,7 @@
         <v>15</v>
       </c>
       <c r="C48">
-        <v>0.428975461745873</v>
+        <v>0.4233680717804375</v>
       </c>
       <c r="D48" t="s">
         <v>7</v>
@@ -5159,7 +5159,7 @@
         <v>15</v>
       </c>
       <c r="C49">
-        <v>0.3484875365028581</v>
+        <v>0.3435176319205248</v>
       </c>
       <c r="D49" t="s">
         <v>7</v>
@@ -5176,7 +5176,7 @@
         <v>15</v>
       </c>
       <c r="C50">
-        <v>0.3896756533676329</v>
+        <v>0.3823714107828452</v>
       </c>
       <c r="D50" t="s">
         <v>7</v>
@@ -5193,7 +5193,7 @@
         <v>15</v>
       </c>
       <c r="C51">
-        <v>0.3684724416934421</v>
+        <v>0.3616264468180383</v>
       </c>
       <c r="D51" t="s">
         <v>7</v>
@@ -5210,7 +5210,7 @@
         <v>6</v>
       </c>
       <c r="C52">
-        <v>0.5326253927344151</v>
+        <v>0.5261927823127682</v>
       </c>
       <c r="D52" t="s">
         <v>7</v>
@@ -5227,7 +5227,7 @@
         <v>15</v>
       </c>
       <c r="C53">
-        <v>0.4448334497955047</v>
+        <v>0.441997107079971</v>
       </c>
       <c r="D53" t="s">
         <v>7</v>
@@ -5244,7 +5244,7 @@
         <v>6</v>
       </c>
       <c r="C54">
-        <v>0.3960441600488505</v>
+        <v>0.3934991594526069</v>
       </c>
       <c r="D54" t="s">
         <v>7</v>
@@ -5261,7 +5261,7 @@
         <v>10</v>
       </c>
       <c r="C55">
-        <v>0.2906101140192583</v>
+        <v>0.2849570389199365</v>
       </c>
       <c r="D55" t="s">
         <v>7</v>
@@ -5278,7 +5278,7 @@
         <v>10</v>
       </c>
       <c r="C56">
-        <v>0.359377709199482</v>
+        <v>0.3558654344054911</v>
       </c>
       <c r="D56" t="s">
         <v>7</v>
@@ -5295,7 +5295,7 @@
         <v>6</v>
       </c>
       <c r="C57">
-        <v>0.5866865374405409</v>
+        <v>0.5816727349403208</v>
       </c>
       <c r="D57" t="s">
         <v>7</v>
@@ -5312,7 +5312,7 @@
         <v>15</v>
       </c>
       <c r="C58">
-        <v>0.3387049529650369</v>
+        <v>0.3304942310832242</v>
       </c>
       <c r="D58" t="s">
         <v>7</v>
@@ -5329,7 +5329,7 @@
         <v>6</v>
       </c>
       <c r="C59">
-        <v>0.418040944778058</v>
+        <v>0.4023510367548296</v>
       </c>
       <c r="D59" t="s">
         <v>7</v>
@@ -5346,7 +5346,7 @@
         <v>6</v>
       </c>
       <c r="C60">
-        <v>0.2802636851558155</v>
+        <v>0.2761861902523435</v>
       </c>
       <c r="D60" t="s">
         <v>7</v>
@@ -5363,7 +5363,7 @@
         <v>6</v>
       </c>
       <c r="C61">
-        <v>0.3465987220348992</v>
+        <v>0.3428988857524589</v>
       </c>
       <c r="D61" t="s">
         <v>7</v>
@@ -5380,7 +5380,7 @@
         <v>10</v>
       </c>
       <c r="C62">
-        <v>0.3554827409459266</v>
+        <v>0.3455134135112166</v>
       </c>
       <c r="D62" t="s">
         <v>7</v>
@@ -5397,7 +5397,7 @@
         <v>6</v>
       </c>
       <c r="C63">
-        <v>0.377822842625364</v>
+        <v>0.3715722676211589</v>
       </c>
       <c r="D63" t="s">
         <v>7</v>
@@ -5414,7 +5414,7 @@
         <v>44</v>
       </c>
       <c r="C64">
-        <v>0.2411085964039868</v>
+        <v>0.2369168953961513</v>
       </c>
       <c r="D64" t="s">
         <v>7</v>
@@ -5431,7 +5431,7 @@
         <v>15</v>
       </c>
       <c r="C65">
-        <v>0.3380481255559311</v>
+        <v>0.3340518525879855</v>
       </c>
       <c r="D65" t="s">
         <v>7</v>
@@ -5445,10 +5445,10 @@
         <v>140</v>
       </c>
       <c r="B66" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C66">
-        <v>0.3326191692625839</v>
+        <v>0.3305173626011721</v>
       </c>
       <c r="D66" t="s">
         <v>7</v>
@@ -5465,7 +5465,7 @@
         <v>15</v>
       </c>
       <c r="C67">
-        <v>0.3670901745753551</v>
+        <v>0.3624983250487309</v>
       </c>
       <c r="D67" t="s">
         <v>7</v>
@@ -5482,7 +5482,7 @@
         <v>6</v>
       </c>
       <c r="C68">
-        <v>0.2662243770271415</v>
+        <v>0.2562574243338254</v>
       </c>
       <c r="D68" t="s">
         <v>7</v>
@@ -5499,7 +5499,7 @@
         <v>79</v>
       </c>
       <c r="C69">
-        <v>0.5752178585727976</v>
+        <v>0.6303965300737046</v>
       </c>
       <c r="D69" t="s">
         <v>7</v>
@@ -5516,7 +5516,7 @@
         <v>79</v>
       </c>
       <c r="C70">
-        <v>0.5139168238589952</v>
+        <v>0.5617303980475821</v>
       </c>
       <c r="D70" t="s">
         <v>7</v>
@@ -5533,7 +5533,7 @@
         <v>6</v>
       </c>
       <c r="C71">
-        <v>0.5105534951542032</v>
+        <v>0.480411174447221</v>
       </c>
       <c r="D71" t="s">
         <v>7</v>
@@ -5550,7 +5550,7 @@
         <v>6</v>
       </c>
       <c r="C72">
-        <v>0.3741996669766918</v>
+        <v>0.3616993955647609</v>
       </c>
       <c r="D72" t="s">
         <v>7</v>
@@ -5567,7 +5567,7 @@
         <v>6</v>
       </c>
       <c r="C73">
-        <v>0.545060761004782</v>
+        <v>0.5357651501135829</v>
       </c>
       <c r="D73" t="s">
         <v>7</v>
@@ -5584,7 +5584,7 @@
         <v>6</v>
       </c>
       <c r="C74">
-        <v>0.4999662791352072</v>
+        <v>0.4845437728885268</v>
       </c>
       <c r="D74" t="s">
         <v>7</v>
@@ -5601,7 +5601,7 @@
         <v>10</v>
       </c>
       <c r="C75">
-        <v>0.2566796673355865</v>
+        <v>0.2541955445262615</v>
       </c>
       <c r="D75" t="s">
         <v>7</v>
@@ -5618,7 +5618,7 @@
         <v>10</v>
       </c>
       <c r="C76">
-        <v>0.3861670199087062</v>
+        <v>0.3809370408374679</v>
       </c>
       <c r="D76" t="s">
         <v>7</v>
@@ -5635,7 +5635,7 @@
         <v>10</v>
       </c>
       <c r="C77">
-        <v>0.3507708557075714</v>
+        <v>0.3488099600822705</v>
       </c>
       <c r="D77" t="s">
         <v>7</v>
@@ -5652,7 +5652,7 @@
         <v>10</v>
       </c>
       <c r="C78">
-        <v>0.4321583143919466</v>
+        <v>0.4317646871450993</v>
       </c>
       <c r="D78" t="s">
         <v>7</v>
@@ -5669,7 +5669,7 @@
         <v>6</v>
       </c>
       <c r="C79">
-        <v>0.2536855763458504</v>
+        <v>0.2500509288923488</v>
       </c>
       <c r="D79" t="s">
         <v>7</v>
@@ -5686,7 +5686,7 @@
         <v>10</v>
       </c>
       <c r="C80">
-        <v>0.3780323775834545</v>
+        <v>0.3763295152472192</v>
       </c>
       <c r="D80" t="s">
         <v>7</v>
@@ -5703,7 +5703,7 @@
         <v>15</v>
       </c>
       <c r="C81">
-        <v>0.3250940696668205</v>
+        <v>0.318127218475848</v>
       </c>
       <c r="D81" t="s">
         <v>7</v>
@@ -5720,7 +5720,7 @@
         <v>10</v>
       </c>
       <c r="C82">
-        <v>0.4345841003048698</v>
+        <v>0.4312318788542558</v>
       </c>
       <c r="D82" t="s">
         <v>7</v>
@@ -5737,7 +5737,7 @@
         <v>6</v>
       </c>
       <c r="C83">
-        <v>0.3996691271634397</v>
+        <v>0.396635457080874</v>
       </c>
       <c r="D83" t="s">
         <v>7</v>
@@ -5754,7 +5754,7 @@
         <v>15</v>
       </c>
       <c r="C84">
-        <v>0.3039098653722838</v>
+        <v>0.2999412811216872</v>
       </c>
       <c r="D84" t="s">
         <v>7</v>
@@ -5771,7 +5771,7 @@
         <v>15</v>
       </c>
       <c r="C85">
-        <v>0.3511342050494848</v>
+        <v>0.3471447810830471</v>
       </c>
       <c r="D85" t="s">
         <v>7</v>
@@ -5788,7 +5788,7 @@
         <v>6</v>
       </c>
       <c r="C86">
-        <v>0.2942281260880815</v>
+        <v>0.2891873074079594</v>
       </c>
       <c r="D86" t="s">
         <v>7</v>
@@ -5805,7 +5805,7 @@
         <v>6</v>
       </c>
       <c r="C87">
-        <v>0.2654540862652238</v>
+        <v>0.262716332460824</v>
       </c>
       <c r="D87" t="s">
         <v>7</v>
@@ -5822,7 +5822,7 @@
         <v>79</v>
       </c>
       <c r="C88">
-        <v>0.3175290193067311</v>
+        <v>0.3586697590136387</v>
       </c>
       <c r="D88" t="s">
         <v>7</v>
@@ -5839,7 +5839,7 @@
         <v>10</v>
       </c>
       <c r="C89">
-        <v>0.3091833187353051</v>
+        <v>0.304093917974551</v>
       </c>
       <c r="D89" t="s">
         <v>7</v>
@@ -5856,7 +5856,7 @@
         <v>10</v>
       </c>
       <c r="C90">
-        <v>0.2941001741876766</v>
+        <v>0.2887036086633403</v>
       </c>
       <c r="D90" t="s">
         <v>7</v>
@@ -5873,7 +5873,7 @@
         <v>15</v>
       </c>
       <c r="C91">
-        <v>0.2707349989006477</v>
+        <v>0.2666599847064514</v>
       </c>
       <c r="D91" t="s">
         <v>7</v>
@@ -5890,7 +5890,7 @@
         <v>44</v>
       </c>
       <c r="C92">
-        <v>0.3390803863832717</v>
+        <v>0.339259539149075</v>
       </c>
       <c r="D92" t="s">
         <v>7</v>
@@ -5907,7 +5907,7 @@
         <v>15</v>
       </c>
       <c r="C93">
-        <v>0.4067607070222479</v>
+        <v>0.4025063195184892</v>
       </c>
       <c r="D93" t="s">
         <v>7</v>
@@ -5924,7 +5924,7 @@
         <v>6</v>
       </c>
       <c r="C94">
-        <v>0.2681426861307242</v>
+        <v>0.2634342665085479</v>
       </c>
       <c r="D94" t="s">
         <v>7</v>
@@ -5941,7 +5941,7 @@
         <v>15</v>
       </c>
       <c r="C95">
-        <v>0.3313015334207891</v>
+        <v>0.3249173539227785</v>
       </c>
       <c r="D95" t="s">
         <v>7</v>
@@ -5958,7 +5958,7 @@
         <v>15</v>
       </c>
       <c r="C96">
-        <v>0.3916184379003206</v>
+        <v>0.3847829847262648</v>
       </c>
       <c r="D96" t="s">
         <v>7</v>
@@ -5975,7 +5975,7 @@
         <v>44</v>
       </c>
       <c r="C97">
-        <v>0.3636423743697733</v>
+        <v>0.3621818003696727</v>
       </c>
       <c r="D97" t="s">
         <v>7</v>
@@ -5992,7 +5992,7 @@
         <v>44</v>
       </c>
       <c r="C98">
-        <v>0.3674296938775312</v>
+        <v>0.3663540130078058</v>
       </c>
       <c r="D98" t="s">
         <v>7</v>
@@ -6009,7 +6009,7 @@
         <v>6</v>
       </c>
       <c r="C99">
-        <v>0.4408367175454333</v>
+        <v>0.4344227560630397</v>
       </c>
       <c r="D99" t="s">
         <v>7</v>
@@ -6026,7 +6026,7 @@
         <v>44</v>
       </c>
       <c r="C100">
-        <v>0.4035193228528987</v>
+        <v>0.40043261148049</v>
       </c>
       <c r="D100" t="s">
         <v>7</v>
@@ -6043,7 +6043,7 @@
         <v>44</v>
       </c>
       <c r="C101">
-        <v>0.4567652865107409</v>
+        <v>0.4581797797144687</v>
       </c>
       <c r="D101" t="s">
         <v>7</v>
@@ -6060,7 +6060,7 @@
         <v>6</v>
       </c>
       <c r="C102">
-        <v>0.4613246281683068</v>
+        <v>0.455724614425064</v>
       </c>
       <c r="D102" t="s">
         <v>7</v>
@@ -6077,7 +6077,7 @@
         <v>6</v>
       </c>
       <c r="C103">
-        <v>0.350512790711995</v>
+        <v>0.3498833412686107</v>
       </c>
       <c r="D103" t="s">
         <v>7</v>
@@ -6094,7 +6094,7 @@
         <v>15</v>
       </c>
       <c r="C104">
-        <v>0.3704359969894747</v>
+        <v>0.3633097905611046</v>
       </c>
       <c r="D104" t="s">
         <v>7</v>
@@ -6111,7 +6111,7 @@
         <v>44</v>
       </c>
       <c r="C105">
-        <v>0.3496659789409031</v>
+        <v>0.3507620203388998</v>
       </c>
       <c r="D105" t="s">
         <v>7</v>
@@ -6128,7 +6128,7 @@
         <v>10</v>
       </c>
       <c r="C106">
-        <v>0.4111007953503558</v>
+        <v>0.4055375610684723</v>
       </c>
       <c r="D106" t="s">
         <v>7</v>
@@ -6145,7 +6145,7 @@
         <v>44</v>
       </c>
       <c r="C107">
-        <v>0.3509383947208228</v>
+        <v>0.3508890499335309</v>
       </c>
       <c r="D107" t="s">
         <v>7</v>
@@ -6162,7 +6162,7 @@
         <v>6</v>
       </c>
       <c r="C108">
-        <v>0.4065108007481238</v>
+        <v>0.4049777632437482</v>
       </c>
       <c r="D108" t="s">
         <v>7</v>
@@ -6179,7 +6179,7 @@
         <v>90</v>
       </c>
       <c r="C109">
-        <v>0.2649498884738904</v>
+        <v>0.264161745185849</v>
       </c>
       <c r="D109" t="s">
         <v>7</v>
@@ -6196,7 +6196,7 @@
         <v>15</v>
       </c>
       <c r="C110">
-        <v>0.2945735820979558</v>
+        <v>0.2915435292569892</v>
       </c>
       <c r="D110" t="s">
         <v>7</v>
@@ -6213,7 +6213,7 @@
         <v>6</v>
       </c>
       <c r="C111">
-        <v>0.5353796735510493</v>
+        <v>0.5329921238719034</v>
       </c>
       <c r="D111" t="s">
         <v>7</v>
@@ -6230,7 +6230,7 @@
         <v>6</v>
       </c>
       <c r="C112">
-        <v>0.3905223239457118</v>
+        <v>0.3848545588968632</v>
       </c>
       <c r="D112" t="s">
         <v>7</v>
@@ -6247,7 +6247,7 @@
         <v>15</v>
       </c>
       <c r="C113">
-        <v>0.5285800306227033</v>
+        <v>0.525927124703529</v>
       </c>
       <c r="D113" t="s">
         <v>7</v>
@@ -6264,7 +6264,7 @@
         <v>6</v>
       </c>
       <c r="C114">
-        <v>0.6859572483384525</v>
+        <v>0.668061393160153</v>
       </c>
       <c r="D114" t="s">
         <v>7</v>
@@ -6281,7 +6281,7 @@
         <v>6</v>
       </c>
       <c r="C115">
-        <v>0.3139025483315097</v>
+        <v>0.3090130497852639</v>
       </c>
       <c r="D115" t="s">
         <v>7</v>
@@ -6298,7 +6298,7 @@
         <v>6</v>
       </c>
       <c r="C116">
-        <v>0.4426836698890262</v>
+        <v>0.4423518019096727</v>
       </c>
       <c r="D116" t="s">
         <v>7</v>
@@ -6315,7 +6315,7 @@
         <v>10</v>
       </c>
       <c r="C117">
-        <v>0.2761325587972868</v>
+        <v>0.2733264992622443</v>
       </c>
       <c r="D117" t="s">
         <v>7</v>
@@ -6332,7 +6332,7 @@
         <v>10</v>
       </c>
       <c r="C118">
-        <v>0.4078913507053042</v>
+        <v>0.4049727985965608</v>
       </c>
       <c r="D118" t="s">
         <v>7</v>
@@ -6349,7 +6349,7 @@
         <v>6</v>
       </c>
       <c r="C119">
-        <v>0.3763142611007187</v>
+        <v>0.3753697405417786</v>
       </c>
       <c r="D119" t="s">
         <v>7</v>
@@ -6366,7 +6366,7 @@
         <v>10</v>
       </c>
       <c r="C120">
-        <v>0.3740157215264653</v>
+        <v>0.3715785922883789</v>
       </c>
       <c r="D120" t="s">
         <v>7</v>
@@ -6383,7 +6383,7 @@
         <v>6</v>
       </c>
       <c r="C121">
-        <v>0.3189678581175269</v>
+        <v>0.3113720368055873</v>
       </c>
       <c r="D121" t="s">
         <v>7</v>
@@ -6400,7 +6400,7 @@
         <v>15</v>
       </c>
       <c r="C122">
-        <v>0.3546441343707352</v>
+        <v>0.3472863770556365</v>
       </c>
       <c r="D122" t="s">
         <v>7</v>
@@ -6417,7 +6417,7 @@
         <v>15</v>
       </c>
       <c r="C123">
-        <v>0.3020082664986499</v>
+        <v>0.2977328383852423</v>
       </c>
       <c r="D123" t="s">
         <v>7</v>
@@ -6434,7 +6434,7 @@
         <v>15</v>
       </c>
       <c r="C124">
-        <v>0.3915947795650886</v>
+        <v>0.3863200256804191</v>
       </c>
       <c r="D124" t="s">
         <v>7</v>
@@ -6451,7 +6451,7 @@
         <v>10</v>
       </c>
       <c r="C125">
-        <v>0.2880372858423364</v>
+        <v>0.2845880307006517</v>
       </c>
       <c r="D125" t="s">
         <v>7</v>
@@ -6468,7 +6468,7 @@
         <v>6</v>
       </c>
       <c r="C126">
-        <v>0.3805236719469925</v>
+        <v>0.3780114004616743</v>
       </c>
       <c r="D126" t="s">
         <v>7</v>
@@ -6485,7 +6485,7 @@
         <v>6</v>
       </c>
       <c r="C127">
-        <v>0.5089749539855166</v>
+        <v>0.5035276801037192</v>
       </c>
       <c r="D127" t="s">
         <v>7</v>
@@ -6502,7 +6502,7 @@
         <v>15</v>
       </c>
       <c r="C128">
-        <v>0.4504933725224523</v>
+        <v>0.4409548223810976</v>
       </c>
       <c r="D128" t="s">
         <v>7</v>
@@ -6519,7 +6519,7 @@
         <v>10</v>
       </c>
       <c r="C129">
-        <v>0.3023225262410847</v>
+        <v>0.2981279624026634</v>
       </c>
       <c r="D129" t="s">
         <v>7</v>
@@ -6536,7 +6536,7 @@
         <v>15</v>
       </c>
       <c r="C130">
-        <v>0.4644546663652233</v>
+        <v>0.4607930045110125</v>
       </c>
       <c r="D130" t="s">
         <v>7</v>
@@ -6553,7 +6553,7 @@
         <v>10</v>
       </c>
       <c r="C131">
-        <v>0.2830431694334888</v>
+        <v>0.2795737786263787</v>
       </c>
       <c r="D131" t="s">
         <v>7</v>
@@ -6570,7 +6570,7 @@
         <v>6</v>
       </c>
       <c r="C132">
-        <v>0.3645834761611966</v>
+        <v>0.3606924208088326</v>
       </c>
       <c r="D132" t="s">
         <v>7</v>
@@ -6587,7 +6587,7 @@
         <v>15</v>
       </c>
       <c r="C133">
-        <v>0.3527482372664351</v>
+        <v>0.3469232179208231</v>
       </c>
       <c r="D133" t="s">
         <v>7</v>
@@ -6604,7 +6604,7 @@
         <v>6</v>
       </c>
       <c r="C134">
-        <v>0.3180921283532087</v>
+        <v>0.3178345101267935</v>
       </c>
       <c r="D134" t="s">
         <v>7</v>
@@ -6621,7 +6621,7 @@
         <v>6</v>
       </c>
       <c r="C135">
-        <v>0.3552984565744476</v>
+        <v>0.3498487195078078</v>
       </c>
       <c r="D135" t="s">
         <v>7</v>
@@ -6638,7 +6638,7 @@
         <v>44</v>
       </c>
       <c r="C136">
-        <v>0.3531851695055268</v>
+        <v>0.3499424984851879</v>
       </c>
       <c r="D136" t="s">
         <v>7</v>
@@ -6655,7 +6655,7 @@
         <v>6</v>
       </c>
       <c r="C137">
-        <v>0.3992815295665175</v>
+        <v>0.3933209787178658</v>
       </c>
       <c r="D137" t="s">
         <v>7</v>
@@ -6672,7 +6672,7 @@
         <v>15</v>
       </c>
       <c r="C138">
-        <v>0.3227998878422417</v>
+        <v>0.3179710458229442</v>
       </c>
       <c r="D138" t="s">
         <v>7</v>
@@ -6689,7 +6689,7 @@
         <v>6</v>
       </c>
       <c r="C139">
-        <v>0.4427156640453834</v>
+        <v>0.4402757647939984</v>
       </c>
       <c r="D139" t="s">
         <v>7</v>
@@ -6706,7 +6706,7 @@
         <v>44</v>
       </c>
       <c r="C140">
-        <v>0.4056683410752389</v>
+        <v>0.4070122175367404</v>
       </c>
       <c r="D140" t="s">
         <v>7</v>
@@ -6723,7 +6723,7 @@
         <v>6</v>
       </c>
       <c r="C141">
-        <v>0.3464714192787845</v>
+        <v>0.3439640069237996</v>
       </c>
       <c r="D141" t="s">
         <v>7</v>
@@ -6740,7 +6740,7 @@
         <v>10</v>
       </c>
       <c r="C142">
-        <v>0.4059302073110285</v>
+        <v>0.4055534461997542</v>
       </c>
       <c r="D142" t="s">
         <v>7</v>
@@ -6757,7 +6757,7 @@
         <v>15</v>
       </c>
       <c r="C143">
-        <v>0.3121103410919873</v>
+        <v>0.304135463461537</v>
       </c>
       <c r="D143" t="s">
         <v>7</v>
@@ -6774,7 +6774,7 @@
         <v>6</v>
       </c>
       <c r="C144">
-        <v>0.5876306152288507</v>
+        <v>0.564188157039164</v>
       </c>
       <c r="D144" t="s">
         <v>7</v>
@@ -6791,7 +6791,7 @@
         <v>6</v>
       </c>
       <c r="C145">
-        <v>0.2698367060463446</v>
+        <v>0.2655238711819132</v>
       </c>
       <c r="D145" t="s">
         <v>7</v>
@@ -6808,7 +6808,7 @@
         <v>6</v>
       </c>
       <c r="C146">
-        <v>0.4436468803715153</v>
+        <v>0.4406535218267651</v>
       </c>
       <c r="D146" t="s">
         <v>7</v>
@@ -6825,7 +6825,7 @@
         <v>6</v>
       </c>
       <c r="C147">
-        <v>0.4430331727848163</v>
+        <v>0.4394390304887004</v>
       </c>
       <c r="D147" t="s">
         <v>7</v>
@@ -6842,7 +6842,7 @@
         <v>6</v>
       </c>
       <c r="C148">
-        <v>0.3410568608326927</v>
+        <v>0.3331830173678353</v>
       </c>
       <c r="D148" t="s">
         <v>7</v>
@@ -6859,7 +6859,7 @@
         <v>10</v>
       </c>
       <c r="C149">
-        <v>0.3934490642266766</v>
+        <v>0.385596584360534</v>
       </c>
       <c r="D149" t="s">
         <v>7</v>
@@ -6876,7 +6876,7 @@
         <v>15</v>
       </c>
       <c r="C150">
-        <v>0.3507126082059528</v>
+        <v>0.3428805136849269</v>
       </c>
       <c r="D150" t="s">
         <v>7</v>
@@ -6893,7 +6893,7 @@
         <v>10</v>
       </c>
       <c r="C151">
-        <v>0.2554218915426055</v>
+        <v>0.2503822374398392</v>
       </c>
       <c r="D151" t="s">
         <v>7</v>
@@ -6910,7 +6910,7 @@
         <v>6</v>
       </c>
       <c r="C152">
-        <v>0.7114191000189132</v>
+        <v>0.6930778180921288</v>
       </c>
       <c r="D152" t="s">
         <v>7</v>
@@ -6927,7 +6927,7 @@
         <v>10</v>
       </c>
       <c r="C153">
-        <v>0.3501963425533418</v>
+        <v>0.3507530793377277</v>
       </c>
       <c r="D153" t="s">
         <v>7</v>
@@ -6944,7 +6944,7 @@
         <v>10</v>
       </c>
       <c r="C154">
-        <v>0.3407134977412515</v>
+        <v>0.3395075839022036</v>
       </c>
       <c r="D154" t="s">
         <v>7</v>
@@ -6961,7 +6961,7 @@
         <v>15</v>
       </c>
       <c r="C155">
-        <v>0.2854371134548503</v>
+        <v>0.2794920407605136</v>
       </c>
       <c r="D155" t="s">
         <v>7</v>
@@ -6978,7 +6978,7 @@
         <v>10</v>
       </c>
       <c r="C156">
-        <v>0.3539525694085282</v>
+        <v>0.352570586076865</v>
       </c>
       <c r="D156" t="s">
         <v>7</v>
@@ -6995,7 +6995,7 @@
         <v>6</v>
       </c>
       <c r="C157">
-        <v>0.3625942292439459</v>
+        <v>0.357644811223298</v>
       </c>
       <c r="D157" t="s">
         <v>7</v>
@@ -7012,7 +7012,7 @@
         <v>44</v>
       </c>
       <c r="C158">
-        <v>0.3798322416946763</v>
+        <v>0.3807980325274031</v>
       </c>
       <c r="D158" t="s">
         <v>7</v>
@@ -7029,7 +7029,7 @@
         <v>44</v>
       </c>
       <c r="C159">
-        <v>0.4019867013544833</v>
+        <v>0.4000028116210905</v>
       </c>
       <c r="D159" t="s">
         <v>7</v>
@@ -7046,7 +7046,7 @@
         <v>6</v>
       </c>
       <c r="C160">
-        <v>0.4053565284969917</v>
+        <v>0.4006571610081797</v>
       </c>
       <c r="D160" t="s">
         <v>7</v>
@@ -7063,7 +7063,7 @@
         <v>6</v>
       </c>
       <c r="C161">
-        <v>0.3719536093618472</v>
+        <v>0.3679085899314681</v>
       </c>
       <c r="D161" t="s">
         <v>7</v>
@@ -7080,7 +7080,7 @@
         <v>6</v>
       </c>
       <c r="C162">
-        <v>0.5725432951507149</v>
+        <v>0.5715720690848046</v>
       </c>
       <c r="D162" t="s">
         <v>7</v>
@@ -7097,7 +7097,7 @@
         <v>44</v>
       </c>
       <c r="C163">
-        <v>0.4744984356189673</v>
+        <v>0.470761276594728</v>
       </c>
       <c r="D163" t="s">
         <v>7</v>
@@ -7114,7 +7114,7 @@
         <v>10</v>
       </c>
       <c r="C164">
-        <v>0.3050193227252472</v>
+        <v>0.2983781177782549</v>
       </c>
       <c r="D164" t="s">
         <v>7</v>
@@ -7131,7 +7131,7 @@
         <v>10</v>
       </c>
       <c r="C165">
-        <v>0.3650739699344572</v>
+        <v>0.3593796570380079</v>
       </c>
       <c r="D165" t="s">
         <v>7</v>
@@ -7148,7 +7148,7 @@
         <v>44</v>
       </c>
       <c r="C166">
-        <v>0.3470995012544706</v>
+        <v>0.3464142876319796</v>
       </c>
       <c r="D166" t="s">
         <v>7</v>
@@ -7165,7 +7165,7 @@
         <v>6</v>
       </c>
       <c r="C167">
-        <v>0.3544724057355421</v>
+        <v>0.3516283424368871</v>
       </c>
       <c r="D167" t="s">
         <v>7</v>
@@ -7182,7 +7182,7 @@
         <v>6</v>
       </c>
       <c r="C168">
-        <v>0.614115150250741</v>
+        <v>0.6064224652096507</v>
       </c>
       <c r="D168" t="s">
         <v>7</v>
@@ -7199,7 +7199,7 @@
         <v>44</v>
       </c>
       <c r="C169">
-        <v>0.368090560040471</v>
+        <v>0.3674487581508515</v>
       </c>
       <c r="D169" t="s">
         <v>7</v>
@@ -7216,7 +7216,7 @@
         <v>6</v>
       </c>
       <c r="C170">
-        <v>0.3705491472245697</v>
+        <v>0.3617511012569462</v>
       </c>
       <c r="D170" t="s">
         <v>7</v>
@@ -7233,7 +7233,7 @@
         <v>44</v>
       </c>
       <c r="C171">
-        <v>0.2636412962725487</v>
+        <v>0.2601095847181945</v>
       </c>
       <c r="D171" t="s">
         <v>7</v>
@@ -7250,7 +7250,7 @@
         <v>10</v>
       </c>
       <c r="C172">
-        <v>0.4507377688796738</v>
+        <v>0.4515780879960856</v>
       </c>
       <c r="D172" t="s">
         <v>7</v>
@@ -7267,7 +7267,7 @@
         <v>10</v>
       </c>
       <c r="C173">
-        <v>0.3610347389161275</v>
+        <v>0.359205679040503</v>
       </c>
       <c r="D173" t="s">
         <v>7</v>
@@ -7284,7 +7284,7 @@
         <v>6</v>
       </c>
       <c r="C174">
-        <v>0.3081199017600114</v>
+        <v>0.3063556428707638</v>
       </c>
       <c r="D174" t="s">
         <v>7</v>
@@ -7301,7 +7301,7 @@
         <v>15</v>
       </c>
       <c r="C175">
-        <v>0.3361432062887905</v>
+        <v>0.3298362489438225</v>
       </c>
       <c r="D175" t="s">
         <v>7</v>
@@ -7318,7 +7318,7 @@
         <v>6</v>
       </c>
       <c r="C176">
-        <v>0.4076225954532831</v>
+        <v>0.4026629395948165</v>
       </c>
       <c r="D176" t="s">
         <v>7</v>
@@ -7335,7 +7335,7 @@
         <v>6</v>
       </c>
       <c r="C177">
-        <v>0.575313154034593</v>
+        <v>0.5729334375544368</v>
       </c>
       <c r="D177" t="s">
         <v>7</v>
@@ -7352,7 +7352,7 @@
         <v>15</v>
       </c>
       <c r="C178">
-        <v>0.4206166336705622</v>
+        <v>0.4151225514301349</v>
       </c>
       <c r="D178" t="s">
         <v>7</v>
@@ -7369,7 +7369,7 @@
         <v>15</v>
       </c>
       <c r="C179">
-        <v>0.3219155427982095</v>
+        <v>0.3175111760158237</v>
       </c>
       <c r="D179" t="s">
         <v>7</v>
@@ -7386,7 +7386,7 @@
         <v>44</v>
       </c>
       <c r="C180">
-        <v>0.3860290995248083</v>
+        <v>0.3842450177261314</v>
       </c>
       <c r="D180" t="s">
         <v>7</v>
@@ -7403,7 +7403,7 @@
         <v>6</v>
       </c>
       <c r="C181">
-        <v>0.3343575362767849</v>
+        <v>0.3328027511991101</v>
       </c>
       <c r="D181" t="s">
         <v>7</v>
@@ -7420,7 +7420,7 @@
         <v>10</v>
       </c>
       <c r="C182">
-        <v>0.3149893672484506</v>
+        <v>0.3128997364994713</v>
       </c>
       <c r="D182" t="s">
         <v>7</v>
@@ -7437,7 +7437,7 @@
         <v>6</v>
       </c>
       <c r="C183">
-        <v>0.3228210668523822</v>
+        <v>0.317009547615681</v>
       </c>
       <c r="D183" t="s">
         <v>7</v>
@@ -7454,7 +7454,7 @@
         <v>6</v>
       </c>
       <c r="C184">
-        <v>0.3375247279803752</v>
+        <v>0.3334635355415005</v>
       </c>
       <c r="D184" t="s">
         <v>7</v>
@@ -7471,7 +7471,7 @@
         <v>15</v>
       </c>
       <c r="C185">
-        <v>0.3493140845936578</v>
+        <v>0.3448198751628412</v>
       </c>
       <c r="D185" t="s">
         <v>7</v>
@@ -7488,7 +7488,7 @@
         <v>44</v>
       </c>
       <c r="C186">
-        <v>0.4322765039583277</v>
+        <v>0.429923516445045</v>
       </c>
       <c r="D186" t="s">
         <v>7</v>
@@ -7505,7 +7505,7 @@
         <v>15</v>
       </c>
       <c r="C187">
-        <v>0.2413737410871</v>
+        <v>0.2370057393918104</v>
       </c>
       <c r="D187" t="s">
         <v>7</v>
@@ -7522,7 +7522,7 @@
         <v>10</v>
       </c>
       <c r="C188">
-        <v>0.4859491608544575</v>
+        <v>0.4833369826390967</v>
       </c>
       <c r="D188" t="s">
         <v>7</v>
@@ -7539,7 +7539,7 @@
         <v>10</v>
       </c>
       <c r="C189">
-        <v>0.3438749075360664</v>
+        <v>0.3394078900131983</v>
       </c>
       <c r="D189" t="s">
         <v>7</v>
@@ -7553,10 +7553,10 @@
         <v>388</v>
       </c>
       <c r="B190" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C190">
-        <v>0.2785476024702784</v>
+        <v>0.2677358374063779</v>
       </c>
       <c r="D190" t="s">
         <v>7</v>
@@ -7573,7 +7573,7 @@
         <v>10</v>
       </c>
       <c r="C191">
-        <v>0.3624031903689905</v>
+        <v>0.3597245379122828</v>
       </c>
       <c r="D191" t="s">
         <v>7</v>
@@ -7590,7 +7590,7 @@
         <v>15</v>
       </c>
       <c r="C192">
-        <v>0.4356359928017999</v>
+        <v>0.4319641396559481</v>
       </c>
       <c r="D192" t="s">
         <v>7</v>
@@ -7607,7 +7607,7 @@
         <v>15</v>
       </c>
       <c r="C193">
-        <v>0.4739236572872539</v>
+        <v>0.4698853659521273</v>
       </c>
       <c r="D193" t="s">
         <v>7</v>
@@ -7624,7 +7624,7 @@
         <v>6</v>
       </c>
       <c r="C194">
-        <v>0.3557742961409078</v>
+        <v>0.3551230224930279</v>
       </c>
       <c r="D194" t="s">
         <v>7</v>
@@ -7641,7 +7641,7 @@
         <v>90</v>
       </c>
       <c r="C195">
-        <v>0.3635426152846116</v>
+        <v>0.3674265355705121</v>
       </c>
       <c r="D195" t="s">
         <v>7</v>
@@ -7655,10 +7655,10 @@
         <v>400</v>
       </c>
       <c r="B196" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="C196">
-        <v>0.3414954242128251</v>
+        <v>0.3427007098638066</v>
       </c>
       <c r="D196" t="s">
         <v>7</v>
@@ -7675,7 +7675,7 @@
         <v>10</v>
       </c>
       <c r="C197">
-        <v>0.3266679327406622</v>
+        <v>0.3242680080605463</v>
       </c>
       <c r="D197" t="s">
         <v>7</v>
@@ -7692,7 +7692,7 @@
         <v>6</v>
       </c>
       <c r="C198">
-        <v>0.5623044250432531</v>
+        <v>0.5412766256287408</v>
       </c>
       <c r="D198" t="s">
         <v>7</v>
@@ -7709,7 +7709,7 @@
         <v>6</v>
       </c>
       <c r="C199">
-        <v>0.6125430051275563</v>
+        <v>0.584160523273034</v>
       </c>
       <c r="D199" t="s">
         <v>7</v>
@@ -7726,7 +7726,7 @@
         <v>10</v>
       </c>
       <c r="C200">
-        <v>0.3387073719857271</v>
+        <v>0.3360508935521485</v>
       </c>
       <c r="D200" t="s">
         <v>7</v>
@@ -7743,7 +7743,7 @@
         <v>15</v>
       </c>
       <c r="C201">
-        <v>0.3457962986129706</v>
+        <v>0.3390423572818747</v>
       </c>
       <c r="D201" t="s">
         <v>7</v>
@@ -7760,7 +7760,7 @@
         <v>10</v>
       </c>
       <c r="C202">
-        <v>0.3743517246921917</v>
+        <v>0.3730451833340153</v>
       </c>
       <c r="D202" t="s">
         <v>7</v>
@@ -7777,7 +7777,7 @@
         <v>6</v>
       </c>
       <c r="C203">
-        <v>0.5429971199338652</v>
+        <v>0.530071513386964</v>
       </c>
       <c r="D203" t="s">
         <v>7</v>
@@ -7794,7 +7794,7 @@
         <v>6</v>
       </c>
       <c r="C204">
-        <v>0.5186862375199359</v>
+        <v>0.5109337459889992</v>
       </c>
       <c r="D204" t="s">
         <v>7</v>
@@ -7811,7 +7811,7 @@
         <v>10</v>
       </c>
       <c r="C205">
-        <v>0.4508976631949783</v>
+        <v>0.4498727134251197</v>
       </c>
       <c r="D205" t="s">
         <v>7</v>
@@ -7828,7 +7828,7 @@
         <v>15</v>
       </c>
       <c r="C206">
-        <v>0.3782220559035051</v>
+        <v>0.3725712597622816</v>
       </c>
       <c r="D206" t="s">
         <v>7</v>
@@ -7845,7 +7845,7 @@
         <v>44</v>
       </c>
       <c r="C207">
-        <v>0.5539401568102398</v>
+        <v>0.5522480487094877</v>
       </c>
       <c r="D207" t="s">
         <v>7</v>
@@ -7862,7 +7862,7 @@
         <v>44</v>
       </c>
       <c r="C208">
-        <v>0.4102780853458416</v>
+        <v>0.4086149538192547</v>
       </c>
       <c r="D208" t="s">
         <v>7</v>
@@ -7879,7 +7879,7 @@
         <v>10</v>
       </c>
       <c r="C209">
-        <v>0.5413927187876494</v>
+        <v>0.535358365259141</v>
       </c>
       <c r="D209" t="s">
         <v>7</v>
@@ -7896,7 +7896,7 @@
         <v>6</v>
       </c>
       <c r="C210">
-        <v>0.4534345217955247</v>
+        <v>0.4474591770575177</v>
       </c>
       <c r="D210" t="s">
         <v>7</v>
@@ -7913,7 +7913,7 @@
         <v>15</v>
       </c>
       <c r="C211">
-        <v>0.439416666741628</v>
+        <v>0.4342493238860198</v>
       </c>
       <c r="D211" t="s">
         <v>7</v>
@@ -7930,7 +7930,7 @@
         <v>10</v>
       </c>
       <c r="C212">
-        <v>0.2881211563689072</v>
+        <v>0.2851874218556277</v>
       </c>
       <c r="D212" t="s">
         <v>7</v>
@@ -7947,7 +7947,7 @@
         <v>15</v>
       </c>
       <c r="C213">
-        <v>0.3691045762980391</v>
+        <v>0.3639106047434822</v>
       </c>
       <c r="D213" t="s">
         <v>7</v>
@@ -7964,7 +7964,7 @@
         <v>15</v>
       </c>
       <c r="C214">
-        <v>0.3751914000070358</v>
+        <v>0.3704971027327663</v>
       </c>
       <c r="D214" t="s">
         <v>7</v>
@@ -7981,7 +7981,7 @@
         <v>10</v>
       </c>
       <c r="C215">
-        <v>0.6266573508386495</v>
+        <v>0.6239477689806501</v>
       </c>
       <c r="D215" t="s">
         <v>7</v>
@@ -7998,7 +7998,7 @@
         <v>15</v>
       </c>
       <c r="C216">
-        <v>0.3377949474695567</v>
+        <v>0.3340860985100582</v>
       </c>
       <c r="D216" t="s">
         <v>7</v>
@@ -8015,7 +8015,7 @@
         <v>15</v>
       </c>
       <c r="C217">
-        <v>0.3286159680771591</v>
+        <v>0.325039987078386</v>
       </c>
       <c r="D217" t="s">
         <v>7</v>
@@ -8032,7 +8032,7 @@
         <v>6</v>
       </c>
       <c r="C218">
-        <v>0.3741361653400642</v>
+        <v>0.3708071697491942</v>
       </c>
       <c r="D218" t="s">
         <v>7</v>
@@ -8049,7 +8049,7 @@
         <v>44</v>
       </c>
       <c r="C219">
-        <v>0.4855048758879948</v>
+        <v>0.4834469237090166</v>
       </c>
       <c r="D219" t="s">
         <v>7</v>
@@ -8066,7 +8066,7 @@
         <v>10</v>
       </c>
       <c r="C220">
-        <v>0.3039043475760219</v>
+        <v>0.3012901202413699</v>
       </c>
       <c r="D220" t="s">
         <v>7</v>
@@ -8083,7 +8083,7 @@
         <v>15</v>
       </c>
       <c r="C221">
-        <v>0.3668190301943769</v>
+        <v>0.3631648356356301</v>
       </c>
       <c r="D221" t="s">
         <v>7</v>
@@ -8100,7 +8100,7 @@
         <v>10</v>
       </c>
       <c r="C222">
-        <v>0.3039675129177595</v>
+        <v>0.2986984381783132</v>
       </c>
       <c r="D222" t="s">
         <v>7</v>
@@ -8117,7 +8117,7 @@
         <v>10</v>
       </c>
       <c r="C223">
-        <v>0.559145004915129</v>
+        <v>0.5585470800076302</v>
       </c>
       <c r="D223" t="s">
         <v>7</v>
@@ -8134,7 +8134,7 @@
         <v>10</v>
       </c>
       <c r="C224">
-        <v>0.3828430335216658</v>
+        <v>0.379625970341352</v>
       </c>
       <c r="D224" t="s">
         <v>7</v>
@@ -8151,7 +8151,7 @@
         <v>15</v>
       </c>
       <c r="C225">
-        <v>0.3733838150041052</v>
+        <v>0.367593854615648</v>
       </c>
       <c r="D225" t="s">
         <v>7</v>
@@ -8168,7 +8168,7 @@
         <v>6</v>
       </c>
       <c r="C226">
-        <v>0.4959513437609812</v>
+        <v>0.4889632742355976</v>
       </c>
       <c r="D226" t="s">
         <v>7</v>
@@ -8185,7 +8185,7 @@
         <v>10</v>
       </c>
       <c r="C227">
-        <v>0.3574968832743508</v>
+        <v>0.3541105401469736</v>
       </c>
       <c r="D227" t="s">
         <v>7</v>
@@ -8202,7 +8202,7 @@
         <v>6</v>
       </c>
       <c r="C228">
-        <v>0.4816183600183679</v>
+        <v>0.4801042691536525</v>
       </c>
       <c r="D228" t="s">
         <v>7</v>
@@ -8219,7 +8219,7 @@
         <v>6</v>
       </c>
       <c r="C229">
-        <v>0.5367738379176054</v>
+        <v>0.514823022013033</v>
       </c>
       <c r="D229" t="s">
         <v>7</v>
@@ -8236,7 +8236,7 @@
         <v>44</v>
       </c>
       <c r="C230">
-        <v>0.3785288301989626</v>
+        <v>0.3796636330794332</v>
       </c>
       <c r="D230" t="s">
         <v>7</v>
@@ -8253,7 +8253,7 @@
         <v>6</v>
       </c>
       <c r="C231">
-        <v>0.3069538930674262</v>
+        <v>0.3040984725755093</v>
       </c>
       <c r="D231" t="s">
         <v>7</v>
@@ -8270,7 +8270,7 @@
         <v>6</v>
       </c>
       <c r="C232">
-        <v>0.6497386231481003</v>
+        <v>0.6396213446286138</v>
       </c>
       <c r="D232" t="s">
         <v>7</v>
@@ -8287,7 +8287,7 @@
         <v>44</v>
       </c>
       <c r="C233">
-        <v>0.468236039387981</v>
+        <v>0.463881140870176</v>
       </c>
       <c r="D233" t="s">
         <v>7</v>
@@ -8304,7 +8304,7 @@
         <v>6</v>
       </c>
       <c r="C234">
-        <v>0.4104949323252272</v>
+        <v>0.407299630991789</v>
       </c>
       <c r="D234" t="s">
         <v>7</v>
@@ -8321,7 +8321,7 @@
         <v>6</v>
       </c>
       <c r="C235">
-        <v>0.5393772623810018</v>
+        <v>0.5265604752104807</v>
       </c>
       <c r="D235" t="s">
         <v>7</v>
@@ -8338,7 +8338,7 @@
         <v>6</v>
       </c>
       <c r="C236">
-        <v>0.2612702022392781</v>
+        <v>0.2544151984046321</v>
       </c>
       <c r="D236" t="s">
         <v>7</v>
@@ -8355,7 +8355,7 @@
         <v>10</v>
       </c>
       <c r="C237">
-        <v>0.3543692429051519</v>
+        <v>0.3515060660423022</v>
       </c>
       <c r="D237" t="s">
         <v>7</v>
@@ -8372,7 +8372,7 @@
         <v>6</v>
       </c>
       <c r="C238">
-        <v>0.3222078940091243</v>
+        <v>0.3187454843865296</v>
       </c>
       <c r="D238" t="s">
         <v>7</v>
@@ -8389,7 +8389,7 @@
         <v>6</v>
       </c>
       <c r="C239">
-        <v>0.4077159947115215</v>
+        <v>0.4053937802998382</v>
       </c>
       <c r="D239" t="s">
         <v>7</v>
@@ -8406,7 +8406,7 @@
         <v>90</v>
       </c>
       <c r="C240">
-        <v>0.3721774718566679</v>
+        <v>0.3659828005382771</v>
       </c>
       <c r="D240" t="s">
         <v>7</v>
@@ -8420,10 +8420,10 @@
         <v>490</v>
       </c>
       <c r="B241" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="C241">
-        <v>0.2433747260458472</v>
+        <v>0.2365797828062899</v>
       </c>
       <c r="D241" t="s">
         <v>7</v>
@@ -8437,10 +8437,10 @@
         <v>492</v>
       </c>
       <c r="B242" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C242">
-        <v>0.3066572761382347</v>
+        <v>0.3029198380470375</v>
       </c>
       <c r="D242" t="s">
         <v>7</v>
@@ -8457,7 +8457,7 @@
         <v>15</v>
       </c>
       <c r="C243">
-        <v>0.467528112104981</v>
+        <v>0.4615145136969455</v>
       </c>
       <c r="D243" t="s">
         <v>7</v>
@@ -8474,7 +8474,7 @@
         <v>90</v>
       </c>
       <c r="C244">
-        <v>0.3659217696377142</v>
+        <v>0.3609764216052976</v>
       </c>
       <c r="D244" t="s">
         <v>7</v>
@@ -8491,7 +8491,7 @@
         <v>6</v>
       </c>
       <c r="C245">
-        <v>0.6713804484255201</v>
+        <v>0.6556996063224717</v>
       </c>
       <c r="D245" t="s">
         <v>7</v>
@@ -8508,7 +8508,7 @@
         <v>6</v>
       </c>
       <c r="C246">
-        <v>0.4619845478485745</v>
+        <v>0.4524579893186171</v>
       </c>
       <c r="D246" t="s">
         <v>7</v>
@@ -8525,7 +8525,7 @@
         <v>6</v>
       </c>
       <c r="C247">
-        <v>0.4460376994763179</v>
+        <v>0.4421069067664105</v>
       </c>
       <c r="D247" t="s">
         <v>7</v>
@@ -8542,7 +8542,7 @@
         <v>10</v>
       </c>
       <c r="C248">
-        <v>0.376431345408876</v>
+        <v>0.3730227980393712</v>
       </c>
       <c r="D248" t="s">
         <v>7</v>
@@ -8559,7 +8559,7 @@
         <v>6</v>
       </c>
       <c r="C249">
-        <v>0.4769308951287688</v>
+        <v>0.4673892891495007</v>
       </c>
       <c r="D249" t="s">
         <v>7</v>
@@ -8576,7 +8576,7 @@
         <v>15</v>
       </c>
       <c r="C250">
-        <v>0.3797564451442427</v>
+        <v>0.3747267412857377</v>
       </c>
       <c r="D250" t="s">
         <v>7</v>
@@ -8593,7 +8593,7 @@
         <v>44</v>
       </c>
       <c r="C251">
-        <v>0.4917488824495321</v>
+        <v>0.4893986464751204</v>
       </c>
       <c r="D251" t="s">
         <v>7</v>
@@ -8610,7 +8610,7 @@
         <v>6</v>
       </c>
       <c r="C252">
-        <v>0.4621345194059519</v>
+        <v>0.4610894773248488</v>
       </c>
       <c r="D252" t="s">
         <v>7</v>
@@ -8627,7 +8627,7 @@
         <v>6</v>
       </c>
       <c r="C253">
-        <v>0.3672623700275011</v>
+        <v>0.3624809435957666</v>
       </c>
       <c r="D253" t="s">
         <v>7</v>
@@ -8644,7 +8644,7 @@
         <v>6</v>
       </c>
       <c r="C254">
-        <v>0.4745440679804606</v>
+        <v>0.4740045897596761</v>
       </c>
       <c r="D254" t="s">
         <v>7</v>
@@ -8661,7 +8661,7 @@
         <v>15</v>
       </c>
       <c r="C255">
-        <v>0.4467230938139757</v>
+        <v>0.4400104588754182</v>
       </c>
       <c r="D255" t="s">
         <v>7</v>
@@ -8678,7 +8678,7 @@
         <v>6</v>
       </c>
       <c r="C256">
-        <v>0.5808962699141962</v>
+        <v>0.5727272073393423</v>
       </c>
       <c r="D256" t="s">
         <v>7</v>
@@ -8695,7 +8695,7 @@
         <v>6</v>
       </c>
       <c r="C257">
-        <v>0.3972305702805617</v>
+        <v>0.3911678407612567</v>
       </c>
       <c r="D257" t="s">
         <v>7</v>
@@ -8712,7 +8712,7 @@
         <v>6</v>
       </c>
       <c r="C258">
-        <v>0.5401195914597928</v>
+        <v>0.5158455728760613</v>
       </c>
       <c r="D258" t="s">
         <v>7</v>
@@ -8729,7 +8729,7 @@
         <v>6</v>
       </c>
       <c r="C259">
-        <v>0.3187354885186393</v>
+        <v>0.3121121637966094</v>
       </c>
       <c r="D259" t="s">
         <v>7</v>
@@ -8746,7 +8746,7 @@
         <v>6</v>
       </c>
       <c r="C260">
-        <v>0.4082505245598554</v>
+        <v>0.4016680948012837</v>
       </c>
       <c r="D260" t="s">
         <v>7</v>
@@ -8763,7 +8763,7 @@
         <v>6</v>
       </c>
       <c r="C261">
-        <v>0.4343187889360684</v>
+        <v>0.4304294965720206</v>
       </c>
       <c r="D261" t="s">
         <v>7</v>
@@ -8780,7 +8780,7 @@
         <v>6</v>
       </c>
       <c r="C262">
-        <v>0.4248047082751661</v>
+        <v>0.4098832143033049</v>
       </c>
       <c r="D262" t="s">
         <v>7</v>
@@ -8797,7 +8797,7 @@
         <v>6</v>
       </c>
       <c r="C263">
-        <v>0.4914265973220349</v>
+        <v>0.4868200829764714</v>
       </c>
       <c r="D263" t="s">
         <v>7</v>
@@ -8814,7 +8814,7 @@
         <v>6</v>
       </c>
       <c r="C264">
-        <v>0.4195553335894438</v>
+        <v>0.4115130751747961</v>
       </c>
       <c r="D264" t="s">
         <v>7</v>
@@ -8831,7 +8831,7 @@
         <v>6</v>
       </c>
       <c r="C265">
-        <v>0.3201101819094134</v>
+        <v>0.3098950655347125</v>
       </c>
       <c r="D265" t="s">
         <v>7</v>
@@ -8848,7 +8848,7 @@
         <v>90</v>
       </c>
       <c r="C266">
-        <v>0.3360797308459521</v>
+        <v>0.3335881192565437</v>
       </c>
       <c r="D266" t="s">
         <v>7</v>
@@ -8865,7 +8865,7 @@
         <v>6</v>
       </c>
       <c r="C267">
-        <v>0.2876181657059387</v>
+        <v>0.2832379905339202</v>
       </c>
       <c r="D267" t="s">
         <v>7</v>
@@ -8882,7 +8882,7 @@
         <v>6</v>
       </c>
       <c r="C268">
-        <v>0.4586770186223819</v>
+        <v>0.4563057573110308</v>
       </c>
       <c r="D268" t="s">
         <v>7</v>
@@ -8899,7 +8899,7 @@
         <v>44</v>
       </c>
       <c r="C269">
-        <v>0.3777765555733613</v>
+        <v>0.3755121927242653</v>
       </c>
       <c r="D269" t="s">
         <v>7</v>
@@ -8916,7 +8916,7 @@
         <v>6</v>
       </c>
       <c r="C270">
-        <v>0.5510074061370909</v>
+        <v>0.5357467880290233</v>
       </c>
       <c r="D270" t="s">
         <v>7</v>
@@ -8933,7 +8933,7 @@
         <v>6</v>
       </c>
       <c r="C271">
-        <v>0.5752194339335136</v>
+        <v>0.5472665090953376</v>
       </c>
       <c r="D271" t="s">
         <v>7</v>
@@ -8950,7 +8950,7 @@
         <v>6</v>
       </c>
       <c r="C272">
-        <v>0.3393085749834798</v>
+        <v>0.329767416137605</v>
       </c>
       <c r="D272" t="s">
         <v>7</v>
@@ -8967,7 +8967,7 @@
         <v>6</v>
       </c>
       <c r="C273">
-        <v>0.5484497548144663</v>
+        <v>0.5391828427496783</v>
       </c>
       <c r="D273" t="s">
         <v>7</v>
@@ -8984,7 +8984,7 @@
         <v>15</v>
       </c>
       <c r="C274">
-        <v>0.3566305204150331</v>
+        <v>0.3534318317217603</v>
       </c>
       <c r="D274" t="s">
         <v>7</v>
@@ -9001,7 +9001,7 @@
         <v>15</v>
       </c>
       <c r="C275">
-        <v>0.2602235164734286</v>
+        <v>0.2552834466407648</v>
       </c>
       <c r="D275" t="s">
         <v>7</v>
@@ -9018,7 +9018,7 @@
         <v>6</v>
       </c>
       <c r="C276">
-        <v>0.3356125217906785</v>
+        <v>0.3334980963961576</v>
       </c>
       <c r="D276" t="s">
         <v>7</v>
@@ -9032,10 +9032,10 @@
         <v>562</v>
       </c>
       <c r="B277" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="C277">
-        <v>0.3833036982855891</v>
+        <v>0.4086115522892595</v>
       </c>
       <c r="D277" t="s">
         <v>7</v>
@@ -9052,7 +9052,7 @@
         <v>6</v>
       </c>
       <c r="C278">
-        <v>0.4511810914535584</v>
+        <v>0.4463123214762043</v>
       </c>
       <c r="D278" t="s">
         <v>7</v>
@@ -9069,7 +9069,7 @@
         <v>6</v>
       </c>
       <c r="C279">
-        <v>0.5819364180795003</v>
+        <v>0.5657360423902152</v>
       </c>
       <c r="D279" t="s">
         <v>7</v>
@@ -9086,7 +9086,7 @@
         <v>6</v>
       </c>
       <c r="C280">
-        <v>0.4698542271897259</v>
+        <v>0.4637155656716211</v>
       </c>
       <c r="D280" t="s">
         <v>7</v>
@@ -9103,7 +9103,7 @@
         <v>6</v>
       </c>
       <c r="C281">
-        <v>0.3703746920095099</v>
+        <v>0.3670883107884595</v>
       </c>
       <c r="D281" t="s">
         <v>7</v>
@@ -9120,7 +9120,7 @@
         <v>15</v>
       </c>
       <c r="C282">
-        <v>0.3789099141469114</v>
+        <v>0.3750075222928968</v>
       </c>
       <c r="D282" t="s">
         <v>7</v>
@@ -9137,7 +9137,7 @@
         <v>6</v>
       </c>
       <c r="C283">
-        <v>0.39274494688999</v>
+        <v>0.3901365448432866</v>
       </c>
       <c r="D283" t="s">
         <v>7</v>
@@ -9154,7 +9154,7 @@
         <v>6</v>
       </c>
       <c r="C284">
-        <v>0.3263026243309614</v>
+        <v>0.3199304532095547</v>
       </c>
       <c r="D284" t="s">
         <v>7</v>
@@ -9171,7 +9171,7 @@
         <v>15</v>
       </c>
       <c r="C285">
-        <v>0.2933204873692673</v>
+        <v>0.2873051152788437</v>
       </c>
       <c r="D285" t="s">
         <v>7</v>
@@ -9188,7 +9188,7 @@
         <v>6</v>
       </c>
       <c r="C286">
-        <v>0.3133903807423313</v>
+        <v>0.3094181449471252</v>
       </c>
       <c r="D286" t="s">
         <v>7</v>
@@ -9205,7 +9205,7 @@
         <v>44</v>
       </c>
       <c r="C287">
-        <v>0.5020866422744739</v>
+        <v>0.5016708193685903</v>
       </c>
       <c r="D287" t="s">
         <v>7</v>
@@ -9222,7 +9222,7 @@
         <v>15</v>
       </c>
       <c r="C288">
-        <v>0.2518567574199793</v>
+        <v>0.2465732638561469</v>
       </c>
       <c r="D288" t="s">
         <v>7</v>
@@ -9239,7 +9239,7 @@
         <v>6</v>
       </c>
       <c r="C289">
-        <v>0.3692506217142567</v>
+        <v>0.3675150456401096</v>
       </c>
       <c r="D289" t="s">
         <v>7</v>
@@ -9256,7 +9256,7 @@
         <v>15</v>
       </c>
       <c r="C290">
-        <v>0.3857685525049637</v>
+        <v>0.3826014220099081</v>
       </c>
       <c r="D290" t="s">
         <v>7</v>
@@ -9273,7 +9273,7 @@
         <v>6</v>
       </c>
       <c r="C291">
-        <v>0.479888109000133</v>
+        <v>0.4602268929723713</v>
       </c>
       <c r="D291" t="s">
         <v>7</v>
@@ -9290,7 +9290,7 @@
         <v>79</v>
       </c>
       <c r="C292">
-        <v>0.4370979051100437</v>
+        <v>0.486746206063516</v>
       </c>
       <c r="D292" t="s">
         <v>7</v>
@@ -9307,7 +9307,7 @@
         <v>6</v>
       </c>
       <c r="C293">
-        <v>0.6394420513558626</v>
+        <v>0.6198957533641464</v>
       </c>
       <c r="D293" t="s">
         <v>7</v>
@@ -9324,7 +9324,7 @@
         <v>15</v>
       </c>
       <c r="C294">
-        <v>0.4152711526580308</v>
+        <v>0.409690806421421</v>
       </c>
       <c r="D294" t="s">
         <v>7</v>
@@ -9341,7 +9341,7 @@
         <v>10</v>
       </c>
       <c r="C295">
-        <v>0.3767584980418999</v>
+        <v>0.3737032247404276</v>
       </c>
       <c r="D295" t="s">
         <v>7</v>
@@ -9358,7 +9358,7 @@
         <v>15</v>
       </c>
       <c r="C296">
-        <v>0.2807865678957987</v>
+        <v>0.2771847055905297</v>
       </c>
       <c r="D296" t="s">
         <v>7</v>
@@ -9375,7 +9375,7 @@
         <v>10</v>
       </c>
       <c r="C297">
-        <v>0.5165195832041586</v>
+        <v>0.5173973655729445</v>
       </c>
       <c r="D297" t="s">
         <v>7</v>
@@ -9392,7 +9392,7 @@
         <v>10</v>
       </c>
       <c r="C298">
-        <v>0.3996531629557994</v>
+        <v>0.3948333682134985</v>
       </c>
       <c r="D298" t="s">
         <v>7</v>
@@ -9409,7 +9409,7 @@
         <v>44</v>
       </c>
       <c r="C299">
-        <v>0.3217930581193317</v>
+        <v>0.3145355796124201</v>
       </c>
       <c r="D299" t="s">
         <v>7</v>
@@ -9426,7 +9426,7 @@
         <v>10</v>
       </c>
       <c r="C300">
-        <v>0.3588216202846792</v>
+        <v>0.3549704427854145</v>
       </c>
       <c r="D300" t="s">
         <v>7</v>
@@ -9443,7 +9443,7 @@
         <v>6</v>
       </c>
       <c r="C301">
-        <v>0.3651607757176786</v>
+        <v>0.3620484599316319</v>
       </c>
       <c r="D301" t="s">
         <v>7</v>
@@ -9460,7 +9460,7 @@
         <v>44</v>
       </c>
       <c r="C302">
-        <v>0.5140415001731807</v>
+        <v>0.5138289255297454</v>
       </c>
       <c r="D302" t="s">
         <v>7</v>
@@ -9477,7 +9477,7 @@
         <v>10</v>
       </c>
       <c r="C303">
-        <v>0.341016039496665</v>
+        <v>0.3390941480594509</v>
       </c>
       <c r="D303" t="s">
         <v>7</v>
@@ -9494,7 +9494,7 @@
         <v>10</v>
       </c>
       <c r="C304">
-        <v>0.2862679774029669</v>
+        <v>0.2805110979544425</v>
       </c>
       <c r="D304" t="s">
         <v>7</v>
@@ -9511,7 +9511,7 @@
         <v>44</v>
       </c>
       <c r="C305">
-        <v>0.4642279452496298</v>
+        <v>0.4635582706491105</v>
       </c>
       <c r="D305" t="s">
         <v>7</v>
@@ -9528,7 +9528,7 @@
         <v>15</v>
       </c>
       <c r="C306">
-        <v>0.4202644499284598</v>
+        <v>0.4145996241731137</v>
       </c>
       <c r="D306" t="s">
         <v>7</v>
@@ -9545,7 +9545,7 @@
         <v>6</v>
       </c>
       <c r="C307">
-        <v>0.4527634361577014</v>
+        <v>0.4516763150970041</v>
       </c>
       <c r="D307" t="s">
         <v>7</v>
@@ -9562,7 +9562,7 @@
         <v>6</v>
       </c>
       <c r="C308">
-        <v>0.363707626036357</v>
+        <v>0.3597115626734285</v>
       </c>
       <c r="D308" t="s">
         <v>7</v>
@@ -9579,7 +9579,7 @@
         <v>10</v>
       </c>
       <c r="C309">
-        <v>0.2699507709782042</v>
+        <v>0.2673465951161779</v>
       </c>
       <c r="D309" t="s">
         <v>7</v>
@@ -9596,7 +9596,7 @@
         <v>6</v>
       </c>
       <c r="C310">
-        <v>0.4188825687795267</v>
+        <v>0.408232967534265</v>
       </c>
       <c r="D310" t="s">
         <v>7</v>
@@ -9613,7 +9613,7 @@
         <v>15</v>
       </c>
       <c r="C311">
-        <v>0.3531006745579697</v>
+        <v>0.3487404067218108</v>
       </c>
       <c r="D311" t="s">
         <v>7</v>
@@ -9630,7 +9630,7 @@
         <v>10</v>
       </c>
       <c r="C312">
-        <v>0.3073322112340575</v>
+        <v>0.3052686911174595</v>
       </c>
       <c r="D312" t="s">
         <v>7</v>
@@ -9647,7 +9647,7 @@
         <v>10</v>
       </c>
       <c r="C313">
-        <v>0.2847734851528541</v>
+        <v>0.2837778384697631</v>
       </c>
       <c r="D313" t="s">
         <v>7</v>
@@ -9664,7 +9664,7 @@
         <v>10</v>
       </c>
       <c r="C314">
-        <v>0.3379436281896377</v>
+        <v>0.3324916428543011</v>
       </c>
       <c r="D314" t="s">
         <v>7</v>
@@ -9681,7 +9681,7 @@
         <v>44</v>
       </c>
       <c r="C315">
-        <v>0.5112185816367065</v>
+        <v>0.5077009515781277</v>
       </c>
       <c r="D315" t="s">
         <v>7</v>
@@ -9698,7 +9698,7 @@
         <v>6</v>
       </c>
       <c r="C316">
-        <v>0.4071636140258336</v>
+        <v>0.399814116398546</v>
       </c>
       <c r="D316" t="s">
         <v>7</v>
@@ -9715,7 +9715,7 @@
         <v>6</v>
       </c>
       <c r="C317">
-        <v>0.5199076383421941</v>
+        <v>0.5107413486164124</v>
       </c>
       <c r="D317" t="s">
         <v>7</v>
@@ -9732,7 +9732,7 @@
         <v>6</v>
       </c>
       <c r="C318">
-        <v>0.5742442027706895</v>
+        <v>0.5665695687972865</v>
       </c>
       <c r="D318" t="s">
         <v>7</v>
@@ -9749,7 +9749,7 @@
         <v>6</v>
       </c>
       <c r="C319">
-        <v>0.3142549239722319</v>
+        <v>0.3104931238537325</v>
       </c>
       <c r="D319" t="s">
         <v>7</v>
@@ -9766,7 +9766,7 @@
         <v>15</v>
       </c>
       <c r="C320">
-        <v>0.2712017216778262</v>
+        <v>0.2684752809125104</v>
       </c>
       <c r="D320" t="s">
         <v>7</v>
@@ -9783,7 +9783,7 @@
         <v>6</v>
       </c>
       <c r="C321">
-        <v>0.309562728182086</v>
+        <v>0.3077015350180304</v>
       </c>
       <c r="D321" t="s">
         <v>7</v>
@@ -9800,7 +9800,7 @@
         <v>6</v>
       </c>
       <c r="C322">
-        <v>0.4335211909117278</v>
+        <v>0.4309639870595725</v>
       </c>
       <c r="D322" t="s">
         <v>7</v>
@@ -9817,7 +9817,7 @@
         <v>10</v>
       </c>
       <c r="C323">
-        <v>0.4058365174089516</v>
+        <v>0.4037207406727693</v>
       </c>
       <c r="D323" t="s">
         <v>7</v>
@@ -9834,7 +9834,7 @@
         <v>44</v>
       </c>
       <c r="C324">
-        <v>0.4210085744395568</v>
+        <v>0.4207316562536017</v>
       </c>
       <c r="D324" t="s">
         <v>7</v>
@@ -9851,7 +9851,7 @@
         <v>10</v>
       </c>
       <c r="C325">
-        <v>0.2749540226592071</v>
+        <v>0.2721439245213856</v>
       </c>
       <c r="D325" t="s">
         <v>7</v>
@@ -9868,7 +9868,7 @@
         <v>10</v>
       </c>
       <c r="C326">
-        <v>0.3629440808977026</v>
+        <v>0.3611334511097342</v>
       </c>
       <c r="D326" t="s">
         <v>7</v>
@@ -9885,7 +9885,7 @@
         <v>44</v>
       </c>
       <c r="C327">
-        <v>0.3473699753843887</v>
+        <v>0.3479601964053797</v>
       </c>
       <c r="D327" t="s">
         <v>7</v>
@@ -9902,7 +9902,7 @@
         <v>15</v>
       </c>
       <c r="C328">
-        <v>0.2955943871396476</v>
+        <v>0.2898840323285728</v>
       </c>
       <c r="D328" t="s">
         <v>7</v>
@@ -9919,7 +9919,7 @@
         <v>15</v>
       </c>
       <c r="C329">
-        <v>0.3210191544958206</v>
+        <v>0.3169055634290532</v>
       </c>
       <c r="D329" t="s">
         <v>7</v>
@@ -9936,7 +9936,7 @@
         <v>15</v>
       </c>
       <c r="C330">
-        <v>0.3044819590833273</v>
+        <v>0.2993400318562207</v>
       </c>
       <c r="D330" t="s">
         <v>7</v>
@@ -9953,7 +9953,7 @@
         <v>10</v>
       </c>
       <c r="C331">
-        <v>0.3621789566677379</v>
+        <v>0.3603501067594256</v>
       </c>
       <c r="D331" t="s">
         <v>7</v>
@@ -9970,7 +9970,7 @@
         <v>10</v>
       </c>
       <c r="C332">
-        <v>0.3960756227371886</v>
+        <v>0.3929297893005765</v>
       </c>
       <c r="D332" t="s">
         <v>7</v>
@@ -9987,7 +9987,7 @@
         <v>6</v>
       </c>
       <c r="C333">
-        <v>0.4711440114121606</v>
+        <v>0.4630761966751208</v>
       </c>
       <c r="D333" t="s">
         <v>7</v>
@@ -10004,7 +10004,7 @@
         <v>15</v>
       </c>
       <c r="C334">
-        <v>0.3027920816593779</v>
+        <v>0.2964159475548304</v>
       </c>
       <c r="D334" t="s">
         <v>7</v>
@@ -10021,7 +10021,7 @@
         <v>15</v>
       </c>
       <c r="C335">
-        <v>0.3384357220007716</v>
+        <v>0.336588340599565</v>
       </c>
       <c r="D335" t="s">
         <v>7</v>
@@ -10038,7 +10038,7 @@
         <v>10</v>
       </c>
       <c r="C336">
-        <v>0.2955520573676881</v>
+        <v>0.291518623335303</v>
       </c>
       <c r="D336" t="s">
         <v>7</v>
@@ -10055,7 +10055,7 @@
         <v>44</v>
       </c>
       <c r="C337">
-        <v>0.5083904485963793</v>
+        <v>0.5085666676479978</v>
       </c>
       <c r="D337" t="s">
         <v>7</v>
@@ -10072,7 +10072,7 @@
         <v>10</v>
       </c>
       <c r="C338">
-        <v>0.3076671657252991</v>
+        <v>0.3026176483141224</v>
       </c>
       <c r="D338" t="s">
         <v>7</v>
@@ -10089,7 +10089,7 @@
         <v>15</v>
       </c>
       <c r="C339">
-        <v>0.4866788728278647</v>
+        <v>0.4835737570254297</v>
       </c>
       <c r="D339" t="s">
         <v>7</v>
@@ -10106,7 +10106,7 @@
         <v>15</v>
       </c>
       <c r="C340">
-        <v>0.3319224649693254</v>
+        <v>0.3250763958305026</v>
       </c>
       <c r="D340" t="s">
         <v>7</v>
@@ -10123,7 +10123,7 @@
         <v>6</v>
       </c>
       <c r="C341">
-        <v>0.2562049710781969</v>
+        <v>0.2515527063979699</v>
       </c>
       <c r="D341" t="s">
         <v>7</v>
@@ -10140,7 +10140,7 @@
         <v>10</v>
       </c>
       <c r="C342">
-        <v>0.2788386902775188</v>
+        <v>0.274153613802874</v>
       </c>
       <c r="D342" t="s">
         <v>7</v>
@@ -10157,7 +10157,7 @@
         <v>10</v>
       </c>
       <c r="C343">
-        <v>0.4068537796651799</v>
+        <v>0.4042415201152397</v>
       </c>
       <c r="D343" t="s">
         <v>7</v>
@@ -10174,7 +10174,7 @@
         <v>15</v>
       </c>
       <c r="C344">
-        <v>0.3075110764991976</v>
+        <v>0.3045205345537625</v>
       </c>
       <c r="D344" t="s">
         <v>7</v>
@@ -10191,7 +10191,7 @@
         <v>6</v>
       </c>
       <c r="C345">
-        <v>0.3635797524737669</v>
+        <v>0.3594762029946419</v>
       </c>
       <c r="D345" t="s">
         <v>7</v>
@@ -10208,7 +10208,7 @@
         <v>10</v>
       </c>
       <c r="C346">
-        <v>0.3807348232669976</v>
+        <v>0.3753648305355839</v>
       </c>
       <c r="D346" t="s">
         <v>7</v>
@@ -10225,7 +10225,7 @@
         <v>15</v>
       </c>
       <c r="C347">
-        <v>0.3513732134382796</v>
+        <v>0.3455718804031652</v>
       </c>
       <c r="D347" t="s">
         <v>7</v>
@@ -10242,7 +10242,7 @@
         <v>6</v>
       </c>
       <c r="C348">
-        <v>0.3180399291509251</v>
+        <v>0.3074432875627549</v>
       </c>
       <c r="D348" t="s">
         <v>7</v>
@@ -10259,7 +10259,7 @@
         <v>6</v>
       </c>
       <c r="C349">
-        <v>0.5355330991510647</v>
+        <v>0.5135677795918249</v>
       </c>
       <c r="D349" t="s">
         <v>7</v>
@@ -10276,7 +10276,7 @@
         <v>15</v>
       </c>
       <c r="C350">
-        <v>0.3884437293359401</v>
+        <v>0.380637944351854</v>
       </c>
       <c r="D350" t="s">
         <v>7</v>
@@ -10293,7 +10293,7 @@
         <v>79</v>
       </c>
       <c r="C351">
-        <v>0.269424734642764</v>
+        <v>0.30767120650532</v>
       </c>
       <c r="D351" t="s">
         <v>7</v>
@@ -10310,7 +10310,7 @@
         <v>15</v>
       </c>
       <c r="C352">
-        <v>0.4332365231767719</v>
+        <v>0.4273081739045716</v>
       </c>
       <c r="D352" t="s">
         <v>7</v>
@@ -10327,7 +10327,7 @@
         <v>10</v>
       </c>
       <c r="C353">
-        <v>0.3907395632429125</v>
+        <v>0.3880168246785771</v>
       </c>
       <c r="D353" t="s">
         <v>7</v>
@@ -10344,7 +10344,7 @@
         <v>6</v>
       </c>
       <c r="C354">
-        <v>0.2650705888120313</v>
+        <v>0.2613237021323689</v>
       </c>
       <c r="D354" t="s">
         <v>7</v>
@@ -10361,7 +10361,7 @@
         <v>6</v>
       </c>
       <c r="C355">
-        <v>0.3380656660017344</v>
+        <v>0.3301968908866532</v>
       </c>
       <c r="D355" t="s">
         <v>7</v>
@@ -10378,7 +10378,7 @@
         <v>10</v>
       </c>
       <c r="C356">
-        <v>0.3253388590616574</v>
+        <v>0.3212158321852635</v>
       </c>
       <c r="D356" t="s">
         <v>7</v>
@@ -10395,7 +10395,7 @@
         <v>6</v>
       </c>
       <c r="C357">
-        <v>0.4344200158129855</v>
+        <v>0.4308434270464221</v>
       </c>
       <c r="D357" t="s">
         <v>7</v>
@@ -10412,7 +10412,7 @@
         <v>6</v>
       </c>
       <c r="C358">
-        <v>0.3703488318211703</v>
+        <v>0.3566295155066911</v>
       </c>
       <c r="D358" t="s">
         <v>7</v>
@@ -10429,7 +10429,7 @@
         <v>44</v>
       </c>
       <c r="C359">
-        <v>0.4818351331819922</v>
+        <v>0.479474326432445</v>
       </c>
       <c r="D359" t="s">
         <v>7</v>
@@ -10446,7 +10446,7 @@
         <v>6</v>
       </c>
       <c r="C360">
-        <v>0.5018564300612518</v>
+        <v>0.4711771538299555</v>
       </c>
       <c r="D360" t="s">
         <v>7</v>
@@ -10463,7 +10463,7 @@
         <v>15</v>
       </c>
       <c r="C361">
-        <v>0.3179286888901702</v>
+        <v>0.3135592526234125</v>
       </c>
       <c r="D361" t="s">
         <v>7</v>
@@ -10480,7 +10480,7 @@
         <v>6</v>
       </c>
       <c r="C362">
-        <v>0.3343850199301769</v>
+        <v>0.331745313631599</v>
       </c>
       <c r="D362" t="s">
         <v>7</v>
@@ -10497,7 +10497,7 @@
         <v>10</v>
       </c>
       <c r="C363">
-        <v>0.2988635787777628</v>
+        <v>0.2952343981726941</v>
       </c>
       <c r="D363" t="s">
         <v>7</v>
@@ -10514,7 +10514,7 @@
         <v>10</v>
       </c>
       <c r="C364">
-        <v>0.3078490298728246</v>
+        <v>0.3017420958173301</v>
       </c>
       <c r="D364" t="s">
         <v>7</v>
@@ -10531,7 +10531,7 @@
         <v>15</v>
       </c>
       <c r="C365">
-        <v>0.3155836159118277</v>
+        <v>0.3112286518482177</v>
       </c>
       <c r="D365" t="s">
         <v>7</v>
@@ -10548,7 +10548,7 @@
         <v>15</v>
       </c>
       <c r="C366">
-        <v>0.2730510265689933</v>
+        <v>0.2670219647749826</v>
       </c>
       <c r="D366" t="s">
         <v>7</v>
@@ -10565,7 +10565,7 @@
         <v>15</v>
       </c>
       <c r="C367">
-        <v>0.3001816188839767</v>
+        <v>0.2915402487343922</v>
       </c>
       <c r="D367" t="s">
         <v>7</v>
@@ -10582,7 +10582,7 @@
         <v>15</v>
       </c>
       <c r="C368">
-        <v>0.34326543587904</v>
+        <v>0.3393718398705277</v>
       </c>
       <c r="D368" t="s">
         <v>7</v>
@@ -10599,7 +10599,7 @@
         <v>6</v>
       </c>
       <c r="C369">
-        <v>0.4752978901289066</v>
+        <v>0.4648663500347679</v>
       </c>
       <c r="D369" t="s">
         <v>7</v>
@@ -10616,7 +10616,7 @@
         <v>15</v>
       </c>
       <c r="C370">
-        <v>0.3677059874788612</v>
+        <v>0.3633709134090088</v>
       </c>
       <c r="D370" t="s">
         <v>7</v>
@@ -10633,7 +10633,7 @@
         <v>6</v>
       </c>
       <c r="C371">
-        <v>0.5099768483985874</v>
+        <v>0.5026088737105343</v>
       </c>
       <c r="D371" t="s">
         <v>7</v>
@@ -10650,7 +10650,7 @@
         <v>6</v>
       </c>
       <c r="C372">
-        <v>0.3304779804596841</v>
+        <v>0.3251152316613581</v>
       </c>
       <c r="D372" t="s">
         <v>7</v>
@@ -10667,7 +10667,7 @@
         <v>6</v>
       </c>
       <c r="C373">
-        <v>0.4283493391246398</v>
+        <v>0.4230300016133531</v>
       </c>
       <c r="D373" t="s">
         <v>7</v>
@@ -10684,7 +10684,7 @@
         <v>6</v>
       </c>
       <c r="C374">
-        <v>0.5050129438518015</v>
+        <v>0.486606835038531</v>
       </c>
       <c r="D374" t="s">
         <v>7</v>
@@ -10701,7 +10701,7 @@
         <v>6</v>
       </c>
       <c r="C375">
-        <v>0.4432111578560545</v>
+        <v>0.437340702820295</v>
       </c>
       <c r="D375" t="s">
         <v>7</v>
@@ -10718,7 +10718,7 @@
         <v>15</v>
       </c>
       <c r="C376">
-        <v>0.400880816374967</v>
+        <v>0.3986313446715231</v>
       </c>
       <c r="D376" t="s">
         <v>7</v>
@@ -10735,7 +10735,7 @@
         <v>6</v>
       </c>
       <c r="C377">
-        <v>0.5222064043234128</v>
+        <v>0.5134256545794209</v>
       </c>
       <c r="D377" t="s">
         <v>7</v>
@@ -10752,7 +10752,7 @@
         <v>6</v>
       </c>
       <c r="C378">
-        <v>0.282460825437609</v>
+        <v>0.2789083149529728</v>
       </c>
       <c r="D378" t="s">
         <v>7</v>
@@ -10769,7 +10769,7 @@
         <v>10</v>
       </c>
       <c r="C379">
-        <v>0.3150026215436118</v>
+        <v>0.310003296042193</v>
       </c>
       <c r="D379" t="s">
         <v>7</v>
@@ -10786,7 +10786,7 @@
         <v>6</v>
       </c>
       <c r="C380">
-        <v>0.3497363192872168</v>
+        <v>0.3466933329521261</v>
       </c>
       <c r="D380" t="s">
         <v>7</v>
@@ -10803,7 +10803,7 @@
         <v>10</v>
       </c>
       <c r="C381">
-        <v>0.4740058115104633</v>
+        <v>0.4700892345997365</v>
       </c>
       <c r="D381" t="s">
         <v>7</v>
@@ -10820,7 +10820,7 @@
         <v>6</v>
       </c>
       <c r="C382">
-        <v>0.346764465547226</v>
+        <v>0.3454313504928811</v>
       </c>
       <c r="D382" t="s">
         <v>7</v>
@@ -10837,7 +10837,7 @@
         <v>10</v>
       </c>
       <c r="C383">
-        <v>0.373563559915764</v>
+        <v>0.37126231603825</v>
       </c>
       <c r="D383" t="s">
         <v>7</v>
@@ -10854,7 +10854,7 @@
         <v>44</v>
       </c>
       <c r="C384">
-        <v>0.4919147384049176</v>
+        <v>0.4902124071192181</v>
       </c>
       <c r="D384" t="s">
         <v>7</v>
@@ -10871,7 +10871,7 @@
         <v>6</v>
       </c>
       <c r="C385">
-        <v>0.3896018325778609</v>
+        <v>0.3874539757875712</v>
       </c>
       <c r="D385" t="s">
         <v>7</v>
@@ -10888,7 +10888,7 @@
         <v>15</v>
       </c>
       <c r="C386">
-        <v>0.3133180531837769</v>
+        <v>0.3083202079019423</v>
       </c>
       <c r="D386" t="s">
         <v>7</v>
@@ -10905,7 +10905,7 @@
         <v>10</v>
       </c>
       <c r="C387">
-        <v>0.4679781380932894</v>
+        <v>0.4659513775184309</v>
       </c>
       <c r="D387" t="s">
         <v>7</v>
@@ -10922,7 +10922,7 @@
         <v>44</v>
       </c>
       <c r="C388">
-        <v>0.3572038526890338</v>
+        <v>0.3557603004203539</v>
       </c>
       <c r="D388" t="s">
         <v>7</v>
@@ -10939,7 +10939,7 @@
         <v>6</v>
       </c>
       <c r="C389">
-        <v>0.3780470899693529</v>
+        <v>0.375143083036504</v>
       </c>
       <c r="D389" t="s">
         <v>7</v>
@@ -10956,7 +10956,7 @@
         <v>15</v>
       </c>
       <c r="C390">
-        <v>0.3579556075963025</v>
+        <v>0.3526840368731656</v>
       </c>
       <c r="D390" t="s">
         <v>7</v>
@@ -10973,7 +10973,7 @@
         <v>15</v>
       </c>
       <c r="C391">
-        <v>0.3785658851539945</v>
+        <v>0.370976101544301</v>
       </c>
       <c r="D391" t="s">
         <v>7</v>
@@ -10990,7 +10990,7 @@
         <v>10</v>
       </c>
       <c r="C392">
-        <v>0.355741699612033</v>
+        <v>0.3521032507962491</v>
       </c>
       <c r="D392" t="s">
         <v>7</v>
@@ -11007,7 +11007,7 @@
         <v>10</v>
       </c>
       <c r="C393">
-        <v>0.4561117874847074</v>
+        <v>0.4557230412036504</v>
       </c>
       <c r="D393" t="s">
         <v>7</v>
@@ -11024,7 +11024,7 @@
         <v>15</v>
       </c>
       <c r="C394">
-        <v>0.3828111969087217</v>
+        <v>0.3769314186539973</v>
       </c>
       <c r="D394" t="s">
         <v>7</v>
@@ -11041,7 +11041,7 @@
         <v>10</v>
       </c>
       <c r="C395">
-        <v>0.4161448850851163</v>
+        <v>0.4135788296296223</v>
       </c>
       <c r="D395" t="s">
         <v>7</v>
@@ -11058,7 +11058,7 @@
         <v>6</v>
       </c>
       <c r="C396">
-        <v>0.4136607867095036</v>
+        <v>0.4122318510693349</v>
       </c>
       <c r="D396" t="s">
         <v>7</v>
@@ -11075,7 +11075,7 @@
         <v>10</v>
       </c>
       <c r="C397">
-        <v>0.3900709117182337</v>
+        <v>0.3861222079851723</v>
       </c>
       <c r="D397" t="s">
         <v>7</v>
@@ -11092,7 +11092,7 @@
         <v>6</v>
       </c>
       <c r="C398">
-        <v>0.5166344469058195</v>
+        <v>0.4959586570802403</v>
       </c>
       <c r="D398" t="s">
         <v>7</v>
@@ -11109,7 +11109,7 @@
         <v>15</v>
       </c>
       <c r="C399">
-        <v>0.3469227574063841</v>
+        <v>0.3438489741318798</v>
       </c>
       <c r="D399" t="s">
         <v>7</v>
@@ -11126,7 +11126,7 @@
         <v>6</v>
       </c>
       <c r="C400">
-        <v>0.317476785210755</v>
+        <v>0.3163980762472792</v>
       </c>
       <c r="D400" t="s">
         <v>7</v>
@@ -11143,7 +11143,7 @@
         <v>15</v>
       </c>
       <c r="C401">
-        <v>0.4587751895135407</v>
+        <v>0.455643904593342</v>
       </c>
       <c r="D401" t="s">
         <v>7</v>
@@ -11160,7 +11160,7 @@
         <v>6</v>
       </c>
       <c r="C402">
-        <v>0.4019140610892505</v>
+        <v>0.3985413710809583</v>
       </c>
       <c r="D402" t="s">
         <v>7</v>
@@ -11177,7 +11177,7 @@
         <v>6</v>
       </c>
       <c r="C403">
-        <v>0.2931894169464963</v>
+        <v>0.2910514201427636</v>
       </c>
       <c r="D403" t="s">
         <v>7</v>
@@ -11194,7 +11194,7 @@
         <v>44</v>
       </c>
       <c r="C404">
-        <v>0.3173854687910198</v>
+        <v>0.3136715325395758</v>
       </c>
       <c r="D404" t="s">
         <v>7</v>
@@ -11211,7 +11211,7 @@
         <v>6</v>
       </c>
       <c r="C405">
-        <v>0.4205301903818507</v>
+        <v>0.411603161002154</v>
       </c>
       <c r="D405" t="s">
         <v>7</v>
@@ -11225,10 +11225,10 @@
         <v>820</v>
       </c>
       <c r="B406" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="C406">
-        <v>0.4916167964759152</v>
+        <v>0.4921401167383042</v>
       </c>
       <c r="D406" t="s">
         <v>7</v>
@@ -11245,7 +11245,7 @@
         <v>6</v>
       </c>
       <c r="C407">
-        <v>0.3817202312977135</v>
+        <v>0.3789773875830229</v>
       </c>
       <c r="D407" t="s">
         <v>7</v>
@@ -11262,7 +11262,7 @@
         <v>6</v>
       </c>
       <c r="C408">
-        <v>0.4734426073990602</v>
+        <v>0.4646872914404461</v>
       </c>
       <c r="D408" t="s">
         <v>7</v>
@@ -11279,7 +11279,7 @@
         <v>6</v>
       </c>
       <c r="C409">
-        <v>0.5130959572438536</v>
+        <v>0.5082064286438356</v>
       </c>
       <c r="D409" t="s">
         <v>7</v>
@@ -11296,7 +11296,7 @@
         <v>15</v>
       </c>
       <c r="C410">
-        <v>0.3302831339563063</v>
+        <v>0.3254759838537029</v>
       </c>
       <c r="D410" t="s">
         <v>7</v>
@@ -11313,7 +11313,7 @@
         <v>10</v>
       </c>
       <c r="C411">
-        <v>0.3241466270282546</v>
+        <v>0.3197946781767519</v>
       </c>
       <c r="D411" t="s">
         <v>7</v>
@@ -11330,7 +11330,7 @@
         <v>6</v>
       </c>
       <c r="C412">
-        <v>0.4785869478502672</v>
+        <v>0.4757372637002838</v>
       </c>
       <c r="D412" t="s">
         <v>7</v>
@@ -11347,7 +11347,7 @@
         <v>15</v>
       </c>
       <c r="C413">
-        <v>0.2810957467636199</v>
+        <v>0.2762991480379078</v>
       </c>
       <c r="D413" t="s">
         <v>7</v>
@@ -11364,7 +11364,7 @@
         <v>10</v>
       </c>
       <c r="C414">
-        <v>0.3566670128553855</v>
+        <v>0.3541782583901451</v>
       </c>
       <c r="D414" t="s">
         <v>7</v>
@@ -11381,7 +11381,7 @@
         <v>15</v>
       </c>
       <c r="C415">
-        <v>0.3420937850526287</v>
+        <v>0.338694149857548</v>
       </c>
       <c r="D415" t="s">
         <v>7</v>
@@ -11398,7 +11398,7 @@
         <v>15</v>
       </c>
       <c r="C416">
-        <v>0.3742353273248115</v>
+        <v>0.3664711590326702</v>
       </c>
       <c r="D416" t="s">
         <v>7</v>
@@ -11415,7 +11415,7 @@
         <v>6</v>
       </c>
       <c r="C417">
-        <v>0.3198840271206917</v>
+        <v>0.3120896296653531</v>
       </c>
       <c r="D417" t="s">
         <v>7</v>
@@ -11432,7 +11432,7 @@
         <v>44</v>
       </c>
       <c r="C418">
-        <v>0.3181847601448357</v>
+        <v>0.3172456188776043</v>
       </c>
       <c r="D418" t="s">
         <v>7</v>
@@ -11449,7 +11449,7 @@
         <v>15</v>
       </c>
       <c r="C419">
-        <v>0.4143289756792773</v>
+        <v>0.409642998810138</v>
       </c>
       <c r="D419" t="s">
         <v>7</v>
@@ -11466,7 +11466,7 @@
         <v>44</v>
       </c>
       <c r="C420">
-        <v>0.4528897926210088</v>
+        <v>0.4511014777436628</v>
       </c>
       <c r="D420" t="s">
         <v>7</v>
@@ -11483,7 +11483,7 @@
         <v>44</v>
       </c>
       <c r="C421">
-        <v>0.4006252975805643</v>
+        <v>0.3967291701518157</v>
       </c>
       <c r="D421" t="s">
         <v>7</v>
@@ -11500,7 +11500,7 @@
         <v>6</v>
       </c>
       <c r="C422">
-        <v>0.3735265231332319</v>
+        <v>0.3711147863654267</v>
       </c>
       <c r="D422" t="s">
         <v>7</v>
@@ -11517,7 +11517,7 @@
         <v>44</v>
       </c>
       <c r="C423">
-        <v>0.4640165755358109</v>
+        <v>0.4649017336919584</v>
       </c>
       <c r="D423" t="s">
         <v>7</v>
@@ -11534,7 +11534,7 @@
         <v>10</v>
       </c>
       <c r="C424">
-        <v>0.3325229993088122</v>
+        <v>0.3296969371904548</v>
       </c>
       <c r="D424" t="s">
         <v>7</v>
@@ -11551,7 +11551,7 @@
         <v>6</v>
       </c>
       <c r="C425">
-        <v>0.3247809281701205</v>
+        <v>0.3227609808474454</v>
       </c>
       <c r="D425" t="s">
         <v>7</v>
@@ -11568,7 +11568,7 @@
         <v>15</v>
       </c>
       <c r="C426">
-        <v>0.3772309142513167</v>
+        <v>0.3742120209534412</v>
       </c>
       <c r="D426" t="s">
         <v>7</v>
@@ -11585,7 +11585,7 @@
         <v>15</v>
       </c>
       <c r="C427">
-        <v>0.2608351460719957</v>
+        <v>0.2566696528212971</v>
       </c>
       <c r="D427" t="s">
         <v>7</v>
@@ -11602,7 +11602,7 @@
         <v>15</v>
       </c>
       <c r="C428">
-        <v>0.2793402396159717</v>
+        <v>0.2747590284037176</v>
       </c>
       <c r="D428" t="s">
         <v>7</v>
@@ -11619,7 +11619,7 @@
         <v>10</v>
       </c>
       <c r="C429">
-        <v>0.3836820575179162</v>
+        <v>0.3781873244582644</v>
       </c>
       <c r="D429" t="s">
         <v>7</v>
@@ -11636,7 +11636,7 @@
         <v>6</v>
       </c>
       <c r="C430">
-        <v>0.3160536192646429</v>
+        <v>0.3118507017086689</v>
       </c>
       <c r="D430" t="s">
         <v>7</v>
@@ -11653,7 +11653,7 @@
         <v>15</v>
       </c>
       <c r="C431">
-        <v>0.2998975711920567</v>
+        <v>0.2928670506584419</v>
       </c>
       <c r="D431" t="s">
         <v>7</v>
@@ -11670,7 +11670,7 @@
         <v>15</v>
       </c>
       <c r="C432">
-        <v>0.331597973018401</v>
+        <v>0.3286567825375022</v>
       </c>
       <c r="D432" t="s">
         <v>7</v>
@@ -11687,7 +11687,7 @@
         <v>6</v>
       </c>
       <c r="C433">
-        <v>0.3185244884909684</v>
+        <v>0.3173235009287645</v>
       </c>
       <c r="D433" t="s">
         <v>7</v>
@@ -11704,7 +11704,7 @@
         <v>15</v>
       </c>
       <c r="C434">
-        <v>0.3616339994183591</v>
+        <v>0.3585622753600495</v>
       </c>
       <c r="D434" t="s">
         <v>7</v>
@@ -11721,7 +11721,7 @@
         <v>10</v>
       </c>
       <c r="C435">
-        <v>0.426279773788339</v>
+        <v>0.4251448969871074</v>
       </c>
       <c r="D435" t="s">
         <v>7</v>
@@ -11738,7 +11738,7 @@
         <v>15</v>
       </c>
       <c r="C436">
-        <v>0.3591371610925511</v>
+        <v>0.3539190868136093</v>
       </c>
       <c r="D436" t="s">
         <v>7</v>
@@ -11755,7 +11755,7 @@
         <v>10</v>
       </c>
       <c r="C437">
-        <v>0.3331881383000567</v>
+        <v>0.3307273956499053</v>
       </c>
       <c r="D437" t="s">
         <v>7</v>
@@ -11772,7 +11772,7 @@
         <v>15</v>
       </c>
       <c r="C438">
-        <v>0.3953120153372238</v>
+        <v>0.387522960156024</v>
       </c>
       <c r="D438" t="s">
         <v>7</v>
@@ -11789,7 +11789,7 @@
         <v>6</v>
       </c>
       <c r="C439">
-        <v>0.3424144269501241</v>
+        <v>0.3305297324265407</v>
       </c>
       <c r="D439" t="s">
         <v>7</v>
@@ -11806,7 +11806,7 @@
         <v>10</v>
       </c>
       <c r="C440">
-        <v>0.3412019405599855</v>
+        <v>0.337231621835752</v>
       </c>
       <c r="D440" t="s">
         <v>7</v>
@@ -11823,7 +11823,7 @@
         <v>15</v>
       </c>
       <c r="C441">
-        <v>0.3039308640375215</v>
+        <v>0.298044032831654</v>
       </c>
       <c r="D441" t="s">
         <v>7</v>
@@ -11840,7 +11840,7 @@
         <v>6</v>
       </c>
       <c r="C442">
-        <v>0.3635243741334956</v>
+        <v>0.356901196531142</v>
       </c>
       <c r="D442" t="s">
         <v>7</v>
@@ -11857,7 +11857,7 @@
         <v>15</v>
       </c>
       <c r="C443">
-        <v>0.3113812451305115</v>
+        <v>0.307011368204434</v>
       </c>
       <c r="D443" t="s">
         <v>7</v>
@@ -11874,7 +11874,7 @@
         <v>10</v>
       </c>
       <c r="C444">
-        <v>0.3377911189301578</v>
+        <v>0.3373965553600082</v>
       </c>
       <c r="D444" t="s">
         <v>7</v>
@@ -11891,7 +11891,7 @@
         <v>6</v>
       </c>
       <c r="C445">
-        <v>0.3497565401390224</v>
+        <v>0.345558195433679</v>
       </c>
       <c r="D445" t="s">
         <v>7</v>
@@ -11908,7 +11908,7 @@
         <v>44</v>
       </c>
       <c r="C446">
-        <v>0.3922462912833353</v>
+        <v>0.3885195372491845</v>
       </c>
       <c r="D446" t="s">
         <v>7</v>
@@ -11925,7 +11925,7 @@
         <v>15</v>
       </c>
       <c r="C447">
-        <v>0.3041494228845325</v>
+        <v>0.3005308970286985</v>
       </c>
       <c r="D447" t="s">
         <v>7</v>
@@ -11942,7 +11942,7 @@
         <v>6</v>
       </c>
       <c r="C448">
-        <v>0.3988597409304627</v>
+        <v>0.3927395997134802</v>
       </c>
       <c r="D448" t="s">
         <v>7</v>
@@ -11959,7 +11959,7 @@
         <v>6</v>
       </c>
       <c r="C449">
-        <v>0.3762184921137278</v>
+        <v>0.373596095360096</v>
       </c>
       <c r="D449" t="s">
         <v>7</v>
@@ -11976,7 +11976,7 @@
         <v>44</v>
       </c>
       <c r="C450">
-        <v>0.3703665128163428</v>
+        <v>0.3703940658628674</v>
       </c>
       <c r="D450" t="s">
         <v>7</v>
@@ -11993,7 +11993,7 @@
         <v>44</v>
       </c>
       <c r="C451">
-        <v>0.4568756961313837</v>
+        <v>0.4546029615767068</v>
       </c>
       <c r="D451" t="s">
         <v>7</v>
@@ -12010,7 +12010,7 @@
         <v>6</v>
       </c>
       <c r="C452">
-        <v>0.2827762978712109</v>
+        <v>0.2793662839734509</v>
       </c>
       <c r="D452" t="s">
         <v>7</v>
@@ -12027,7 +12027,7 @@
         <v>10</v>
       </c>
       <c r="C453">
-        <v>0.3941841036599131</v>
+        <v>0.3918001031817109</v>
       </c>
       <c r="D453" t="s">
         <v>7</v>
@@ -12044,7 +12044,7 @@
         <v>15</v>
       </c>
       <c r="C454">
-        <v>0.2947473069018948</v>
+        <v>0.2880072373896687</v>
       </c>
       <c r="D454" t="s">
         <v>7</v>
@@ -12061,7 +12061,7 @@
         <v>10</v>
       </c>
       <c r="C455">
-        <v>0.3309425170789219</v>
+        <v>0.3265079782558651</v>
       </c>
       <c r="D455" t="s">
         <v>7</v>
@@ -12078,7 +12078,7 @@
         <v>6</v>
       </c>
       <c r="C456">
-        <v>0.3505895778151284</v>
+        <v>0.3368104496784967</v>
       </c>
       <c r="D456" t="s">
         <v>7</v>
@@ -12095,7 +12095,7 @@
         <v>15</v>
       </c>
       <c r="C457">
-        <v>0.3872018054345991</v>
+        <v>0.3813446338888398</v>
       </c>
       <c r="D457" t="s">
         <v>7</v>
@@ -12112,7 +12112,7 @@
         <v>6</v>
       </c>
       <c r="C458">
-        <v>0.3357582341024452</v>
+        <v>0.3342329174955648</v>
       </c>
       <c r="D458" t="s">
         <v>7</v>
@@ -12129,7 +12129,7 @@
         <v>6</v>
       </c>
       <c r="C459">
-        <v>0.3507381635844327</v>
+        <v>0.3434806358538459</v>
       </c>
       <c r="D459" t="s">
         <v>7</v>
@@ -12146,7 +12146,7 @@
         <v>15</v>
       </c>
       <c r="C460">
-        <v>0.3898248151995047</v>
+        <v>0.3818033641680585</v>
       </c>
       <c r="D460" t="s">
         <v>7</v>
@@ -12163,7 +12163,7 @@
         <v>10</v>
       </c>
       <c r="C461">
-        <v>0.3292635202021108</v>
+        <v>0.3259337062344202</v>
       </c>
       <c r="D461" t="s">
         <v>7</v>
@@ -12180,7 +12180,7 @@
         <v>10</v>
       </c>
       <c r="C462">
-        <v>0.3020884787026801</v>
+        <v>0.2984958893624328</v>
       </c>
       <c r="D462" t="s">
         <v>7</v>
@@ -12197,7 +12197,7 @@
         <v>15</v>
       </c>
       <c r="C463">
-        <v>0.3290988686133663</v>
+        <v>0.3243299808650127</v>
       </c>
       <c r="D463" t="s">
         <v>7</v>
@@ -12214,7 +12214,7 @@
         <v>6</v>
       </c>
       <c r="C464">
-        <v>0.4401225507382625</v>
+        <v>0.4231239800959847</v>
       </c>
       <c r="D464" t="s">
         <v>7</v>
@@ -12231,7 +12231,7 @@
         <v>44</v>
       </c>
       <c r="C465">
-        <v>0.4056166773141336</v>
+        <v>0.4056076483756846</v>
       </c>
       <c r="D465" t="s">
         <v>7</v>
@@ -12248,7 +12248,7 @@
         <v>6</v>
       </c>
       <c r="C466">
-        <v>0.5711362775788509</v>
+        <v>0.5596277970509876</v>
       </c>
       <c r="D466" t="s">
         <v>7</v>
@@ -12265,7 +12265,7 @@
         <v>6</v>
       </c>
       <c r="C467">
-        <v>0.4615192046468659</v>
+        <v>0.4521557149116521</v>
       </c>
       <c r="D467" t="s">
         <v>7</v>
@@ -12282,7 +12282,7 @@
         <v>6</v>
       </c>
       <c r="C468">
-        <v>0.4069828858218998</v>
+        <v>0.4019611026499396</v>
       </c>
       <c r="D468" t="s">
         <v>7</v>
@@ -12299,7 +12299,7 @@
         <v>15</v>
       </c>
       <c r="C469">
-        <v>0.3018741319553296</v>
+        <v>0.2973591291999924</v>
       </c>
       <c r="D469" t="s">
         <v>7</v>
@@ -12316,7 +12316,7 @@
         <v>6</v>
       </c>
       <c r="C470">
-        <v>0.337776417518129</v>
+        <v>0.3317357216997716</v>
       </c>
       <c r="D470" t="s">
         <v>7</v>
@@ -12333,7 +12333,7 @@
         <v>10</v>
       </c>
       <c r="C471">
-        <v>0.3351166778175548</v>
+        <v>0.3337370101010737</v>
       </c>
       <c r="D471" t="s">
         <v>7</v>
@@ -12350,7 +12350,7 @@
         <v>15</v>
       </c>
       <c r="C472">
-        <v>0.3616106943071908</v>
+        <v>0.3591736066826279</v>
       </c>
       <c r="D472" t="s">
         <v>7</v>
@@ -12367,7 +12367,7 @@
         <v>10</v>
       </c>
       <c r="C473">
-        <v>0.3561869227662535</v>
+        <v>0.3533643581800312</v>
       </c>
       <c r="D473" t="s">
         <v>7</v>
@@ -12384,7 +12384,7 @@
         <v>10</v>
       </c>
       <c r="C474">
-        <v>0.3880470330068618</v>
+        <v>0.3847727530628554</v>
       </c>
       <c r="D474" t="s">
         <v>7</v>
@@ -12401,7 +12401,7 @@
         <v>6</v>
       </c>
       <c r="C475">
-        <v>0.3742631477366594</v>
+        <v>0.3698874186053104</v>
       </c>
       <c r="D475" t="s">
         <v>7</v>
@@ -12418,7 +12418,7 @@
         <v>6</v>
       </c>
       <c r="C476">
-        <v>0.3166353472815191</v>
+        <v>0.3131162654506845</v>
       </c>
       <c r="D476" t="s">
         <v>7</v>
@@ -12435,7 +12435,7 @@
         <v>15</v>
       </c>
       <c r="C477">
-        <v>0.3534526540337829</v>
+        <v>0.3491023713723275</v>
       </c>
       <c r="D477" t="s">
         <v>7</v>
@@ -12452,7 +12452,7 @@
         <v>6</v>
       </c>
       <c r="C478">
-        <v>0.4223264987054359</v>
+        <v>0.4213605830994959</v>
       </c>
       <c r="D478" t="s">
         <v>7</v>
@@ -12469,7 +12469,7 @@
         <v>44</v>
       </c>
       <c r="C479">
-        <v>0.4200488163297086</v>
+        <v>0.4180003837685235</v>
       </c>
       <c r="D479" t="s">
         <v>7</v>
@@ -12486,7 +12486,7 @@
         <v>6</v>
       </c>
       <c r="C480">
-        <v>0.4514351849346507</v>
+        <v>0.4453502421266167</v>
       </c>
       <c r="D480" t="s">
         <v>7</v>
@@ -12503,7 +12503,7 @@
         <v>44</v>
       </c>
       <c r="C481">
-        <v>0.3811394420795335</v>
+        <v>0.3792799669648689</v>
       </c>
       <c r="D481" t="s">
         <v>7</v>
@@ -12520,7 +12520,7 @@
         <v>10</v>
       </c>
       <c r="C482">
-        <v>0.3288384918364493</v>
+        <v>0.3261032386568871</v>
       </c>
       <c r="D482" t="s">
         <v>7</v>
@@ -12537,7 +12537,7 @@
         <v>10</v>
       </c>
       <c r="C483">
-        <v>0.3446280567111195</v>
+        <v>0.3425985754053199</v>
       </c>
       <c r="D483" t="s">
         <v>7</v>
@@ -12554,7 +12554,7 @@
         <v>44</v>
       </c>
       <c r="C484">
-        <v>0.3820042284062229</v>
+        <v>0.3787477239025471</v>
       </c>
       <c r="D484" t="s">
         <v>7</v>
@@ -12571,7 +12571,7 @@
         <v>15</v>
       </c>
       <c r="C485">
-        <v>0.4024708034122653</v>
+        <v>0.3950721030284169</v>
       </c>
       <c r="D485" t="s">
         <v>7</v>
@@ -12588,7 +12588,7 @@
         <v>15</v>
       </c>
       <c r="C486">
-        <v>0.4226357280140805</v>
+        <v>0.416995168831459</v>
       </c>
       <c r="D486" t="s">
         <v>7</v>
@@ -12605,7 +12605,7 @@
         <v>44</v>
       </c>
       <c r="C487">
-        <v>0.4509265078934047</v>
+        <v>0.4492242609525252</v>
       </c>
       <c r="D487" t="s">
         <v>7</v>
@@ -12622,7 +12622,7 @@
         <v>10</v>
       </c>
       <c r="C488">
-        <v>0.3837807891370171</v>
+        <v>0.3779315381115447</v>
       </c>
       <c r="D488" t="s">
         <v>7</v>
@@ -12639,7 +12639,7 @@
         <v>6</v>
       </c>
       <c r="C489">
-        <v>0.4968743394763223</v>
+        <v>0.484355452486484</v>
       </c>
       <c r="D489" t="s">
         <v>7</v>
@@ -12656,7 +12656,7 @@
         <v>15</v>
       </c>
       <c r="C490">
-        <v>0.3428082574731809</v>
+        <v>0.3395734071927177</v>
       </c>
       <c r="D490" t="s">
         <v>7</v>
@@ -12673,7 +12673,7 @@
         <v>15</v>
       </c>
       <c r="C491">
-        <v>0.281045675292399</v>
+        <v>0.276806746553911</v>
       </c>
       <c r="D491" t="s">
         <v>7</v>
@@ -12690,7 +12690,7 @@
         <v>6</v>
       </c>
       <c r="C492">
-        <v>0.5304550786594751</v>
+        <v>0.4999140627748311</v>
       </c>
       <c r="D492" t="s">
         <v>7</v>
@@ -12707,7 +12707,7 @@
         <v>6</v>
       </c>
       <c r="C493">
-        <v>0.3295031102426207</v>
+        <v>0.3261759260719906</v>
       </c>
       <c r="D493" t="s">
         <v>7</v>
@@ -12724,7 +12724,7 @@
         <v>44</v>
       </c>
       <c r="C494">
-        <v>0.3193176679625419</v>
+        <v>0.3144698561178459</v>
       </c>
       <c r="D494" t="s">
         <v>7</v>
@@ -12741,7 +12741,7 @@
         <v>44</v>
       </c>
       <c r="C495">
-        <v>0.5471474828345227</v>
+        <v>0.5464291554632484</v>
       </c>
       <c r="D495" t="s">
         <v>7</v>
@@ -12758,7 +12758,7 @@
         <v>6</v>
       </c>
       <c r="C496">
-        <v>0.4905229698219487</v>
+        <v>0.4871059457615867</v>
       </c>
       <c r="D496" t="s">
         <v>7</v>
@@ -12775,7 +12775,7 @@
         <v>10</v>
       </c>
       <c r="C497">
-        <v>0.3751617727867874</v>
+        <v>0.369356228360872</v>
       </c>
       <c r="D497" t="s">
         <v>7</v>
@@ -12792,7 +12792,7 @@
         <v>6</v>
       </c>
       <c r="C498">
-        <v>0.7208180903680157</v>
+        <v>0.6990401241405413</v>
       </c>
       <c r="D498" t="s">
         <v>7</v>
@@ -12809,7 +12809,7 @@
         <v>15</v>
       </c>
       <c r="C499">
-        <v>0.4164872252154111</v>
+        <v>0.4114278043485819</v>
       </c>
       <c r="D499" t="s">
         <v>7</v>
@@ -12826,7 +12826,7 @@
         <v>6</v>
       </c>
       <c r="C500">
-        <v>0.3943267507387416</v>
+        <v>0.3886298683993562</v>
       </c>
       <c r="D500" t="s">
         <v>7</v>
@@ -12843,7 +12843,7 @@
         <v>15</v>
       </c>
       <c r="C501">
-        <v>0.3728521907159971</v>
+        <v>0.3664631868487004</v>
       </c>
       <c r="D501" t="s">
         <v>7</v>
@@ -12860,7 +12860,7 @@
         <v>6</v>
       </c>
       <c r="C502">
-        <v>0.6301891065138235</v>
+        <v>0.615994367220091</v>
       </c>
       <c r="D502" t="s">
         <v>7</v>
@@ -12877,7 +12877,7 @@
         <v>15</v>
       </c>
       <c r="C503">
-        <v>0.3821492204497333</v>
+        <v>0.3737009139590765</v>
       </c>
       <c r="D503" t="s">
         <v>7</v>
@@ -12894,7 +12894,7 @@
         <v>15</v>
       </c>
       <c r="C504">
-        <v>0.3123464980621902</v>
+        <v>0.306685729211892</v>
       </c>
       <c r="D504" t="s">
         <v>7</v>
@@ -12911,7 +12911,7 @@
         <v>6</v>
       </c>
       <c r="C505">
-        <v>0.4573156491572166</v>
+        <v>0.4533850176780899</v>
       </c>
       <c r="D505" t="s">
         <v>7</v>
@@ -12928,7 +12928,7 @@
         <v>15</v>
       </c>
       <c r="C506">
-        <v>0.4966510128918018</v>
+        <v>0.4906347149838955</v>
       </c>
       <c r="D506" t="s">
         <v>7</v>
@@ -12945,7 +12945,7 @@
         <v>10</v>
       </c>
       <c r="C507">
-        <v>0.3226515520479352</v>
+        <v>0.318034494234029</v>
       </c>
       <c r="D507" t="s">
         <v>7</v>
@@ -12962,7 +12962,7 @@
         <v>15</v>
       </c>
       <c r="C508">
-        <v>0.3581285198657512</v>
+        <v>0.3499279547098815</v>
       </c>
       <c r="D508" t="s">
         <v>7</v>
@@ -12979,7 +12979,7 @@
         <v>10</v>
       </c>
       <c r="C509">
-        <v>0.4868700420546586</v>
+        <v>0.4871169910017538</v>
       </c>
       <c r="D509" t="s">
         <v>7</v>
@@ -12996,7 +12996,7 @@
         <v>10</v>
       </c>
       <c r="C510">
-        <v>0.3832140657500053</v>
+        <v>0.3791164715424325</v>
       </c>
       <c r="D510" t="s">
         <v>7</v>
@@ -13013,7 +13013,7 @@
         <v>44</v>
       </c>
       <c r="C511">
-        <v>0.4002956522463696</v>
+        <v>0.3984104313729391</v>
       </c>
       <c r="D511" t="s">
         <v>7</v>
@@ -13030,7 +13030,7 @@
         <v>6</v>
       </c>
       <c r="C512">
-        <v>0.2945093231863476</v>
+        <v>0.2927760512283072</v>
       </c>
       <c r="D512" t="s">
         <v>7</v>
@@ -13047,7 +13047,7 @@
         <v>6</v>
       </c>
       <c r="C513">
-        <v>0.389275447609536</v>
+        <v>0.3819438445224634</v>
       </c>
       <c r="D513" t="s">
         <v>7</v>
@@ -13064,7 +13064,7 @@
         <v>44</v>
       </c>
       <c r="C514">
-        <v>0.4245501843823383</v>
+        <v>0.4249131398562046</v>
       </c>
       <c r="D514" t="s">
         <v>7</v>
@@ -13081,7 +13081,7 @@
         <v>6</v>
       </c>
       <c r="C515">
-        <v>0.5617419992367746</v>
+        <v>0.5480627802357901</v>
       </c>
       <c r="D515" t="s">
         <v>7</v>
@@ -13098,7 +13098,7 @@
         <v>6</v>
       </c>
       <c r="C516">
-        <v>0.3103045015107687</v>
+        <v>0.308006647019007</v>
       </c>
       <c r="D516" t="s">
         <v>7</v>
@@ -13115,7 +13115,7 @@
         <v>15</v>
       </c>
       <c r="C517">
-        <v>0.3360781606157007</v>
+        <v>0.3317361866030943</v>
       </c>
       <c r="D517" t="s">
         <v>7</v>
@@ -13132,7 +13132,7 @@
         <v>10</v>
       </c>
       <c r="C518">
-        <v>0.3342259312229136</v>
+        <v>0.3310945920211142</v>
       </c>
       <c r="D518" t="s">
         <v>7</v>
@@ -13149,7 +13149,7 @@
         <v>44</v>
       </c>
       <c r="C519">
-        <v>0.481233076827528</v>
+        <v>0.4801018212364839</v>
       </c>
       <c r="D519" t="s">
         <v>7</v>
@@ -13166,7 +13166,7 @@
         <v>15</v>
       </c>
       <c r="C520">
-        <v>0.3477510435961427</v>
+        <v>0.3423448541208454</v>
       </c>
       <c r="D520" t="s">
         <v>7</v>
@@ -13183,7 +13183,7 @@
         <v>10</v>
       </c>
       <c r="C521">
-        <v>0.3332957457588769</v>
+        <v>0.3287231787463962</v>
       </c>
       <c r="D521" t="s">
         <v>7</v>
@@ -13200,7 +13200,7 @@
         <v>15</v>
       </c>
       <c r="C522">
-        <v>0.3739859518526156</v>
+        <v>0.3684477926033294</v>
       </c>
       <c r="D522" t="s">
         <v>7</v>
@@ -13217,7 +13217,7 @@
         <v>6</v>
       </c>
       <c r="C523">
-        <v>0.4547305845510159</v>
+        <v>0.4522050526536761</v>
       </c>
       <c r="D523" t="s">
         <v>7</v>
@@ -13234,7 +13234,7 @@
         <v>6</v>
       </c>
       <c r="C524">
-        <v>0.2949141063007796</v>
+        <v>0.2876506084706189</v>
       </c>
       <c r="D524" t="s">
         <v>7</v>
@@ -13251,7 +13251,7 @@
         <v>44</v>
       </c>
       <c r="C525">
-        <v>0.4526918593537551</v>
+        <v>0.4459967989335649</v>
       </c>
       <c r="D525" t="s">
         <v>7</v>
@@ -13268,7 +13268,7 @@
         <v>44</v>
       </c>
       <c r="C526">
-        <v>0.452569278729548</v>
+        <v>0.4485744324122278</v>
       </c>
       <c r="D526" t="s">
         <v>7</v>
@@ -13285,7 +13285,7 @@
         <v>10</v>
       </c>
       <c r="C527">
-        <v>0.3761839404766265</v>
+        <v>0.3722775368526367</v>
       </c>
       <c r="D527" t="s">
         <v>7</v>
@@ -13302,7 +13302,7 @@
         <v>6</v>
       </c>
       <c r="C528">
-        <v>0.4737974547594956</v>
+        <v>0.4676748415016272</v>
       </c>
       <c r="D528" t="s">
         <v>7</v>
@@ -13319,7 +13319,7 @@
         <v>10</v>
       </c>
       <c r="C529">
-        <v>0.3481609487251634</v>
+        <v>0.3461130979107216</v>
       </c>
       <c r="D529" t="s">
         <v>7</v>
@@ -13336,7 +13336,7 @@
         <v>44</v>
       </c>
       <c r="C530">
-        <v>0.5070412521509874</v>
+        <v>0.5044745212910274</v>
       </c>
       <c r="D530" t="s">
         <v>7</v>
@@ -13353,7 +13353,7 @@
         <v>44</v>
       </c>
       <c r="C531">
-        <v>0.6060838145642971</v>
+        <v>0.6030733673507404</v>
       </c>
       <c r="D531" t="s">
         <v>7</v>
@@ -13370,7 +13370,7 @@
         <v>44</v>
       </c>
       <c r="C532">
-        <v>0.3157390365205732</v>
+        <v>0.3132517331555756</v>
       </c>
       <c r="D532" t="s">
         <v>7</v>
@@ -13387,7 +13387,7 @@
         <v>15</v>
       </c>
       <c r="C533">
-        <v>0.4727195100380562</v>
+        <v>0.4656702283479625</v>
       </c>
       <c r="D533" t="s">
         <v>7</v>
@@ -13404,7 +13404,7 @@
         <v>15</v>
       </c>
       <c r="C534">
-        <v>0.3199035927362817</v>
+        <v>0.3114998073613152</v>
       </c>
       <c r="D534" t="s">
         <v>7</v>
@@ -13421,7 +13421,7 @@
         <v>6</v>
       </c>
       <c r="C535">
-        <v>0.3023043600393073</v>
+        <v>0.3001928280825698</v>
       </c>
       <c r="D535" t="s">
         <v>7</v>
@@ -13438,7 +13438,7 @@
         <v>15</v>
       </c>
       <c r="C536">
-        <v>0.3221586764954804</v>
+        <v>0.3171837533315937</v>
       </c>
       <c r="D536" t="s">
         <v>7</v>
@@ -13455,7 +13455,7 @@
         <v>6</v>
       </c>
       <c r="C537">
-        <v>0.4222813201451429</v>
+        <v>0.4152060755926826</v>
       </c>
       <c r="D537" t="s">
         <v>7</v>
@@ -13472,7 +13472,7 @@
         <v>15</v>
       </c>
       <c r="C538">
-        <v>0.2949399381791736</v>
+        <v>0.2907657776595584</v>
       </c>
       <c r="D538" t="s">
         <v>7</v>
@@ -13489,7 +13489,7 @@
         <v>6</v>
       </c>
       <c r="C539">
-        <v>0.3095952973161565</v>
+        <v>0.3060678668152193</v>
       </c>
       <c r="D539" t="s">
         <v>7</v>
@@ -13506,7 +13506,7 @@
         <v>15</v>
       </c>
       <c r="C540">
-        <v>0.2881023938442137</v>
+        <v>0.283939379391095</v>
       </c>
       <c r="D540" t="s">
         <v>7</v>
@@ -13523,7 +13523,7 @@
         <v>6</v>
       </c>
       <c r="C541">
-        <v>0.4452570861377024</v>
+        <v>0.4416864847108284</v>
       </c>
       <c r="D541" t="s">
         <v>7</v>
@@ -13540,7 +13540,7 @@
         <v>44</v>
       </c>
       <c r="C542">
-        <v>0.4030427253243088</v>
+        <v>0.4003353632535511</v>
       </c>
       <c r="D542" t="s">
         <v>7</v>
@@ -13557,7 +13557,7 @@
         <v>6</v>
       </c>
       <c r="C543">
-        <v>0.4522944302958911</v>
+        <v>0.4343917864809401</v>
       </c>
       <c r="D543" t="s">
         <v>7</v>
@@ -13574,7 +13574,7 @@
         <v>6</v>
       </c>
       <c r="C544">
-        <v>0.3765856908900599</v>
+        <v>0.3728560145159255</v>
       </c>
       <c r="D544" t="s">
         <v>7</v>
@@ -15371,7 +15371,7 @@
         <v>15</v>
       </c>
       <c r="B2">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -15379,7 +15379,7 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -15387,7 +15387,7 @@
         <v>79</v>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -15395,7 +15395,7 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:2">

</xml_diff>

<commit_message>
updated aggregator for Scotland - new polling source
</commit_message>
<xml_diff>
--- a/frontend/data/uk_election_predictions.xlsx
+++ b/frontend/data/uk_election_predictions.xlsx
@@ -13843,7 +13843,7 @@
         <v>1143</v>
       </c>
       <c r="C563">
-        <v>0.3032762648047834</v>
+        <v>0.2778510537375036</v>
       </c>
       <c r="D563" t="s">
         <v>1144</v>
@@ -13860,7 +13860,7 @@
         <v>1143</v>
       </c>
       <c r="C564">
-        <v>0.3531039416695648</v>
+        <v>0.3278804824240203</v>
       </c>
       <c r="D564" t="s">
         <v>1144</v>
@@ -13877,7 +13877,7 @@
         <v>1143</v>
       </c>
       <c r="C565">
-        <v>0.3076666390457057</v>
+        <v>0.2751971003895707</v>
       </c>
       <c r="D565" t="s">
         <v>1144</v>
@@ -13894,7 +13894,7 @@
         <v>1143</v>
       </c>
       <c r="C566">
-        <v>0.4907216867804695</v>
+        <v>0.4574381408777259</v>
       </c>
       <c r="D566" t="s">
         <v>1144</v>
@@ -13911,7 +13911,7 @@
         <v>1143</v>
       </c>
       <c r="C567">
-        <v>0.4238249431858235</v>
+        <v>0.3954275260752005</v>
       </c>
       <c r="D567" t="s">
         <v>1144</v>
@@ -13928,7 +13928,7 @@
         <v>1143</v>
       </c>
       <c r="C568">
-        <v>0.3684223588301463</v>
+        <v>0.3429164531248907</v>
       </c>
       <c r="D568" t="s">
         <v>1144</v>
@@ -13945,7 +13945,7 @@
         <v>1143</v>
       </c>
       <c r="C569">
-        <v>0.3066190561849952</v>
+        <v>0.2807094492642338</v>
       </c>
       <c r="D569" t="s">
         <v>1144</v>
@@ -13959,10 +13959,10 @@
         <v>1158</v>
       </c>
       <c r="B570" t="s">
-        <v>1143</v>
+        <v>10</v>
       </c>
       <c r="C570">
-        <v>0.3098005487786876</v>
+        <v>0.2961480648555327</v>
       </c>
       <c r="D570" t="s">
         <v>1144</v>
@@ -13979,7 +13979,7 @@
         <v>1143</v>
       </c>
       <c r="C571">
-        <v>0.3025596542441778</v>
+        <v>0.2767573836990959</v>
       </c>
       <c r="D571" t="s">
         <v>1144</v>
@@ -13996,7 +13996,7 @@
         <v>1143</v>
       </c>
       <c r="C572">
-        <v>0.3597870223807797</v>
+        <v>0.3324425591822937</v>
       </c>
       <c r="D572" t="s">
         <v>1144</v>
@@ -14013,7 +14013,7 @@
         <v>1143</v>
       </c>
       <c r="C573">
-        <v>0.3050634886121578</v>
+        <v>0.2811055033079313</v>
       </c>
       <c r="D573" t="s">
         <v>1144</v>
@@ -14030,7 +14030,7 @@
         <v>45</v>
       </c>
       <c r="C574">
-        <v>0.3227511442277982</v>
+        <v>0.335414871319458</v>
       </c>
       <c r="D574" t="s">
         <v>1144</v>
@@ -14047,7 +14047,7 @@
         <v>1143</v>
       </c>
       <c r="C575">
-        <v>0.3371033177670684</v>
+        <v>0.3071793543488098</v>
       </c>
       <c r="D575" t="s">
         <v>1144</v>
@@ -14064,7 +14064,7 @@
         <v>1143</v>
       </c>
       <c r="C576">
-        <v>0.3897751160083814</v>
+        <v>0.3604746859907967</v>
       </c>
       <c r="D576" t="s">
         <v>1144</v>
@@ -14078,10 +14078,10 @@
         <v>1172</v>
       </c>
       <c r="B577" t="s">
-        <v>1143</v>
+        <v>6</v>
       </c>
       <c r="C577">
-        <v>0.2841597472232418</v>
+        <v>0.3033545451788696</v>
       </c>
       <c r="D577" t="s">
         <v>1144</v>
@@ -14098,7 +14098,7 @@
         <v>1143</v>
       </c>
       <c r="C578">
-        <v>0.3890065758143285</v>
+        <v>0.3596182830515524</v>
       </c>
       <c r="D578" t="s">
         <v>1144</v>
@@ -14115,7 +14115,7 @@
         <v>1143</v>
       </c>
       <c r="C579">
-        <v>0.3281385619552016</v>
+        <v>0.3015362942315583</v>
       </c>
       <c r="D579" t="s">
         <v>1144</v>
@@ -14132,7 +14132,7 @@
         <v>10</v>
       </c>
       <c r="C580">
-        <v>0.3685731822947451</v>
+        <v>0.3692136422589501</v>
       </c>
       <c r="D580" t="s">
         <v>1144</v>
@@ -14149,7 +14149,7 @@
         <v>1143</v>
       </c>
       <c r="C581">
-        <v>0.4449098081558612</v>
+        <v>0.4129505501857075</v>
       </c>
       <c r="D581" t="s">
         <v>1144</v>
@@ -14163,10 +14163,10 @@
         <v>1182</v>
       </c>
       <c r="B582" t="s">
-        <v>1143</v>
+        <v>6</v>
       </c>
       <c r="C582">
-        <v>0.3118414788894101</v>
+        <v>0.3029006331683956</v>
       </c>
       <c r="D582" t="s">
         <v>1144</v>
@@ -14183,7 +14183,7 @@
         <v>6</v>
       </c>
       <c r="C583">
-        <v>0.3676439037715044</v>
+        <v>0.3929266122330919</v>
       </c>
       <c r="D583" t="s">
         <v>1144</v>
@@ -14197,10 +14197,10 @@
         <v>1186</v>
       </c>
       <c r="B584" t="s">
-        <v>1143</v>
+        <v>6</v>
       </c>
       <c r="C584">
-        <v>0.3041133165010727</v>
+        <v>0.2932849087433811</v>
       </c>
       <c r="D584" t="s">
         <v>1144</v>
@@ -14217,7 +14217,7 @@
         <v>1143</v>
       </c>
       <c r="C585">
-        <v>0.3921049488558505</v>
+        <v>0.363708684858251</v>
       </c>
       <c r="D585" t="s">
         <v>1144</v>
@@ -14234,7 +14234,7 @@
         <v>1143</v>
       </c>
       <c r="C586">
-        <v>0.3110312942285105</v>
+        <v>0.2854320270876021</v>
       </c>
       <c r="D586" t="s">
         <v>1144</v>
@@ -14251,7 +14251,7 @@
         <v>6</v>
       </c>
       <c r="C587">
-        <v>0.3292717537634981</v>
+        <v>0.3453653431796098</v>
       </c>
       <c r="D587" t="s">
         <v>1144</v>
@@ -14265,10 +14265,10 @@
         <v>1194</v>
       </c>
       <c r="B588" t="s">
-        <v>1143</v>
+        <v>6</v>
       </c>
       <c r="C588">
-        <v>0.2915438760173306</v>
+        <v>0.2735817841992918</v>
       </c>
       <c r="D588" t="s">
         <v>1144</v>
@@ -14285,7 +14285,7 @@
         <v>45</v>
       </c>
       <c r="C589">
-        <v>0.3456207620168386</v>
+        <v>0.357462837887167</v>
       </c>
       <c r="D589" t="s">
         <v>1144</v>
@@ -14302,7 +14302,7 @@
         <v>6</v>
       </c>
       <c r="C590">
-        <v>0.4030196804948968</v>
+        <v>0.4251514422423212</v>
       </c>
       <c r="D590" t="s">
         <v>1144</v>
@@ -14319,7 +14319,7 @@
         <v>1143</v>
       </c>
       <c r="C591">
-        <v>0.4704354123402085</v>
+        <v>0.4383068928645414</v>
       </c>
       <c r="D591" t="s">
         <v>1144</v>
@@ -14336,7 +14336,7 @@
         <v>1143</v>
       </c>
       <c r="C592">
-        <v>0.3851910777979292</v>
+        <v>0.3542111829477864</v>
       </c>
       <c r="D592" t="s">
         <v>1144</v>
@@ -14353,7 +14353,7 @@
         <v>1143</v>
       </c>
       <c r="C593">
-        <v>0.5418925974074438</v>
+        <v>0.5112859425084417</v>
       </c>
       <c r="D593" t="s">
         <v>1144</v>
@@ -14370,7 +14370,7 @@
         <v>1143</v>
       </c>
       <c r="C594">
-        <v>0.4222690750438409</v>
+        <v>0.3946718449923842</v>
       </c>
       <c r="D594" t="s">
         <v>1144</v>
@@ -14384,10 +14384,10 @@
         <v>1208</v>
       </c>
       <c r="B595" t="s">
-        <v>1143</v>
+        <v>6</v>
       </c>
       <c r="C595">
-        <v>0.3346530825625604</v>
+        <v>0.3497580567706906</v>
       </c>
       <c r="D595" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1143</v>
       </c>
       <c r="C596">
-        <v>0.4327481944721272</v>
+        <v>0.4051188448878583</v>
       </c>
       <c r="D596" t="s">
         <v>1144</v>
@@ -14421,7 +14421,7 @@
         <v>1143</v>
       </c>
       <c r="C597">
-        <v>0.3741442853546899</v>
+        <v>0.3473858265553106</v>
       </c>
       <c r="D597" t="s">
         <v>1144</v>
@@ -14438,7 +14438,7 @@
         <v>10</v>
       </c>
       <c r="C598">
-        <v>0.2849978342499468</v>
+        <v>0.2782432998597438</v>
       </c>
       <c r="D598" t="s">
         <v>1144</v>
@@ -14455,7 +14455,7 @@
         <v>1143</v>
       </c>
       <c r="C599">
-        <v>0.3218449368484785</v>
+        <v>0.2952111168057661</v>
       </c>
       <c r="D599" t="s">
         <v>1144</v>
@@ -14472,7 +14472,7 @@
         <v>1143</v>
       </c>
       <c r="C600">
-        <v>0.3039958818503642</v>
+        <v>0.2776591372914131</v>
       </c>
       <c r="D600" t="s">
         <v>1144</v>
@@ -14489,7 +14489,7 @@
         <v>1143</v>
       </c>
       <c r="C601">
-        <v>0.3155177535017599</v>
+        <v>0.2901105183098396</v>
       </c>
       <c r="D601" t="s">
         <v>1144</v>
@@ -14506,7 +14506,7 @@
         <v>1143</v>
       </c>
       <c r="C602">
-        <v>0.3967551010112958</v>
+        <v>0.3649148793048337</v>
       </c>
       <c r="D602" t="s">
         <v>1144</v>
@@ -14523,7 +14523,7 @@
         <v>1143</v>
       </c>
       <c r="C603">
-        <v>0.3240206318110657</v>
+        <v>0.2968127707577324</v>
       </c>
       <c r="D603" t="s">
         <v>1144</v>
@@ -14540,7 +14540,7 @@
         <v>6</v>
       </c>
       <c r="C604">
-        <v>0.2969274373347594</v>
+        <v>0.3186467881333611</v>
       </c>
       <c r="D604" t="s">
         <v>1144</v>
@@ -14557,7 +14557,7 @@
         <v>45</v>
       </c>
       <c r="C605">
-        <v>0.2957363704839646</v>
+        <v>0.2992967032903776</v>
       </c>
       <c r="D605" t="s">
         <v>1144</v>
@@ -14574,7 +14574,7 @@
         <v>6</v>
       </c>
       <c r="C606">
-        <v>0.3656187619977456</v>
+        <v>0.3875941813405891</v>
       </c>
       <c r="D606" t="s">
         <v>1144</v>
@@ -14588,10 +14588,10 @@
         <v>1232</v>
       </c>
       <c r="B607" t="s">
-        <v>1143</v>
+        <v>10</v>
       </c>
       <c r="C607">
-        <v>0.317704705795591</v>
+        <v>0.3000683811756371</v>
       </c>
       <c r="D607" t="s">
         <v>1144</v>
@@ -14608,7 +14608,7 @@
         <v>1143</v>
       </c>
       <c r="C608">
-        <v>0.3221291059284625</v>
+        <v>0.2937333620891303</v>
       </c>
       <c r="D608" t="s">
         <v>1144</v>
@@ -14625,7 +14625,7 @@
         <v>1143</v>
       </c>
       <c r="C609">
-        <v>0.3294718102079252</v>
+        <v>0.3049127584107788</v>
       </c>
       <c r="D609" t="s">
         <v>1144</v>
@@ -14642,7 +14642,7 @@
         <v>1143</v>
       </c>
       <c r="C610">
-        <v>0.268710503691466</v>
+        <v>0.2443450113787726</v>
       </c>
       <c r="D610" t="s">
         <v>1144</v>
@@ -14659,7 +14659,7 @@
         <v>45</v>
       </c>
       <c r="C611">
-        <v>0.4846106870503183</v>
+        <v>0.4973402187105948</v>
       </c>
       <c r="D611" t="s">
         <v>1144</v>
@@ -14676,7 +14676,7 @@
         <v>45</v>
       </c>
       <c r="C612">
-        <v>0.4297736490016794</v>
+        <v>0.4323010177825921</v>
       </c>
       <c r="D612" t="s">
         <v>1144</v>
@@ -14693,7 +14693,7 @@
         <v>1143</v>
       </c>
       <c r="C613">
-        <v>0.3518523567980054</v>
+        <v>0.3229712387563671</v>
       </c>
       <c r="D613" t="s">
         <v>1144</v>
@@ -14710,7 +14710,7 @@
         <v>1143</v>
       </c>
       <c r="C614">
-        <v>0.3913391249140533</v>
+        <v>0.3636035455794478</v>
       </c>
       <c r="D614" t="s">
         <v>1144</v>
@@ -14727,7 +14727,7 @@
         <v>1143</v>
       </c>
       <c r="C615">
-        <v>0.3579411795091575</v>
+        <v>0.333638255468842</v>
       </c>
       <c r="D615" t="s">
         <v>1144</v>
@@ -14744,7 +14744,7 @@
         <v>1143</v>
       </c>
       <c r="C616">
-        <v>0.3924376116817266</v>
+        <v>0.3643448636617475</v>
       </c>
       <c r="D616" t="s">
         <v>1144</v>
@@ -14761,7 +14761,7 @@
         <v>1143</v>
       </c>
       <c r="C617">
-        <v>0.3580591422994894</v>
+        <v>0.3342648823405743</v>
       </c>
       <c r="D617" t="s">
         <v>1144</v>
@@ -14778,7 +14778,7 @@
         <v>10</v>
       </c>
       <c r="C618">
-        <v>0.3179779610056626</v>
+        <v>0.311023473183448</v>
       </c>
       <c r="D618" t="s">
         <v>1144</v>
@@ -14795,7 +14795,7 @@
         <v>1143</v>
       </c>
       <c r="C619">
-        <v>0.4310891558384365</v>
+        <v>0.403612761275682</v>
       </c>
       <c r="D619" t="s">
         <v>1144</v>
@@ -14812,7 +14812,7 @@
         <v>15</v>
       </c>
       <c r="C620">
-        <v>0.2890539426284621</v>
+        <v>0.2891314228241091</v>
       </c>
       <c r="D620" t="s">
         <v>1259</v>
@@ -14829,7 +14829,7 @@
         <v>15</v>
       </c>
       <c r="C621">
-        <v>0.3264652590983719</v>
+        <v>0.3268663846519788</v>
       </c>
       <c r="D621" t="s">
         <v>1259</v>
@@ -14846,7 +14846,7 @@
         <v>15</v>
       </c>
       <c r="C622">
-        <v>0.2274980912335571</v>
+        <v>0.2275404253202313</v>
       </c>
       <c r="D622" t="s">
         <v>1259</v>
@@ -14863,7 +14863,7 @@
         <v>1266</v>
       </c>
       <c r="C623">
-        <v>0.2429884473956745</v>
+        <v>0.2392847862985188</v>
       </c>
       <c r="D623" t="s">
         <v>1259</v>
@@ -14880,7 +14880,7 @@
         <v>10</v>
       </c>
       <c r="C624">
-        <v>0.2690408351901146</v>
+        <v>0.2722995902607807</v>
       </c>
       <c r="D624" t="s">
         <v>1259</v>
@@ -14894,10 +14894,10 @@
         <v>1270</v>
       </c>
       <c r="B625" t="s">
-        <v>1266</v>
+        <v>10</v>
       </c>
       <c r="C625">
-        <v>0.2504897389124233</v>
+        <v>0.2521530024585635</v>
       </c>
       <c r="D625" t="s">
         <v>1259</v>
@@ -14914,7 +14914,7 @@
         <v>15</v>
       </c>
       <c r="C626">
-        <v>0.3024316527710464</v>
+        <v>0.3027961559975631</v>
       </c>
       <c r="D626" t="s">
         <v>1259</v>
@@ -14931,7 +14931,7 @@
         <v>1266</v>
       </c>
       <c r="C627">
-        <v>0.3259183667833081</v>
+        <v>0.3217575982867497</v>
       </c>
       <c r="D627" t="s">
         <v>1259</v>
@@ -14948,7 +14948,7 @@
         <v>1266</v>
       </c>
       <c r="C628">
-        <v>0.2870318579605975</v>
+        <v>0.2830052487288737</v>
       </c>
       <c r="D628" t="s">
         <v>1259</v>
@@ -14965,7 +14965,7 @@
         <v>1266</v>
       </c>
       <c r="C629">
-        <v>0.2223251664995292</v>
+        <v>0.2188305089201392</v>
       </c>
       <c r="D629" t="s">
         <v>1259</v>
@@ -14982,7 +14982,7 @@
         <v>1266</v>
       </c>
       <c r="C630">
-        <v>0.3930299238157548</v>
+        <v>0.3895353849245772</v>
       </c>
       <c r="D630" t="s">
         <v>1259</v>
@@ -14999,7 +14999,7 @@
         <v>1266</v>
       </c>
       <c r="C631">
-        <v>0.4040703574019626</v>
+        <v>0.3997078850171333</v>
       </c>
       <c r="D631" t="s">
         <v>1259</v>
@@ -15016,7 +15016,7 @@
         <v>1266</v>
       </c>
       <c r="C632">
-        <v>0.4557776174784538</v>
+        <v>0.4518529565287717</v>
       </c>
       <c r="D632" t="s">
         <v>1259</v>
@@ -15033,7 +15033,7 @@
         <v>15</v>
       </c>
       <c r="C633">
-        <v>0.265804185567516</v>
+        <v>0.2662182419519051</v>
       </c>
       <c r="D633" t="s">
         <v>1259</v>
@@ -15050,7 +15050,7 @@
         <v>15</v>
       </c>
       <c r="C634">
-        <v>0.3325964414456429</v>
+        <v>0.3330863011539898</v>
       </c>
       <c r="D634" t="s">
         <v>1259</v>
@@ -15067,7 +15067,7 @@
         <v>1266</v>
       </c>
       <c r="C635">
-        <v>0.4695927819330701</v>
+        <v>0.4650725858900553</v>
       </c>
       <c r="D635" t="s">
         <v>1259</v>
@@ -15084,7 +15084,7 @@
         <v>6</v>
       </c>
       <c r="C636">
-        <v>0.3618594904497027</v>
+        <v>0.3621577104358017</v>
       </c>
       <c r="D636" t="s">
         <v>1259</v>
@@ -15101,7 +15101,7 @@
         <v>1266</v>
       </c>
       <c r="C637">
-        <v>0.3234625111819353</v>
+        <v>0.3193161758528884</v>
       </c>
       <c r="D637" t="s">
         <v>1259</v>
@@ -15118,7 +15118,7 @@
         <v>1266</v>
       </c>
       <c r="C638">
-        <v>0.4903627901137151</v>
+        <v>0.487291006358283</v>
       </c>
       <c r="D638" t="s">
         <v>1259</v>
@@ -15135,7 +15135,7 @@
         <v>10</v>
       </c>
       <c r="C639">
-        <v>0.3080109935756575</v>
+        <v>0.3113728459237843</v>
       </c>
       <c r="D639" t="s">
         <v>1259</v>
@@ -15152,7 +15152,7 @@
         <v>10</v>
       </c>
       <c r="C640">
-        <v>0.2600392705901694</v>
+        <v>0.263217694231395</v>
       </c>
       <c r="D640" t="s">
         <v>1259</v>
@@ -15169,7 +15169,7 @@
         <v>1266</v>
       </c>
       <c r="C641">
-        <v>0.2878169316923523</v>
+        <v>0.2837883937185025</v>
       </c>
       <c r="D641" t="s">
         <v>1259</v>
@@ -15186,7 +15186,7 @@
         <v>1266</v>
       </c>
       <c r="C642">
-        <v>0.3355545985743619</v>
+        <v>0.3311501451174218</v>
       </c>
       <c r="D642" t="s">
         <v>1259</v>
@@ -15203,7 +15203,7 @@
         <v>15</v>
       </c>
       <c r="C643">
-        <v>0.3026071747601911</v>
+        <v>0.302798518075402</v>
       </c>
       <c r="D643" t="s">
         <v>1259</v>
@@ -15220,7 +15220,7 @@
         <v>15</v>
       </c>
       <c r="C644">
-        <v>0.2912869579012972</v>
+        <v>0.2919865086088561</v>
       </c>
       <c r="D644" t="s">
         <v>1259</v>
@@ -15237,7 +15237,7 @@
         <v>1266</v>
       </c>
       <c r="C645">
-        <v>0.2499418303546379</v>
+        <v>0.2458327937744067</v>
       </c>
       <c r="D645" t="s">
         <v>1259</v>
@@ -15254,7 +15254,7 @@
         <v>15</v>
       </c>
       <c r="C646">
-        <v>0.3302226417810288</v>
+        <v>0.3305884568402281</v>
       </c>
       <c r="D646" t="s">
         <v>1259</v>
@@ -15271,7 +15271,7 @@
         <v>1266</v>
       </c>
       <c r="C647">
-        <v>0.3296166688505361</v>
+        <v>0.3255603298081895</v>
       </c>
       <c r="D647" t="s">
         <v>1259</v>
@@ -15288,7 +15288,7 @@
         <v>15</v>
       </c>
       <c r="C648">
-        <v>0.2697526705414868</v>
+        <v>0.2702503401802666</v>
       </c>
       <c r="D648" t="s">
         <v>1259</v>
@@ -15305,7 +15305,7 @@
         <v>15</v>
       </c>
       <c r="C649">
-        <v>0.2930271360542232</v>
+        <v>0.2934592544460942</v>
       </c>
       <c r="D649" t="s">
         <v>1259</v>
@@ -15322,7 +15322,7 @@
         <v>1266</v>
       </c>
       <c r="C650">
-        <v>0.2818298737363125</v>
+        <v>0.2780759251476082</v>
       </c>
       <c r="D650" t="s">
         <v>1259</v>
@@ -15339,7 +15339,7 @@
         <v>15</v>
       </c>
       <c r="C651">
-        <v>0.301028925047235</v>
+        <v>0.3014870811565031</v>
       </c>
       <c r="D651" t="s">
         <v>1259</v>
@@ -15379,7 +15379,7 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -15395,7 +15395,7 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -15419,7 +15419,7 @@
         <v>1266</v>
       </c>
       <c r="B8">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -15427,7 +15427,7 @@
         <v>1143</v>
       </c>
       <c r="B9">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:2">

</xml_diff>

<commit_message>
forgot to write to excel file again
</commit_message>
<xml_diff>
--- a/frontend/data/uk_election_predictions.xlsx
+++ b/frontend/data/uk_election_predictions.xlsx
@@ -13843,7 +13843,7 @@
         <v>1143</v>
       </c>
       <c r="C563">
-        <v>0.2778510537375036</v>
+        <v>0.2754534067785577</v>
       </c>
       <c r="D563" t="s">
         <v>1144</v>
@@ -13860,7 +13860,7 @@
         <v>1143</v>
       </c>
       <c r="C564">
-        <v>0.3278804824240203</v>
+        <v>0.3217552589307947</v>
       </c>
       <c r="D564" t="s">
         <v>1144</v>
@@ -13877,7 +13877,7 @@
         <v>1143</v>
       </c>
       <c r="C565">
-        <v>0.2751971003895707</v>
+        <v>0.2712719546541894</v>
       </c>
       <c r="D565" t="s">
         <v>1144</v>
@@ -13894,7 +13894,7 @@
         <v>1143</v>
       </c>
       <c r="C566">
-        <v>0.4574381408777259</v>
+        <v>0.4599578364420591</v>
       </c>
       <c r="D566" t="s">
         <v>1144</v>
@@ -13911,7 +13911,7 @@
         <v>1143</v>
       </c>
       <c r="C567">
-        <v>0.3954275260752005</v>
+        <v>0.4095146333369669</v>
       </c>
       <c r="D567" t="s">
         <v>1144</v>
@@ -13928,7 +13928,7 @@
         <v>1143</v>
       </c>
       <c r="C568">
-        <v>0.3429164531248907</v>
+        <v>0.3468779710443464</v>
       </c>
       <c r="D568" t="s">
         <v>1144</v>
@@ -13945,7 +13945,7 @@
         <v>1143</v>
       </c>
       <c r="C569">
-        <v>0.2807094492642338</v>
+        <v>0.2819164947080606</v>
       </c>
       <c r="D569" t="s">
         <v>1144</v>
@@ -13962,7 +13962,7 @@
         <v>10</v>
       </c>
       <c r="C570">
-        <v>0.2961480648555327</v>
+        <v>0.2922538829959456</v>
       </c>
       <c r="D570" t="s">
         <v>1144</v>
@@ -13979,7 +13979,7 @@
         <v>1143</v>
       </c>
       <c r="C571">
-        <v>0.2767573836990959</v>
+        <v>0.2799547040370936</v>
       </c>
       <c r="D571" t="s">
         <v>1144</v>
@@ -13996,7 +13996,7 @@
         <v>1143</v>
       </c>
       <c r="C572">
-        <v>0.3324425591822937</v>
+        <v>0.3300073093208997</v>
       </c>
       <c r="D572" t="s">
         <v>1144</v>
@@ -14013,7 +14013,7 @@
         <v>1143</v>
       </c>
       <c r="C573">
-        <v>0.2811055033079313</v>
+        <v>0.2805324853412571</v>
       </c>
       <c r="D573" t="s">
         <v>1144</v>
@@ -14030,7 +14030,7 @@
         <v>45</v>
       </c>
       <c r="C574">
-        <v>0.335414871319458</v>
+        <v>0.3687604786717376</v>
       </c>
       <c r="D574" t="s">
         <v>1144</v>
@@ -14047,7 +14047,7 @@
         <v>1143</v>
       </c>
       <c r="C575">
-        <v>0.3071793543488098</v>
+        <v>0.3015709519450364</v>
       </c>
       <c r="D575" t="s">
         <v>1144</v>
@@ -14064,7 +14064,7 @@
         <v>1143</v>
       </c>
       <c r="C576">
-        <v>0.3604746859907967</v>
+        <v>0.3674308555554007</v>
       </c>
       <c r="D576" t="s">
         <v>1144</v>
@@ -14081,7 +14081,7 @@
         <v>6</v>
       </c>
       <c r="C577">
-        <v>0.3033545451788696</v>
+        <v>0.2966752447379611</v>
       </c>
       <c r="D577" t="s">
         <v>1144</v>
@@ -14098,7 +14098,7 @@
         <v>1143</v>
       </c>
       <c r="C578">
-        <v>0.3596182830515524</v>
+        <v>0.3631428679854594</v>
       </c>
       <c r="D578" t="s">
         <v>1144</v>
@@ -14115,7 +14115,7 @@
         <v>1143</v>
       </c>
       <c r="C579">
-        <v>0.3015362942315583</v>
+        <v>0.3054834405529114</v>
       </c>
       <c r="D579" t="s">
         <v>1144</v>
@@ -14132,7 +14132,7 @@
         <v>10</v>
       </c>
       <c r="C580">
-        <v>0.3692136422589501</v>
+        <v>0.357103663493369</v>
       </c>
       <c r="D580" t="s">
         <v>1144</v>
@@ -14149,7 +14149,7 @@
         <v>1143</v>
       </c>
       <c r="C581">
-        <v>0.4129505501857075</v>
+        <v>0.4010937252652034</v>
       </c>
       <c r="D581" t="s">
         <v>1144</v>
@@ -14166,7 +14166,7 @@
         <v>6</v>
       </c>
       <c r="C582">
-        <v>0.3029006331683956</v>
+        <v>0.296311647312829</v>
       </c>
       <c r="D582" t="s">
         <v>1144</v>
@@ -14183,7 +14183,7 @@
         <v>6</v>
       </c>
       <c r="C583">
-        <v>0.3929266122330919</v>
+        <v>0.3877448800199075</v>
       </c>
       <c r="D583" t="s">
         <v>1144</v>
@@ -14197,10 +14197,10 @@
         <v>1186</v>
       </c>
       <c r="B584" t="s">
-        <v>6</v>
+        <v>1143</v>
       </c>
       <c r="C584">
-        <v>0.2932849087433811</v>
+        <v>0.2887079332281093</v>
       </c>
       <c r="D584" t="s">
         <v>1144</v>
@@ -14217,7 +14217,7 @@
         <v>1143</v>
       </c>
       <c r="C585">
-        <v>0.363708684858251</v>
+        <v>0.3693780743037599</v>
       </c>
       <c r="D585" t="s">
         <v>1144</v>
@@ -14234,7 +14234,7 @@
         <v>1143</v>
       </c>
       <c r="C586">
-        <v>0.2854320270876021</v>
+        <v>0.2801336688646776</v>
       </c>
       <c r="D586" t="s">
         <v>1144</v>
@@ -14251,7 +14251,7 @@
         <v>6</v>
       </c>
       <c r="C587">
-        <v>0.3453653431796098</v>
+        <v>0.3287710800260244</v>
       </c>
       <c r="D587" t="s">
         <v>1144</v>
@@ -14265,10 +14265,10 @@
         <v>1194</v>
       </c>
       <c r="B588" t="s">
-        <v>6</v>
+        <v>1143</v>
       </c>
       <c r="C588">
-        <v>0.2735817841992918</v>
+        <v>0.2681818349557712</v>
       </c>
       <c r="D588" t="s">
         <v>1144</v>
@@ -14285,7 +14285,7 @@
         <v>45</v>
       </c>
       <c r="C589">
-        <v>0.357462837887167</v>
+        <v>0.3916150747493796</v>
       </c>
       <c r="D589" t="s">
         <v>1144</v>
@@ -14302,7 +14302,7 @@
         <v>6</v>
       </c>
       <c r="C590">
-        <v>0.4251514422423212</v>
+        <v>0.410420021121837</v>
       </c>
       <c r="D590" t="s">
         <v>1144</v>
@@ -14319,7 +14319,7 @@
         <v>1143</v>
       </c>
       <c r="C591">
-        <v>0.4383068928645414</v>
+        <v>0.4219222946389186</v>
       </c>
       <c r="D591" t="s">
         <v>1144</v>
@@ -14336,7 +14336,7 @@
         <v>1143</v>
       </c>
       <c r="C592">
-        <v>0.3542111829477864</v>
+        <v>0.3270613617209647</v>
       </c>
       <c r="D592" t="s">
         <v>1144</v>
@@ -14353,7 +14353,7 @@
         <v>1143</v>
       </c>
       <c r="C593">
-        <v>0.5112859425084417</v>
+        <v>0.5173383757395047</v>
       </c>
       <c r="D593" t="s">
         <v>1144</v>
@@ -14370,7 +14370,7 @@
         <v>1143</v>
       </c>
       <c r="C594">
-        <v>0.3946718449923842</v>
+        <v>0.3887938758872745</v>
       </c>
       <c r="D594" t="s">
         <v>1144</v>
@@ -14387,7 +14387,7 @@
         <v>6</v>
       </c>
       <c r="C595">
-        <v>0.3497580567706906</v>
+        <v>0.337543487651305</v>
       </c>
       <c r="D595" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1143</v>
       </c>
       <c r="C596">
-        <v>0.4051188448878583</v>
+        <v>0.3936227625512888</v>
       </c>
       <c r="D596" t="s">
         <v>1144</v>
@@ -14421,7 +14421,7 @@
         <v>1143</v>
       </c>
       <c r="C597">
-        <v>0.3473858265553106</v>
+        <v>0.3632435099993138</v>
       </c>
       <c r="D597" t="s">
         <v>1144</v>
@@ -14438,7 +14438,7 @@
         <v>10</v>
       </c>
       <c r="C598">
-        <v>0.2782432998597438</v>
+        <v>0.266914164262071</v>
       </c>
       <c r="D598" t="s">
         <v>1144</v>
@@ -14455,7 +14455,7 @@
         <v>1143</v>
       </c>
       <c r="C599">
-        <v>0.2952111168057661</v>
+        <v>0.3042814912995248</v>
       </c>
       <c r="D599" t="s">
         <v>1144</v>
@@ -14472,7 +14472,7 @@
         <v>1143</v>
       </c>
       <c r="C600">
-        <v>0.2776591372914131</v>
+        <v>0.2781088630637019</v>
       </c>
       <c r="D600" t="s">
         <v>1144</v>
@@ -14486,10 +14486,10 @@
         <v>1220</v>
       </c>
       <c r="B601" t="s">
-        <v>1143</v>
+        <v>45</v>
       </c>
       <c r="C601">
-        <v>0.2901105183098396</v>
+        <v>0.2916491957457273</v>
       </c>
       <c r="D601" t="s">
         <v>1144</v>
@@ -14506,7 +14506,7 @@
         <v>1143</v>
       </c>
       <c r="C602">
-        <v>0.3649148793048337</v>
+        <v>0.36987647682363</v>
       </c>
       <c r="D602" t="s">
         <v>1144</v>
@@ -14523,7 +14523,7 @@
         <v>1143</v>
       </c>
       <c r="C603">
-        <v>0.2968127707577324</v>
+        <v>0.298544854354126</v>
       </c>
       <c r="D603" t="s">
         <v>1144</v>
@@ -14540,7 +14540,7 @@
         <v>6</v>
       </c>
       <c r="C604">
-        <v>0.3186467881333611</v>
+        <v>0.3132720927243448</v>
       </c>
       <c r="D604" t="s">
         <v>1144</v>
@@ -14557,7 +14557,7 @@
         <v>45</v>
       </c>
       <c r="C605">
-        <v>0.2992967032903776</v>
+        <v>0.3288100647079791</v>
       </c>
       <c r="D605" t="s">
         <v>1144</v>
@@ -14574,7 +14574,7 @@
         <v>6</v>
       </c>
       <c r="C606">
-        <v>0.3875941813405891</v>
+        <v>0.3756896859321552</v>
       </c>
       <c r="D606" t="s">
         <v>1144</v>
@@ -14591,7 +14591,7 @@
         <v>10</v>
       </c>
       <c r="C607">
-        <v>0.3000683811756371</v>
+        <v>0.2873044081796143</v>
       </c>
       <c r="D607" t="s">
         <v>1144</v>
@@ -14608,7 +14608,7 @@
         <v>1143</v>
       </c>
       <c r="C608">
-        <v>0.2937333620891303</v>
+        <v>0.2954830322571341</v>
       </c>
       <c r="D608" t="s">
         <v>1144</v>
@@ -14625,7 +14625,7 @@
         <v>1143</v>
       </c>
       <c r="C609">
-        <v>0.3049127584107788</v>
+        <v>0.3012841560274029</v>
       </c>
       <c r="D609" t="s">
         <v>1144</v>
@@ -14642,7 +14642,7 @@
         <v>1143</v>
       </c>
       <c r="C610">
-        <v>0.2443450113787726</v>
+        <v>0.2499979097946463</v>
       </c>
       <c r="D610" t="s">
         <v>1144</v>
@@ -14659,7 +14659,7 @@
         <v>45</v>
       </c>
       <c r="C611">
-        <v>0.4973402187105948</v>
+        <v>0.5301410827809822</v>
       </c>
       <c r="D611" t="s">
         <v>1144</v>
@@ -14676,7 +14676,7 @@
         <v>45</v>
       </c>
       <c r="C612">
-        <v>0.4323010177825921</v>
+        <v>0.4702653401107232</v>
       </c>
       <c r="D612" t="s">
         <v>1144</v>
@@ -14693,7 +14693,7 @@
         <v>1143</v>
       </c>
       <c r="C613">
-        <v>0.3229712387563671</v>
+        <v>0.3263467065741318</v>
       </c>
       <c r="D613" t="s">
         <v>1144</v>
@@ -14710,7 +14710,7 @@
         <v>1143</v>
       </c>
       <c r="C614">
-        <v>0.3636035455794478</v>
+        <v>0.3780567462472258</v>
       </c>
       <c r="D614" t="s">
         <v>1144</v>
@@ -14727,7 +14727,7 @@
         <v>1143</v>
       </c>
       <c r="C615">
-        <v>0.333638255468842</v>
+        <v>0.3337172300066883</v>
       </c>
       <c r="D615" t="s">
         <v>1144</v>
@@ -14744,7 +14744,7 @@
         <v>1143</v>
       </c>
       <c r="C616">
-        <v>0.3643448636617475</v>
+        <v>0.3762573196510252</v>
       </c>
       <c r="D616" t="s">
         <v>1144</v>
@@ -14761,7 +14761,7 @@
         <v>1143</v>
       </c>
       <c r="C617">
-        <v>0.3342648823405743</v>
+        <v>0.3446620184954829</v>
       </c>
       <c r="D617" t="s">
         <v>1144</v>
@@ -14778,7 +14778,7 @@
         <v>10</v>
       </c>
       <c r="C618">
-        <v>0.311023473183448</v>
+        <v>0.2983525383218857</v>
       </c>
       <c r="D618" t="s">
         <v>1144</v>
@@ -14795,7 +14795,7 @@
         <v>1143</v>
       </c>
       <c r="C619">
-        <v>0.403612761275682</v>
+        <v>0.4187231771809876</v>
       </c>
       <c r="D619" t="s">
         <v>1144</v>
@@ -15395,7 +15395,7 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -15403,7 +15403,7 @@
         <v>45</v>
       </c>
       <c r="B6">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -15427,7 +15427,7 @@
         <v>1143</v>
       </c>
       <c r="B9">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:2">

</xml_diff>

<commit_message>
added incumbency to Scotland
</commit_message>
<xml_diff>
--- a/frontend/data/uk_election_predictions.xlsx
+++ b/frontend/data/uk_election_predictions.xlsx
@@ -13843,7 +13843,7 @@
         <v>1143</v>
       </c>
       <c r="C563">
-        <v>0.2754534067785577</v>
+        <v>0.2690105680143081</v>
       </c>
       <c r="D563" t="s">
         <v>1144</v>
@@ -13860,7 +13860,7 @@
         <v>1143</v>
       </c>
       <c r="C564">
-        <v>0.3217552589307947</v>
+        <v>0.3177251028942784</v>
       </c>
       <c r="D564" t="s">
         <v>1144</v>
@@ -13877,7 +13877,7 @@
         <v>1143</v>
       </c>
       <c r="C565">
-        <v>0.2712719546541894</v>
+        <v>0.2612073347443773</v>
       </c>
       <c r="D565" t="s">
         <v>1144</v>
@@ -13894,7 +13894,7 @@
         <v>1143</v>
       </c>
       <c r="C566">
-        <v>0.4599578364420591</v>
+        <v>0.4692636361466231</v>
       </c>
       <c r="D566" t="s">
         <v>1144</v>
@@ -13911,7 +13911,7 @@
         <v>1143</v>
       </c>
       <c r="C567">
-        <v>0.4095146333369669</v>
+        <v>0.4067040151987543</v>
       </c>
       <c r="D567" t="s">
         <v>1144</v>
@@ -13928,7 +13928,7 @@
         <v>1143</v>
       </c>
       <c r="C568">
-        <v>0.3468779710443464</v>
+        <v>0.3265702287762656</v>
       </c>
       <c r="D568" t="s">
         <v>1144</v>
@@ -13945,7 +13945,7 @@
         <v>1143</v>
       </c>
       <c r="C569">
-        <v>0.2819164947080606</v>
+        <v>0.2725871796309934</v>
       </c>
       <c r="D569" t="s">
         <v>1144</v>
@@ -13962,7 +13962,7 @@
         <v>10</v>
       </c>
       <c r="C570">
-        <v>0.2922538829959456</v>
+        <v>0.2973980033569115</v>
       </c>
       <c r="D570" t="s">
         <v>1144</v>
@@ -13979,7 +13979,7 @@
         <v>1143</v>
       </c>
       <c r="C571">
-        <v>0.2799547040370936</v>
+        <v>0.2785945084718467</v>
       </c>
       <c r="D571" t="s">
         <v>1144</v>
@@ -13996,7 +13996,7 @@
         <v>1143</v>
       </c>
       <c r="C572">
-        <v>0.3300073093208997</v>
+        <v>0.3339394241823059</v>
       </c>
       <c r="D572" t="s">
         <v>1144</v>
@@ -14013,7 +14013,7 @@
         <v>1143</v>
       </c>
       <c r="C573">
-        <v>0.2805324853412571</v>
+        <v>0.2742210821650125</v>
       </c>
       <c r="D573" t="s">
         <v>1144</v>
@@ -14030,7 +14030,7 @@
         <v>45</v>
       </c>
       <c r="C574">
-        <v>0.3687604786717376</v>
+        <v>0.3028456434777809</v>
       </c>
       <c r="D574" t="s">
         <v>1144</v>
@@ -14047,7 +14047,7 @@
         <v>1143</v>
       </c>
       <c r="C575">
-        <v>0.3015709519450364</v>
+        <v>0.3119341197899996</v>
       </c>
       <c r="D575" t="s">
         <v>1144</v>
@@ -14064,7 +14064,7 @@
         <v>1143</v>
       </c>
       <c r="C576">
-        <v>0.3674308555554007</v>
+        <v>0.3698231117449726</v>
       </c>
       <c r="D576" t="s">
         <v>1144</v>
@@ -14081,7 +14081,7 @@
         <v>6</v>
       </c>
       <c r="C577">
-        <v>0.2966752447379611</v>
+        <v>0.2919594411842059</v>
       </c>
       <c r="D577" t="s">
         <v>1144</v>
@@ -14098,7 +14098,7 @@
         <v>1143</v>
       </c>
       <c r="C578">
-        <v>0.3631428679854594</v>
+        <v>0.3539930473586655</v>
       </c>
       <c r="D578" t="s">
         <v>1144</v>
@@ -14115,7 +14115,7 @@
         <v>1143</v>
       </c>
       <c r="C579">
-        <v>0.3054834405529114</v>
+        <v>0.2940333724000349</v>
       </c>
       <c r="D579" t="s">
         <v>1144</v>
@@ -14132,7 +14132,7 @@
         <v>10</v>
       </c>
       <c r="C580">
-        <v>0.357103663493369</v>
+        <v>0.3509493963487059</v>
       </c>
       <c r="D580" t="s">
         <v>1144</v>
@@ -14149,7 +14149,7 @@
         <v>1143</v>
       </c>
       <c r="C581">
-        <v>0.4010937252652034</v>
+        <v>0.4147576516194132</v>
       </c>
       <c r="D581" t="s">
         <v>1144</v>
@@ -14163,10 +14163,10 @@
         <v>1182</v>
       </c>
       <c r="B582" t="s">
-        <v>6</v>
+        <v>1143</v>
       </c>
       <c r="C582">
-        <v>0.296311647312829</v>
+        <v>0.2893096138868425</v>
       </c>
       <c r="D582" t="s">
         <v>1144</v>
@@ -14183,7 +14183,7 @@
         <v>6</v>
       </c>
       <c r="C583">
-        <v>0.3877448800199075</v>
+        <v>0.377930850660432</v>
       </c>
       <c r="D583" t="s">
         <v>1144</v>
@@ -14197,10 +14197,10 @@
         <v>1186</v>
       </c>
       <c r="B584" t="s">
-        <v>1143</v>
+        <v>6</v>
       </c>
       <c r="C584">
-        <v>0.2887079332281093</v>
+        <v>0.2909773104359007</v>
       </c>
       <c r="D584" t="s">
         <v>1144</v>
@@ -14217,7 +14217,7 @@
         <v>1143</v>
       </c>
       <c r="C585">
-        <v>0.3693780743037599</v>
+        <v>0.3590663072187273</v>
       </c>
       <c r="D585" t="s">
         <v>1144</v>
@@ -14234,7 +14234,7 @@
         <v>1143</v>
       </c>
       <c r="C586">
-        <v>0.2801336688646776</v>
+        <v>0.2805660414157179</v>
       </c>
       <c r="D586" t="s">
         <v>1144</v>
@@ -14251,7 +14251,7 @@
         <v>6</v>
       </c>
       <c r="C587">
-        <v>0.3287710800260244</v>
+        <v>0.3109198236844402</v>
       </c>
       <c r="D587" t="s">
         <v>1144</v>
@@ -14268,7 +14268,7 @@
         <v>1143</v>
       </c>
       <c r="C588">
-        <v>0.2681818349557712</v>
+        <v>0.2658543187802467</v>
       </c>
       <c r="D588" t="s">
         <v>1144</v>
@@ -14285,7 +14285,7 @@
         <v>45</v>
       </c>
       <c r="C589">
-        <v>0.3916150747493796</v>
+        <v>0.334880147352805</v>
       </c>
       <c r="D589" t="s">
         <v>1144</v>
@@ -14302,7 +14302,7 @@
         <v>6</v>
       </c>
       <c r="C590">
-        <v>0.410420021121837</v>
+        <v>0.4162449782215457</v>
       </c>
       <c r="D590" t="s">
         <v>1144</v>
@@ -14319,7 +14319,7 @@
         <v>1143</v>
       </c>
       <c r="C591">
-        <v>0.4219222946389186</v>
+        <v>0.4498428338083647</v>
       </c>
       <c r="D591" t="s">
         <v>1144</v>
@@ -14336,7 +14336,7 @@
         <v>1143</v>
       </c>
       <c r="C592">
-        <v>0.3270613617209647</v>
+        <v>0.3616150735580669</v>
       </c>
       <c r="D592" t="s">
         <v>1144</v>
@@ -14353,7 +14353,7 @@
         <v>1143</v>
       </c>
       <c r="C593">
-        <v>0.5173383757395047</v>
+        <v>0.5284429984532093</v>
       </c>
       <c r="D593" t="s">
         <v>1144</v>
@@ -14370,7 +14370,7 @@
         <v>1143</v>
       </c>
       <c r="C594">
-        <v>0.3887938758872745</v>
+        <v>0.4029520642890408</v>
       </c>
       <c r="D594" t="s">
         <v>1144</v>
@@ -14387,7 +14387,7 @@
         <v>6</v>
       </c>
       <c r="C595">
-        <v>0.337543487651305</v>
+        <v>0.3381832858024464</v>
       </c>
       <c r="D595" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1143</v>
       </c>
       <c r="C596">
-        <v>0.3936227625512888</v>
+        <v>0.4199716629659814</v>
       </c>
       <c r="D596" t="s">
         <v>1144</v>
@@ -14421,7 +14421,7 @@
         <v>1143</v>
       </c>
       <c r="C597">
-        <v>0.3632435099993138</v>
+        <v>0.3512890035148448</v>
       </c>
       <c r="D597" t="s">
         <v>1144</v>
@@ -14438,7 +14438,7 @@
         <v>10</v>
       </c>
       <c r="C598">
-        <v>0.266914164262071</v>
+        <v>0.2581521998596382</v>
       </c>
       <c r="D598" t="s">
         <v>1144</v>
@@ -14455,7 +14455,7 @@
         <v>1143</v>
       </c>
       <c r="C599">
-        <v>0.3042814912995248</v>
+        <v>0.3027521919912147</v>
       </c>
       <c r="D599" t="s">
         <v>1144</v>
@@ -14472,7 +14472,7 @@
         <v>1143</v>
       </c>
       <c r="C600">
-        <v>0.2781088630637019</v>
+        <v>0.2791350443565828</v>
       </c>
       <c r="D600" t="s">
         <v>1144</v>
@@ -14486,10 +14486,10 @@
         <v>1220</v>
       </c>
       <c r="B601" t="s">
-        <v>45</v>
+        <v>1143</v>
       </c>
       <c r="C601">
-        <v>0.2916491957457273</v>
+        <v>0.2807495838551311</v>
       </c>
       <c r="D601" t="s">
         <v>1144</v>
@@ -14506,7 +14506,7 @@
         <v>1143</v>
       </c>
       <c r="C602">
-        <v>0.36987647682363</v>
+        <v>0.3673640637629877</v>
       </c>
       <c r="D602" t="s">
         <v>1144</v>
@@ -14523,7 +14523,7 @@
         <v>1143</v>
       </c>
       <c r="C603">
-        <v>0.298544854354126</v>
+        <v>0.2923137433218961</v>
       </c>
       <c r="D603" t="s">
         <v>1144</v>
@@ -14540,7 +14540,7 @@
         <v>6</v>
       </c>
       <c r="C604">
-        <v>0.3132720927243448</v>
+        <v>0.3036732982785109</v>
       </c>
       <c r="D604" t="s">
         <v>1144</v>
@@ -14557,7 +14557,7 @@
         <v>45</v>
       </c>
       <c r="C605">
-        <v>0.3288100647079791</v>
+        <v>0.280490914003508</v>
       </c>
       <c r="D605" t="s">
         <v>1144</v>
@@ -14574,7 +14574,7 @@
         <v>6</v>
       </c>
       <c r="C606">
-        <v>0.3756896859321552</v>
+        <v>0.3717057904590055</v>
       </c>
       <c r="D606" t="s">
         <v>1144</v>
@@ -14588,10 +14588,10 @@
         <v>1232</v>
       </c>
       <c r="B607" t="s">
-        <v>10</v>
+        <v>1143</v>
       </c>
       <c r="C607">
-        <v>0.2873044081796143</v>
+        <v>0.2846142319580898</v>
       </c>
       <c r="D607" t="s">
         <v>1144</v>
@@ -14608,7 +14608,7 @@
         <v>1143</v>
       </c>
       <c r="C608">
-        <v>0.2954830322571341</v>
+        <v>0.2988339006103424</v>
       </c>
       <c r="D608" t="s">
         <v>1144</v>
@@ -14625,7 +14625,7 @@
         <v>1143</v>
       </c>
       <c r="C609">
-        <v>0.3012841560274029</v>
+        <v>0.3152593720728452</v>
       </c>
       <c r="D609" t="s">
         <v>1144</v>
@@ -14642,7 +14642,7 @@
         <v>1143</v>
       </c>
       <c r="C610">
-        <v>0.2499979097946463</v>
+        <v>0.2442559023413335</v>
       </c>
       <c r="D610" t="s">
         <v>1144</v>
@@ -14659,7 +14659,7 @@
         <v>45</v>
       </c>
       <c r="C611">
-        <v>0.5301410827809822</v>
+        <v>0.4649064157757105</v>
       </c>
       <c r="D611" t="s">
         <v>1144</v>
@@ -14676,7 +14676,7 @@
         <v>45</v>
       </c>
       <c r="C612">
-        <v>0.4702653401107232</v>
+        <v>0.3840648677724066</v>
       </c>
       <c r="D612" t="s">
         <v>1144</v>
@@ -14693,7 +14693,7 @@
         <v>1143</v>
       </c>
       <c r="C613">
-        <v>0.3263467065741318</v>
+        <v>0.3265343579132391</v>
       </c>
       <c r="D613" t="s">
         <v>1144</v>
@@ -14710,7 +14710,7 @@
         <v>1143</v>
       </c>
       <c r="C614">
-        <v>0.3780567462472258</v>
+        <v>0.3710125022602774</v>
       </c>
       <c r="D614" t="s">
         <v>1144</v>
@@ -14727,7 +14727,7 @@
         <v>1143</v>
       </c>
       <c r="C615">
-        <v>0.3337172300066883</v>
+        <v>0.31410023344431</v>
       </c>
       <c r="D615" t="s">
         <v>1144</v>
@@ -14744,7 +14744,7 @@
         <v>1143</v>
       </c>
       <c r="C616">
-        <v>0.3762573196510252</v>
+        <v>0.3696786189294876</v>
       </c>
       <c r="D616" t="s">
         <v>1144</v>
@@ -14761,7 +14761,7 @@
         <v>1143</v>
       </c>
       <c r="C617">
-        <v>0.3446620184954829</v>
+        <v>0.3260999878488807</v>
       </c>
       <c r="D617" t="s">
         <v>1144</v>
@@ -14778,7 +14778,7 @@
         <v>10</v>
       </c>
       <c r="C618">
-        <v>0.2983525383218857</v>
+        <v>0.2893262440264847</v>
       </c>
       <c r="D618" t="s">
         <v>1144</v>
@@ -14795,7 +14795,7 @@
         <v>1143</v>
       </c>
       <c r="C619">
-        <v>0.4187231771809876</v>
+        <v>0.4169620502023828</v>
       </c>
       <c r="D619" t="s">
         <v>1144</v>
@@ -15379,7 +15379,7 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -15403,7 +15403,7 @@
         <v>45</v>
       </c>
       <c r="B6">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -15427,7 +15427,7 @@
         <v>1143</v>
       </c>
       <c r="B9">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:2">

</xml_diff>

<commit_message>
updated predictions before adding mean reversal for age
</commit_message>
<xml_diff>
--- a/frontend/data/uk_election_predictions.xlsx
+++ b/frontend/data/uk_election_predictions.xlsx
@@ -13843,7 +13843,7 @@
         <v>1143</v>
       </c>
       <c r="C563">
-        <v>0.2825145550332216</v>
+        <v>0.2884541338878192</v>
       </c>
       <c r="D563" t="s">
         <v>1144</v>
@@ -13860,7 +13860,7 @@
         <v>1143</v>
       </c>
       <c r="C564">
-        <v>0.3326470726566873</v>
+        <v>0.3172809661289639</v>
       </c>
       <c r="D564" t="s">
         <v>1144</v>
@@ -13877,7 +13877,7 @@
         <v>1143</v>
       </c>
       <c r="C565">
-        <v>0.2767102227383172</v>
+        <v>0.2773377677243735</v>
       </c>
       <c r="D565" t="s">
         <v>1144</v>
@@ -13894,7 +13894,7 @@
         <v>1143</v>
       </c>
       <c r="C566">
-        <v>0.3696006753066093</v>
+        <v>0.368342835975275</v>
       </c>
       <c r="D566" t="s">
         <v>1144</v>
@@ -13911,7 +13911,7 @@
         <v>1143</v>
       </c>
       <c r="C567">
-        <v>0.3932226175754304</v>
+        <v>0.3884101799882506</v>
       </c>
       <c r="D567" t="s">
         <v>1144</v>
@@ -13928,7 +13928,7 @@
         <v>1143</v>
       </c>
       <c r="C568">
-        <v>0.3660396986876603</v>
+        <v>0.379371034479448</v>
       </c>
       <c r="D568" t="s">
         <v>1144</v>
@@ -13945,7 +13945,7 @@
         <v>1143</v>
       </c>
       <c r="C569">
-        <v>0.2597804062544701</v>
+        <v>0.2600739576711865</v>
       </c>
       <c r="D569" t="s">
         <v>1144</v>
@@ -13962,7 +13962,7 @@
         <v>1143</v>
       </c>
       <c r="C570">
-        <v>0.2847694407499272</v>
+        <v>0.2905986252948766</v>
       </c>
       <c r="D570" t="s">
         <v>1144</v>
@@ -13979,7 +13979,7 @@
         <v>1143</v>
       </c>
       <c r="C571">
-        <v>0.279111681997177</v>
+        <v>0.2806108459847001</v>
       </c>
       <c r="D571" t="s">
         <v>1144</v>
@@ -13996,7 +13996,7 @@
         <v>1143</v>
       </c>
       <c r="C572">
-        <v>0.2719369941301639</v>
+        <v>0.2605653666914444</v>
       </c>
       <c r="D572" t="s">
         <v>1144</v>
@@ -14013,7 +14013,7 @@
         <v>1143</v>
       </c>
       <c r="C573">
-        <v>0.3199991504770234</v>
+        <v>0.3248891226638706</v>
       </c>
       <c r="D573" t="s">
         <v>1144</v>
@@ -14030,7 +14030,7 @@
         <v>44</v>
       </c>
       <c r="C574">
-        <v>0.3107302264252313</v>
+        <v>0.3334316793337581</v>
       </c>
       <c r="D574" t="s">
         <v>1144</v>
@@ -14047,7 +14047,7 @@
         <v>1143</v>
       </c>
       <c r="C575">
-        <v>0.3669250325358958</v>
+        <v>0.3508593410760105</v>
       </c>
       <c r="D575" t="s">
         <v>1144</v>
@@ -14064,7 +14064,7 @@
         <v>1143</v>
       </c>
       <c r="C576">
-        <v>0.3785058952717061</v>
+        <v>0.3744840800853754</v>
       </c>
       <c r="D576" t="s">
         <v>1144</v>
@@ -14081,7 +14081,7 @@
         <v>6</v>
       </c>
       <c r="C577">
-        <v>0.3015655661956503</v>
+        <v>0.2778650220807022</v>
       </c>
       <c r="D577" t="s">
         <v>1144</v>
@@ -14098,7 +14098,7 @@
         <v>1143</v>
       </c>
       <c r="C578">
-        <v>0.3819813955196033</v>
+        <v>0.3722366567780488</v>
       </c>
       <c r="D578" t="s">
         <v>1144</v>
@@ -14115,7 +14115,7 @@
         <v>1143</v>
       </c>
       <c r="C579">
-        <v>0.3138353810690899</v>
+        <v>0.314444678161674</v>
       </c>
       <c r="D579" t="s">
         <v>1144</v>
@@ -14132,7 +14132,7 @@
         <v>10</v>
       </c>
       <c r="C580">
-        <v>0.3178558726104788</v>
+        <v>0.3351580348578205</v>
       </c>
       <c r="D580" t="s">
         <v>1144</v>
@@ -14149,7 +14149,7 @@
         <v>1143</v>
       </c>
       <c r="C581">
-        <v>0.4898225043811229</v>
+        <v>0.446050854412754</v>
       </c>
       <c r="D581" t="s">
         <v>1144</v>
@@ -14166,7 +14166,7 @@
         <v>1143</v>
       </c>
       <c r="C582">
-        <v>0.3069733337969863</v>
+        <v>0.3078860993807473</v>
       </c>
       <c r="D582" t="s">
         <v>1144</v>
@@ -14183,7 +14183,7 @@
         <v>1143</v>
       </c>
       <c r="C583">
-        <v>0.3683584748256013</v>
+        <v>0.3653731380049468</v>
       </c>
       <c r="D583" t="s">
         <v>1144</v>
@@ -14200,7 +14200,7 @@
         <v>1143</v>
       </c>
       <c r="C584">
-        <v>0.3013351697430424</v>
+        <v>0.3014934763097268</v>
       </c>
       <c r="D584" t="s">
         <v>1144</v>
@@ -14217,7 +14217,7 @@
         <v>1143</v>
       </c>
       <c r="C585">
-        <v>0.4083327607031286</v>
+        <v>0.4162026741118093</v>
       </c>
       <c r="D585" t="s">
         <v>1144</v>
@@ -14234,7 +14234,7 @@
         <v>1143</v>
       </c>
       <c r="C586">
-        <v>0.3008054465892636</v>
+        <v>0.2950762094740955</v>
       </c>
       <c r="D586" t="s">
         <v>1144</v>
@@ -14251,7 +14251,7 @@
         <v>6</v>
       </c>
       <c r="C587">
-        <v>0.2858500642732822</v>
+        <v>0.2645086405681463</v>
       </c>
       <c r="D587" t="s">
         <v>1144</v>
@@ -14268,7 +14268,7 @@
         <v>1143</v>
       </c>
       <c r="C588">
-        <v>0.325171024990202</v>
+        <v>0.3199422265530663</v>
       </c>
       <c r="D588" t="s">
         <v>1144</v>
@@ -14282,10 +14282,10 @@
         <v>1196</v>
       </c>
       <c r="B589" t="s">
-        <v>1143</v>
+        <v>44</v>
       </c>
       <c r="C589">
-        <v>0.3393589443667762</v>
+        <v>0.3390551340189545</v>
       </c>
       <c r="D589" t="s">
         <v>1144</v>
@@ -14302,7 +14302,7 @@
         <v>6</v>
       </c>
       <c r="C590">
-        <v>0.385366737919478</v>
+        <v>0.3763925756754392</v>
       </c>
       <c r="D590" t="s">
         <v>1144</v>
@@ -14319,7 +14319,7 @@
         <v>1143</v>
       </c>
       <c r="C591">
-        <v>0.5393213376485435</v>
+        <v>0.5095298202222793</v>
       </c>
       <c r="D591" t="s">
         <v>1144</v>
@@ -14336,7 +14336,7 @@
         <v>1143</v>
       </c>
       <c r="C592">
-        <v>0.4159838557158766</v>
+        <v>0.3989612299461182</v>
       </c>
       <c r="D592" t="s">
         <v>1144</v>
@@ -14353,7 +14353,7 @@
         <v>1143</v>
       </c>
       <c r="C593">
-        <v>0.6558457689044063</v>
+        <v>0.6582965010277916</v>
       </c>
       <c r="D593" t="s">
         <v>1144</v>
@@ -14370,7 +14370,7 @@
         <v>1143</v>
       </c>
       <c r="C594">
-        <v>0.4323160193782327</v>
+        <v>0.4221439994881752</v>
       </c>
       <c r="D594" t="s">
         <v>1144</v>
@@ -14387,7 +14387,7 @@
         <v>6</v>
       </c>
       <c r="C595">
-        <v>0.3007109193839573</v>
+        <v>0.2918106303385109</v>
       </c>
       <c r="D595" t="s">
         <v>1144</v>
@@ -14404,7 +14404,7 @@
         <v>1143</v>
       </c>
       <c r="C596">
-        <v>0.436002935663695</v>
+        <v>0.4301576463632634</v>
       </c>
       <c r="D596" t="s">
         <v>1144</v>
@@ -14421,7 +14421,7 @@
         <v>6</v>
       </c>
       <c r="C597">
-        <v>0.320323679383744</v>
+        <v>0.3044024203225391</v>
       </c>
       <c r="D597" t="s">
         <v>1144</v>
@@ -14435,10 +14435,10 @@
         <v>1214</v>
       </c>
       <c r="B598" t="s">
-        <v>1143</v>
+        <v>10</v>
       </c>
       <c r="C598">
-        <v>0.2369305280610853</v>
+        <v>0.2643341994591614</v>
       </c>
       <c r="D598" t="s">
         <v>1144</v>
@@ -14455,7 +14455,7 @@
         <v>1143</v>
       </c>
       <c r="C599">
-        <v>0.262048740484529</v>
+        <v>0.2648504330079637</v>
       </c>
       <c r="D599" t="s">
         <v>1144</v>
@@ -14472,7 +14472,7 @@
         <v>1143</v>
       </c>
       <c r="C600">
-        <v>0.2742453351379144</v>
+        <v>0.2761861474128283</v>
       </c>
       <c r="D600" t="s">
         <v>1144</v>
@@ -14486,10 +14486,10 @@
         <v>1220</v>
       </c>
       <c r="B601" t="s">
-        <v>1143</v>
+        <v>44</v>
       </c>
       <c r="C601">
-        <v>0.242944303401476</v>
+        <v>0.2572228456529158</v>
       </c>
       <c r="D601" t="s">
         <v>1144</v>
@@ -14506,7 +14506,7 @@
         <v>1143</v>
       </c>
       <c r="C602">
-        <v>0.3603223615600438</v>
+        <v>0.3613122234337758</v>
       </c>
       <c r="D602" t="s">
         <v>1144</v>
@@ -14523,7 +14523,7 @@
         <v>1143</v>
       </c>
       <c r="C603">
-        <v>0.2845776645230053</v>
+        <v>0.2855076528078401</v>
       </c>
       <c r="D603" t="s">
         <v>1144</v>
@@ -14540,7 +14540,7 @@
         <v>6</v>
       </c>
       <c r="C604">
-        <v>0.3130848833601909</v>
+        <v>0.2956557260375929</v>
       </c>
       <c r="D604" t="s">
         <v>1144</v>
@@ -14557,7 +14557,7 @@
         <v>44</v>
       </c>
       <c r="C605">
-        <v>0.2652879260965629</v>
+        <v>0.2914120289876425</v>
       </c>
       <c r="D605" t="s">
         <v>1144</v>
@@ -14574,7 +14574,7 @@
         <v>1143</v>
       </c>
       <c r="C606">
-        <v>0.3546178559487202</v>
+        <v>0.3451617870106473</v>
       </c>
       <c r="D606" t="s">
         <v>1144</v>
@@ -14591,7 +14591,7 @@
         <v>1143</v>
       </c>
       <c r="C607">
-        <v>0.3243076920493616</v>
+        <v>0.31832864658203</v>
       </c>
       <c r="D607" t="s">
         <v>1144</v>
@@ -14608,7 +14608,7 @@
         <v>6</v>
       </c>
       <c r="C608">
-        <v>0.3067845256022596</v>
+        <v>0.2832507191971311</v>
       </c>
       <c r="D608" t="s">
         <v>1144</v>
@@ -14625,7 +14625,7 @@
         <v>1143</v>
       </c>
       <c r="C609">
-        <v>0.2809127536694294</v>
+        <v>0.2805570156583798</v>
       </c>
       <c r="D609" t="s">
         <v>1144</v>
@@ -14639,10 +14639,10 @@
         <v>1238</v>
       </c>
       <c r="B610" t="s">
-        <v>1143</v>
+        <v>10</v>
       </c>
       <c r="C610">
-        <v>0.2405645277382739</v>
+        <v>0.2582097621665965</v>
       </c>
       <c r="D610" t="s">
         <v>1144</v>
@@ -14659,7 +14659,7 @@
         <v>44</v>
       </c>
       <c r="C611">
-        <v>0.4448754641887904</v>
+        <v>0.4919645159808907</v>
       </c>
       <c r="D611" t="s">
         <v>1144</v>
@@ -14676,7 +14676,7 @@
         <v>44</v>
       </c>
       <c r="C612">
-        <v>0.2889917162793297</v>
+        <v>0.3151492916956965</v>
       </c>
       <c r="D612" t="s">
         <v>1144</v>
@@ -14693,7 +14693,7 @@
         <v>1143</v>
       </c>
       <c r="C613">
-        <v>0.3414667532788234</v>
+        <v>0.3360888701446423</v>
       </c>
       <c r="D613" t="s">
         <v>1144</v>
@@ -14710,7 +14710,7 @@
         <v>1143</v>
       </c>
       <c r="C614">
-        <v>0.4221697187448215</v>
+        <v>0.4207979427071842</v>
       </c>
       <c r="D614" t="s">
         <v>1144</v>
@@ -14727,7 +14727,7 @@
         <v>1143</v>
       </c>
       <c r="C615">
-        <v>0.3295598156334839</v>
+        <v>0.3222503224022803</v>
       </c>
       <c r="D615" t="s">
         <v>1144</v>
@@ -14744,7 +14744,7 @@
         <v>1143</v>
       </c>
       <c r="C616">
-        <v>0.4306697553469792</v>
+        <v>0.4158551996754468</v>
       </c>
       <c r="D616" t="s">
         <v>1144</v>
@@ -14761,7 +14761,7 @@
         <v>1143</v>
       </c>
       <c r="C617">
-        <v>0.3319983589359958</v>
+        <v>0.3297967013232817</v>
       </c>
       <c r="D617" t="s">
         <v>1144</v>
@@ -14778,7 +14778,7 @@
         <v>10</v>
       </c>
       <c r="C618">
-        <v>0.3182352833574913</v>
+        <v>0.3389721578373202</v>
       </c>
       <c r="D618" t="s">
         <v>1144</v>
@@ -14795,7 +14795,7 @@
         <v>1143</v>
       </c>
       <c r="C619">
-        <v>0.4403718284674818</v>
+        <v>0.4461214753089645</v>
       </c>
       <c r="D619" t="s">
         <v>1144</v>
@@ -14812,7 +14812,7 @@
         <v>6</v>
       </c>
       <c r="C620">
-        <v>0.3104029982406734</v>
+        <v>0.3125307121551915</v>
       </c>
       <c r="D620" t="s">
         <v>1259</v>
@@ -14829,7 +14829,7 @@
         <v>15</v>
       </c>
       <c r="C621">
-        <v>0.3344987369481774</v>
+        <v>0.3507400549922038</v>
       </c>
       <c r="D621" t="s">
         <v>1259</v>
@@ -14846,7 +14846,7 @@
         <v>6</v>
       </c>
       <c r="C622">
-        <v>0.2711105195139781</v>
+        <v>0.2761082774659481</v>
       </c>
       <c r="D622" t="s">
         <v>1259</v>
@@ -14860,10 +14860,10 @@
         <v>1265</v>
       </c>
       <c r="B623" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C623">
-        <v>0.1998650128147459</v>
+        <v>0.2000750633796806</v>
       </c>
       <c r="D623" t="s">
         <v>1259</v>
@@ -14880,7 +14880,7 @@
         <v>10</v>
       </c>
       <c r="C624">
-        <v>0.2897594197377535</v>
+        <v>0.2883252241547618</v>
       </c>
       <c r="D624" t="s">
         <v>1259</v>
@@ -14897,7 +14897,7 @@
         <v>10</v>
       </c>
       <c r="C625">
-        <v>0.2436249891084367</v>
+        <v>0.2396158513481142</v>
       </c>
       <c r="D625" t="s">
         <v>1259</v>
@@ -14914,7 +14914,7 @@
         <v>15</v>
       </c>
       <c r="C626">
-        <v>0.3103934258040722</v>
+        <v>0.3273877094251895</v>
       </c>
       <c r="D626" t="s">
         <v>1259</v>
@@ -14931,7 +14931,7 @@
         <v>1274</v>
       </c>
       <c r="C627">
-        <v>0.2811903929356518</v>
+        <v>0.2907155384419668</v>
       </c>
       <c r="D627" t="s">
         <v>1259</v>
@@ -14948,7 +14948,7 @@
         <v>6</v>
       </c>
       <c r="C628">
-        <v>0.2167647871252837</v>
+        <v>0.2316826523207751</v>
       </c>
       <c r="D628" t="s">
         <v>1259</v>
@@ -14965,7 +14965,7 @@
         <v>6</v>
       </c>
       <c r="C629">
-        <v>0.265397913992652</v>
+        <v>0.2740322105859919</v>
       </c>
       <c r="D629" t="s">
         <v>1259</v>
@@ -14982,7 +14982,7 @@
         <v>1274</v>
       </c>
       <c r="C630">
-        <v>0.293666246412662</v>
+        <v>0.3249190296566286</v>
       </c>
       <c r="D630" t="s">
         <v>1259</v>
@@ -14999,7 +14999,7 @@
         <v>1274</v>
       </c>
       <c r="C631">
-        <v>0.3052227366862181</v>
+        <v>0.3213592118476376</v>
       </c>
       <c r="D631" t="s">
         <v>1259</v>
@@ -15016,7 +15016,7 @@
         <v>1274</v>
       </c>
       <c r="C632">
-        <v>0.3789411780583819</v>
+        <v>0.3899411003422587</v>
       </c>
       <c r="D632" t="s">
         <v>1259</v>
@@ -15033,7 +15033,7 @@
         <v>15</v>
       </c>
       <c r="C633">
-        <v>0.2604602991478561</v>
+        <v>0.2754347631658899</v>
       </c>
       <c r="D633" t="s">
         <v>1259</v>
@@ -15050,7 +15050,7 @@
         <v>15</v>
       </c>
       <c r="C634">
-        <v>0.3733070460900481</v>
+        <v>0.4043783090255618</v>
       </c>
       <c r="D634" t="s">
         <v>1259</v>
@@ -15067,7 +15067,7 @@
         <v>1274</v>
       </c>
       <c r="C635">
-        <v>0.401939843668326</v>
+        <v>0.4224469967081615</v>
       </c>
       <c r="D635" t="s">
         <v>1259</v>
@@ -15084,7 +15084,7 @@
         <v>6</v>
       </c>
       <c r="C636">
-        <v>0.384706885807842</v>
+        <v>0.395115115047224</v>
       </c>
       <c r="D636" t="s">
         <v>1259</v>
@@ -15101,7 +15101,7 @@
         <v>15</v>
       </c>
       <c r="C637">
-        <v>0.2688666004105387</v>
+        <v>0.2847717563531478</v>
       </c>
       <c r="D637" t="s">
         <v>1259</v>
@@ -15118,7 +15118,7 @@
         <v>1274</v>
       </c>
       <c r="C638">
-        <v>0.4059303674170687</v>
+        <v>0.423901360193371</v>
       </c>
       <c r="D638" t="s">
         <v>1259</v>
@@ -15135,7 +15135,7 @@
         <v>10</v>
       </c>
       <c r="C639">
-        <v>0.3509843947032604</v>
+        <v>0.3465188860892308</v>
       </c>
       <c r="D639" t="s">
         <v>1259</v>
@@ -15152,7 +15152,7 @@
         <v>10</v>
       </c>
       <c r="C640">
-        <v>0.2825080544759188</v>
+        <v>0.2833597484023196</v>
       </c>
       <c r="D640" t="s">
         <v>1259</v>
@@ -15169,7 +15169,7 @@
         <v>15</v>
       </c>
       <c r="C641">
-        <v>0.2549091824216865</v>
+        <v>0.2671652083472434</v>
       </c>
       <c r="D641" t="s">
         <v>1259</v>
@@ -15186,7 +15186,7 @@
         <v>1274</v>
       </c>
       <c r="C642">
-        <v>0.2719646899842941</v>
+        <v>0.2829886519524138</v>
       </c>
       <c r="D642" t="s">
         <v>1259</v>
@@ -15203,7 +15203,7 @@
         <v>15</v>
       </c>
       <c r="C643">
-        <v>0.2914348283479374</v>
+        <v>0.3012074692481571</v>
       </c>
       <c r="D643" t="s">
         <v>1259</v>
@@ -15220,7 +15220,7 @@
         <v>15</v>
       </c>
       <c r="C644">
-        <v>0.264832382107491</v>
+        <v>0.2812053685863024</v>
       </c>
       <c r="D644" t="s">
         <v>1259</v>
@@ -15237,7 +15237,7 @@
         <v>15</v>
       </c>
       <c r="C645">
-        <v>0.2484083793559056</v>
+        <v>0.2554459886194498</v>
       </c>
       <c r="D645" t="s">
         <v>1259</v>
@@ -15254,7 +15254,7 @@
         <v>15</v>
       </c>
       <c r="C646">
-        <v>0.3365939816540054</v>
+        <v>0.3645766184623316</v>
       </c>
       <c r="D646" t="s">
         <v>1259</v>
@@ -15271,7 +15271,7 @@
         <v>6</v>
       </c>
       <c r="C647">
-        <v>0.2877847868598161</v>
+        <v>0.2909655313496472</v>
       </c>
       <c r="D647" t="s">
         <v>1259</v>
@@ -15288,7 +15288,7 @@
         <v>15</v>
       </c>
       <c r="C648">
-        <v>0.2607515713142328</v>
+        <v>0.2818035307281975</v>
       </c>
       <c r="D648" t="s">
         <v>1259</v>
@@ -15305,7 +15305,7 @@
         <v>15</v>
       </c>
       <c r="C649">
-        <v>0.3028602240440963</v>
+        <v>0.3285805759841801</v>
       </c>
       <c r="D649" t="s">
         <v>1259</v>
@@ -15322,7 +15322,7 @@
         <v>6</v>
       </c>
       <c r="C650">
-        <v>0.2571398045357967</v>
+        <v>0.2635631244085863</v>
       </c>
       <c r="D650" t="s">
         <v>1259</v>
@@ -15339,7 +15339,7 @@
         <v>15</v>
       </c>
       <c r="C651">
-        <v>0.2892728605372195</v>
+        <v>0.3081560486231352</v>
       </c>
       <c r="D651" t="s">
         <v>1259</v>
@@ -15371,7 +15371,7 @@
         <v>15</v>
       </c>
       <c r="B2">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -15379,7 +15379,7 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -15395,7 +15395,7 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -15403,7 +15403,7 @@
         <v>44</v>
       </c>
       <c r="B6">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -15427,7 +15427,7 @@
         <v>1143</v>
       </c>
       <c r="B9">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:2">

</xml_diff>